<commit_message>
chore: add AGENTS.md and update Binzhou data file
</commit_message>
<xml_diff>
--- a/Binzhou_Houyi (1) (1).xlsx
+++ b/Binzhou_Houyi (1) (1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Desktop\upload\FishWebClean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8212B8A-3CE1-48DB-9684-2FE0F64859D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3774F72C-24EF-4548-A9DC-93D5F2D0065C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -687,9 +687,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="\$#,##0.00;\-\$#,##0.00"/>
-    <numFmt numFmtId="174" formatCode="\$#,##0.000;\-\$#,##0.000"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="\$#,##0.00;\-\$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0.000;\-\$#,##0.000"/>
+    <numFmt numFmtId="170" formatCode="_([$IQD]\ * #,##0_);_([$IQD]\ * \(#,##0\);_([$IQD]\ * &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -857,7 +858,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -868,7 +869,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -880,7 +881,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -892,10 +893,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -919,13 +920,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -939,15 +940,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -971,10 +963,10 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="3" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -983,14 +975,26 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="174" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="174" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1109,16 +1113,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1235868</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1906</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>957580</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>871062</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>52705</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1141,8 +1145,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9039225" y="2257425"/>
-          <a:ext cx="1040130" cy="909955"/>
+          <a:off x="9820274" y="2547938"/>
+          <a:ext cx="921069" cy="909955"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1478,15 +1482,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
+      <xdr:colOff>147251</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>230982</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>922655</xdr:colOff>
+      <xdr:colOff>830141</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>926465</xdr:rowOff>
+      <xdr:rowOff>916782</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1509,8 +1513,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9058275" y="9693275"/>
-          <a:ext cx="989330" cy="897890"/>
+          <a:off x="10017532" y="10053638"/>
+          <a:ext cx="682890" cy="685800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1526,15 +1530,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:colOff>30956</xdr:colOff>
       <xdr:row>15</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:rowOff>210344</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>636</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>908050</xdr:rowOff>
+      <xdr:colOff>12542</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>157957</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1557,8 +1561,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9048750" y="10661650"/>
-          <a:ext cx="1019810" cy="876300"/>
+          <a:off x="9901237" y="10997407"/>
+          <a:ext cx="910274" cy="876300"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1906,15 +1910,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:colOff>92866</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>15875</xdr:rowOff>
+      <xdr:rowOff>158749</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1271</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>769923</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>819785</xdr:rowOff>
+      <xdr:rowOff>750093</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1937,8 +1941,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9039225" y="17922875"/>
-          <a:ext cx="1020445" cy="803910"/>
+          <a:off x="9963147" y="18172905"/>
+          <a:ext cx="677057" cy="591344"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1954,15 +1958,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:colOff>79681</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1271</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>887508</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>824865</xdr:rowOff>
+      <xdr:rowOff>773906</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1984,9 +1988,9 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9039225" y="18764250"/>
-          <a:ext cx="1029970" cy="805815"/>
+        <a:xfrm flipH="1">
+          <a:off x="9949962" y="18914269"/>
+          <a:ext cx="807827" cy="707231"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2098,15 +2102,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
+      <xdr:colOff>42863</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:rowOff>50006</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>920750</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
+      <xdr:colOff>908115</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>916782</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2129,8 +2133,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9048750" y="21475700"/>
-          <a:ext cx="1006475" cy="901700"/>
+          <a:off x="9913144" y="21588412"/>
+          <a:ext cx="865252" cy="866776"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2244,13 +2248,13 @@
       <xdr:col>8</xdr:col>
       <xdr:colOff>28575</xdr:colOff>
       <xdr:row>34</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:rowOff>283368</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>4446</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>981075</xdr:rowOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>183355</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2273,8 +2277,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9058275" y="25304750"/>
-          <a:ext cx="966470" cy="923925"/>
+          <a:off x="9898856" y="25619868"/>
+          <a:ext cx="904559" cy="923925"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2938,15 +2942,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
+      <xdr:colOff>145257</xdr:colOff>
       <xdr:row>51</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>421482</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>998220</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>397510</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>100489</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>314167</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2969,8 +2973,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9067800" y="40589200"/>
-          <a:ext cx="960120" cy="753110"/>
+          <a:off x="10015538" y="40950357"/>
+          <a:ext cx="883920" cy="749935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3295,14 +3299,14 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>56515</xdr:rowOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>1056641</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>1</xdr:colOff>
       <xdr:row>66</xdr:row>
-      <xdr:rowOff>1019175</xdr:rowOff>
+      <xdr:rowOff>947738</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3325,8 +3329,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9067800" y="48621315"/>
-          <a:ext cx="1009650" cy="962660"/>
+          <a:off x="9908381" y="49598422"/>
+          <a:ext cx="890589" cy="962660"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3344,13 +3348,13 @@
       <xdr:col>8</xdr:col>
       <xdr:colOff>29210</xdr:colOff>
       <xdr:row>67</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:rowOff>197643</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>3176</xdr:colOff>
-      <xdr:row>67</xdr:row>
-      <xdr:rowOff>986155</xdr:rowOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>140810</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3373,8 +3377,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9058910" y="49612550"/>
-          <a:ext cx="983615" cy="967105"/>
+          <a:off x="9899491" y="50834924"/>
+          <a:ext cx="902654" cy="967105"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3557,8 +3561,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9096375" y="54470300"/>
-          <a:ext cx="912495" cy="878205"/>
+          <a:off x="9936956" y="54568725"/>
+          <a:ext cx="855345" cy="878205"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3903,15 +3907,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>90213</xdr:colOff>
+      <xdr:colOff>18775</xdr:colOff>
       <xdr:row>79</xdr:row>
-      <xdr:rowOff>202406</xdr:rowOff>
+      <xdr:rowOff>190500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>10958</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>868208</xdr:colOff>
       <xdr:row>79</xdr:row>
-      <xdr:rowOff>916781</xdr:rowOff>
+      <xdr:rowOff>904875</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3934,7 +3938,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="9960494" y="61233844"/>
+          <a:off x="9889056" y="62150625"/>
           <a:ext cx="849433" cy="714375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4280,7 +4284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -4295,11 +4299,11 @@
     <col min="10" max="10" width="4.7109375" style="3" customWidth="1"/>
     <col min="11" max="11" width="13.85546875" style="4" customWidth="1"/>
     <col min="12" max="12" width="33.140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5703125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="25.28515625" style="1" customWidth="1"/>
     <col min="14" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30">
+    <row r="1" spans="1:13" ht="30">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -4333,7 +4337,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="24" customFormat="1" ht="75" customHeight="1">
+    <row r="2" spans="1:13" s="24" customFormat="1" ht="75" customHeight="1">
       <c r="A2" s="18">
         <v>1</v>
       </c>
@@ -4370,8 +4374,12 @@
       <c r="L2" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" s="24" customFormat="1" ht="84" customHeight="1">
+      <c r="M2" s="46">
+        <f>1420*H2</f>
+        <v>5433.0434782608691</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" s="24" customFormat="1" ht="84" customHeight="1">
       <c r="A3" s="25">
         <v>2</v>
       </c>
@@ -4408,8 +4416,12 @@
       <c r="L3" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" s="24" customFormat="1" ht="78.95" customHeight="1">
+      <c r="M3" s="46">
+        <f t="shared" ref="M3:M66" si="2">1420*H3</f>
+        <v>498.02898550724638</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" s="24" customFormat="1" ht="78.95" customHeight="1">
       <c r="A4" s="18">
         <v>3</v>
       </c>
@@ -4446,8 +4458,12 @@
       <c r="L4" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" s="24" customFormat="1" ht="80.099999999999994" customHeight="1">
+      <c r="M4" s="46">
+        <f t="shared" si="2"/>
+        <v>967.24637681159425</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" s="24" customFormat="1" ht="80.099999999999994" customHeight="1">
       <c r="A5" s="18">
         <v>4</v>
       </c>
@@ -4484,8 +4500,12 @@
       <c r="L5" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" s="24" customFormat="1" ht="63" customHeight="1">
+      <c r="M5" s="46">
+        <f t="shared" si="2"/>
+        <v>1992.1159420289855</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" s="24" customFormat="1" ht="63" customHeight="1">
       <c r="A6" s="18">
         <v>5</v>
       </c>
@@ -4522,8 +4542,12 @@
       <c r="L6" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" s="24" customFormat="1" ht="72" customHeight="1">
+      <c r="M6" s="46">
+        <f t="shared" si="2"/>
+        <v>1131.8840579710145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A7" s="18">
         <v>6</v>
       </c>
@@ -4560,8 +4584,12 @@
       <c r="L7" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" s="24" customFormat="1" ht="66.95" customHeight="1">
+      <c r="M7" s="46">
+        <f t="shared" si="2"/>
+        <v>226.37681159420291</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" s="24" customFormat="1" ht="66.95" customHeight="1">
       <c r="A8" s="18">
         <v>7</v>
       </c>
@@ -4598,8 +4626,12 @@
       <c r="L8" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" s="24" customFormat="1" ht="69.95" customHeight="1">
+      <c r="M8" s="46">
+        <f t="shared" si="2"/>
+        <v>226.37681159420291</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" s="24" customFormat="1" ht="69.95" customHeight="1">
       <c r="A9" s="18">
         <v>8</v>
       </c>
@@ -4636,8 +4668,12 @@
       <c r="L9" s="18" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="10" spans="1:12" s="24" customFormat="1" ht="72" customHeight="1">
+      <c r="M9" s="46">
+        <f t="shared" si="2"/>
+        <v>3622.0289855072465</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A10" s="18">
         <v>9</v>
       </c>
@@ -4674,8 +4710,12 @@
       <c r="L10" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" s="24" customFormat="1" ht="21" customHeight="1">
+      <c r="M10" s="46">
+        <f t="shared" si="2"/>
+        <v>2241.1304347826085</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A11" s="18">
         <v>10</v>
       </c>
@@ -4701,7 +4741,7 @@
         <f t="shared" si="0"/>
         <v>4.63768115942029</v>
       </c>
-      <c r="I11" s="28"/>
+      <c r="I11" s="43"/>
       <c r="J11" s="22">
         <v>2</v>
       </c>
@@ -4712,8 +4752,12 @@
       <c r="L11" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" s="24" customFormat="1" ht="21" customHeight="1">
+      <c r="M11" s="46">
+        <f t="shared" si="2"/>
+        <v>6585.507246376812</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A12" s="18">
         <v>11</v>
       </c>
@@ -4739,7 +4783,7 @@
         <f t="shared" si="0"/>
         <v>7.2463768115942022</v>
       </c>
-      <c r="I12" s="29"/>
+      <c r="I12" s="44"/>
       <c r="J12" s="22">
         <v>2</v>
       </c>
@@ -4750,8 +4794,12 @@
       <c r="L12" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" s="24" customFormat="1" ht="21" customHeight="1">
+      <c r="M12" s="46">
+        <f t="shared" si="2"/>
+        <v>10289.855072463768</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A13" s="18">
         <v>12</v>
       </c>
@@ -4777,7 +4825,7 @@
         <f t="shared" si="0"/>
         <v>4.057971014492753</v>
       </c>
-      <c r="I13" s="29"/>
+      <c r="I13" s="44"/>
       <c r="J13" s="22">
         <v>2</v>
       </c>
@@ -4788,8 +4836,12 @@
       <c r="L13" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" s="24" customFormat="1" ht="21" customHeight="1">
+      <c r="M13" s="46">
+        <f t="shared" si="2"/>
+        <v>5762.3188405797091</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A14" s="18">
         <v>13</v>
       </c>
@@ -4815,7 +4867,7 @@
         <f t="shared" si="0"/>
         <v>4.63768115942029</v>
       </c>
-      <c r="I14" s="30"/>
+      <c r="I14" s="45"/>
       <c r="J14" s="22">
         <v>3</v>
       </c>
@@ -4826,8 +4878,12 @@
       <c r="L14" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" s="24" customFormat="1" ht="75.95" customHeight="1">
+      <c r="M14" s="46">
+        <f t="shared" si="2"/>
+        <v>6585.507246376812</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A15" s="18">
         <v>14</v>
       </c>
@@ -4864,8 +4920,12 @@
       <c r="L15" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" s="24" customFormat="1" ht="74.099999999999994" customHeight="1">
+      <c r="M15" s="46">
+        <f t="shared" si="2"/>
+        <v>7408.695652173913</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" s="24" customFormat="1" ht="74.099999999999994" customHeight="1">
       <c r="A16" s="18">
         <v>15</v>
       </c>
@@ -4902,8 +4962,12 @@
       <c r="L16" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" s="24" customFormat="1" ht="18.95" customHeight="1">
+      <c r="M16" s="46">
+        <f t="shared" si="2"/>
+        <v>2716.5217391304345</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A17" s="18">
         <v>16</v>
       </c>
@@ -4929,7 +4993,7 @@
         <f t="shared" si="0"/>
         <v>0.14492753623188406</v>
       </c>
-      <c r="I17" s="28"/>
+      <c r="I17" s="43"/>
       <c r="J17" s="22">
         <v>5</v>
       </c>
@@ -4940,8 +5004,12 @@
       <c r="L17" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" s="24" customFormat="1" ht="18.95" customHeight="1">
+      <c r="M17" s="46">
+        <f t="shared" si="2"/>
+        <v>205.79710144927537</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A18" s="18">
         <v>17</v>
       </c>
@@ -4967,7 +5035,7 @@
         <f t="shared" si="0"/>
         <v>0.21739130434782608</v>
       </c>
-      <c r="I18" s="29"/>
+      <c r="I18" s="44"/>
       <c r="J18" s="22">
         <v>5</v>
       </c>
@@ -4978,8 +5046,12 @@
       <c r="L18" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" s="24" customFormat="1" ht="18.95" customHeight="1">
+      <c r="M18" s="46">
+        <f t="shared" si="2"/>
+        <v>308.69565217391306</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A19" s="18">
         <v>18</v>
       </c>
@@ -5005,7 +5077,7 @@
         <f t="shared" si="0"/>
         <v>0.52173913043478259</v>
       </c>
-      <c r="I19" s="29"/>
+      <c r="I19" s="44"/>
       <c r="J19" s="22">
         <v>5</v>
       </c>
@@ -5016,8 +5088,12 @@
       <c r="L19" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" s="24" customFormat="1" ht="18.95" customHeight="1">
+      <c r="M19" s="46">
+        <f t="shared" si="2"/>
+        <v>740.86956521739125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A20" s="18">
         <v>19</v>
       </c>
@@ -5043,7 +5119,7 @@
         <f t="shared" si="0"/>
         <v>0.94202898550724634</v>
       </c>
-      <c r="I20" s="30"/>
+      <c r="I20" s="45"/>
       <c r="J20" s="22">
         <v>3</v>
       </c>
@@ -5054,8 +5130,12 @@
       <c r="L20" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="1:12" s="24" customFormat="1" ht="66.95" customHeight="1">
+      <c r="M20" s="46">
+        <f t="shared" si="2"/>
+        <v>1337.6811594202898</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" s="24" customFormat="1" ht="66.95" customHeight="1">
       <c r="A21" s="18">
         <v>20</v>
       </c>
@@ -5092,8 +5172,12 @@
       <c r="L21" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" s="24" customFormat="1" ht="56.1" customHeight="1">
+      <c r="M21" s="46">
+        <f t="shared" si="2"/>
+        <v>4939.130434782609</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" s="24" customFormat="1" ht="56.1" customHeight="1">
       <c r="A22" s="18">
         <v>21</v>
       </c>
@@ -5130,8 +5214,12 @@
       <c r="L22" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" s="24" customFormat="1" ht="72" customHeight="1">
+      <c r="M22" s="46">
+        <f t="shared" si="2"/>
+        <v>4115.942028985507</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A23" s="18">
         <v>22</v>
       </c>
@@ -5168,8 +5256,12 @@
       <c r="L23" s="18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" s="24" customFormat="1" ht="75.95" customHeight="1">
+      <c r="M23" s="46">
+        <f t="shared" si="2"/>
+        <v>16463.768115942028</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A24" s="18">
         <v>23</v>
       </c>
@@ -5206,8 +5298,12 @@
       <c r="L24" s="18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="M24" s="46">
+        <f t="shared" si="2"/>
+        <v>226.37681159420291</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A25" s="18">
         <v>24</v>
       </c>
@@ -5244,8 +5340,12 @@
       <c r="L25" s="18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
+      <c r="M25" s="46">
+        <f t="shared" si="2"/>
+        <v>2942.8985507246375</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
       <c r="A26" s="18">
         <v>25</v>
       </c>
@@ -5282,8 +5382,12 @@
       <c r="L26" s="18" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" s="24" customFormat="1" ht="66" customHeight="1">
+      <c r="M26" s="46">
+        <f t="shared" si="2"/>
+        <v>411.59420289855075</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" s="24" customFormat="1" ht="66" customHeight="1">
       <c r="A27" s="18">
         <v>26</v>
       </c>
@@ -5320,8 +5424,12 @@
       <c r="L27" s="18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" s="24" customFormat="1" ht="68.099999999999994" customHeight="1">
+      <c r="M27" s="46">
+        <f t="shared" si="2"/>
+        <v>452.75362318840581</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" s="24" customFormat="1" ht="68.099999999999994" customHeight="1">
       <c r="A28" s="18"/>
       <c r="B28" s="19" t="s">
         <v>94</v>
@@ -5356,8 +5464,12 @@
       <c r="L28" s="18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" s="24" customFormat="1" ht="72" customHeight="1">
+      <c r="M28" s="46">
+        <f t="shared" si="2"/>
+        <v>452.75362318840581</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A29" s="18">
         <v>28</v>
       </c>
@@ -5394,8 +5506,12 @@
       <c r="L29" s="18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" s="24" customFormat="1" ht="72" customHeight="1">
+      <c r="M29" s="46">
+        <f t="shared" si="2"/>
+        <v>271.6521739130435</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A30" s="18">
         <v>29</v>
       </c>
@@ -5432,8 +5548,12 @@
       <c r="L30" s="18" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="M30" s="46">
+        <f t="shared" si="2"/>
+        <v>452.75362318840581</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A31" s="18">
         <v>30</v>
       </c>
@@ -5470,8 +5590,12 @@
       <c r="L31" s="18" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" s="24" customFormat="1" ht="75.95" customHeight="1">
+      <c r="M31" s="46">
+        <f t="shared" si="2"/>
+        <v>452.75362318840581</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A32" s="18">
         <v>32</v>
       </c>
@@ -5508,8 +5632,12 @@
       <c r="L32" s="18" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="33" spans="1:12" s="24" customFormat="1" ht="69.95" customHeight="1">
+      <c r="M32" s="46">
+        <f t="shared" si="2"/>
+        <v>271.6521739130435</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" s="24" customFormat="1" ht="69.95" customHeight="1">
       <c r="A33" s="18">
         <v>32</v>
       </c>
@@ -5546,8 +5674,12 @@
       <c r="L33" s="18" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="34" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="M33" s="46">
+        <f t="shared" si="2"/>
+        <v>226.37681159420291</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A34" s="18">
         <v>34</v>
       </c>
@@ -5584,8 +5716,12 @@
       <c r="L34" s="18" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="M34" s="46">
+        <f t="shared" si="2"/>
+        <v>45.275362318840578</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A35" s="18">
         <v>35</v>
       </c>
@@ -5608,7 +5744,7 @@
         <v>1.97</v>
       </c>
       <c r="H35" s="21">
-        <f t="shared" ref="H35:H69" si="2">G35/6.9</f>
+        <f t="shared" ref="H35:H69" si="3">G35/6.9</f>
         <v>0.28550724637681157</v>
       </c>
       <c r="I35" s="19"/>
@@ -5616,14 +5752,18 @@
         <v>40</v>
       </c>
       <c r="K35" s="23">
-        <f t="shared" ref="K35:K69" si="3">J35*H35</f>
+        <f t="shared" ref="K35:K69" si="4">J35*H35</f>
         <v>11.420289855072463</v>
       </c>
       <c r="L35" s="18" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="M35" s="46">
+        <f t="shared" si="2"/>
+        <v>405.42028985507244</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A36" s="18">
         <v>36</v>
       </c>
@@ -5646,7 +5786,7 @@
         <v>12</v>
       </c>
       <c r="H36" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7391304347826086</v>
       </c>
       <c r="I36" s="19"/>
@@ -5654,14 +5794,18 @@
         <v>10</v>
       </c>
       <c r="K36" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>17.391304347826086</v>
       </c>
       <c r="L36" s="18" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="M36" s="46">
+        <f t="shared" si="2"/>
+        <v>2469.5652173913045</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A37" s="18">
         <v>37</v>
       </c>
@@ -5684,7 +5828,7 @@
         <v>3</v>
       </c>
       <c r="H37" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.43478260869565216</v>
       </c>
       <c r="I37" s="19"/>
@@ -5692,14 +5836,18 @@
         <v>20</v>
       </c>
       <c r="K37" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8.695652173913043</v>
       </c>
       <c r="L37" s="18" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="M37" s="46">
+        <f t="shared" si="2"/>
+        <v>617.39130434782612</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A38" s="25">
         <v>38</v>
       </c>
@@ -5722,7 +5870,7 @@
         <v>28.6</v>
       </c>
       <c r="H38" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.1449275362318838</v>
       </c>
       <c r="I38" s="19"/>
@@ -5730,14 +5878,18 @@
         <v>2</v>
       </c>
       <c r="K38" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8.2898550724637676</v>
       </c>
       <c r="L38" s="18" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" s="24" customFormat="1" ht="84.95" customHeight="1">
+      <c r="M38" s="46">
+        <f t="shared" si="2"/>
+        <v>5885.797101449275</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A39" s="18">
         <v>39</v>
       </c>
@@ -5760,7 +5912,7 @@
         <v>2.86</v>
       </c>
       <c r="H39" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.41449275362318838</v>
       </c>
       <c r="I39" s="19"/>
@@ -5768,14 +5920,18 @@
         <v>12</v>
       </c>
       <c r="K39" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>4.9739130434782606</v>
       </c>
       <c r="L39" s="18" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" s="24" customFormat="1" ht="84.95" customHeight="1">
+      <c r="M39" s="46">
+        <f t="shared" si="2"/>
+        <v>588.5797101449275</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A40" s="18">
         <v>40</v>
       </c>
@@ -5785,7 +5941,7 @@
       <c r="C40" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D40" s="31" t="s">
+      <c r="D40" s="28" t="s">
         <v>136</v>
       </c>
       <c r="E40" s="19" t="s">
@@ -5798,7 +5954,7 @@
         <v>4.84</v>
       </c>
       <c r="H40" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.70144927536231882</v>
       </c>
       <c r="I40" s="19"/>
@@ -5806,14 +5962,18 @@
         <v>10</v>
       </c>
       <c r="K40" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.0144927536231885</v>
       </c>
       <c r="L40" s="18" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" s="24" customFormat="1" ht="84.95" customHeight="1">
+      <c r="M40" s="46">
+        <f t="shared" si="2"/>
+        <v>996.05797101449275</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A41" s="18">
         <v>41</v>
       </c>
@@ -5836,7 +5996,7 @@
         <v>3.3</v>
       </c>
       <c r="H41" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.47826086956521735</v>
       </c>
       <c r="I41" s="19"/>
@@ -5844,14 +6004,18 @@
         <v>10</v>
       </c>
       <c r="K41" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>4.7826086956521738</v>
       </c>
       <c r="L41" s="18" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" s="24" customFormat="1" ht="84.95" customHeight="1">
+      <c r="M41" s="46">
+        <f t="shared" si="2"/>
+        <v>679.13043478260863</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A42" s="18">
         <v>42</v>
       </c>
@@ -5874,7 +6038,7 @@
         <v>1.43</v>
       </c>
       <c r="H42" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.20724637681159419</v>
       </c>
       <c r="I42" s="19"/>
@@ -5882,14 +6046,18 @@
         <v>20</v>
       </c>
       <c r="K42" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>4.1449275362318838</v>
       </c>
       <c r="L42" s="18" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" s="24" customFormat="1" ht="84.95" customHeight="1">
+      <c r="M42" s="46">
+        <f t="shared" si="2"/>
+        <v>294.28985507246375</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A43" s="18">
         <v>43</v>
       </c>
@@ -5912,7 +6080,7 @@
         <v>0.22</v>
       </c>
       <c r="H43" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I43" s="19"/>
@@ -5920,14 +6088,18 @@
         <v>40</v>
       </c>
       <c r="K43" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.2753623188405796</v>
       </c>
       <c r="L43" s="18" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="44" spans="1:12" s="24" customFormat="1" ht="83.1" customHeight="1">
+      <c r="M43" s="46">
+        <f t="shared" si="2"/>
+        <v>45.275362318840578</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" s="24" customFormat="1" ht="83.1" customHeight="1">
       <c r="A44" s="18">
         <v>44</v>
       </c>
@@ -5950,7 +6122,7 @@
         <v>210</v>
       </c>
       <c r="H44" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>30.434782608695652</v>
       </c>
       <c r="I44" s="19"/>
@@ -5958,14 +6130,18 @@
         <v>1</v>
       </c>
       <c r="K44" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>30.434782608695652</v>
       </c>
       <c r="L44" s="18" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="45" spans="1:12" s="24" customFormat="1" ht="78" customHeight="1">
+      <c r="M44" s="46">
+        <f t="shared" si="2"/>
+        <v>43217.391304347824</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" s="24" customFormat="1" ht="78" customHeight="1">
       <c r="A45" s="18">
         <v>45</v>
       </c>
@@ -5988,7 +6164,7 @@
         <v>7.26</v>
       </c>
       <c r="H45" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0521739130434782</v>
       </c>
       <c r="I45" s="19"/>
@@ -5996,12 +6172,16 @@
         <v>3</v>
       </c>
       <c r="K45" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.1565217391304348</v>
       </c>
-      <c r="L45" s="32"/>
-    </row>
-    <row r="46" spans="1:12" s="24" customFormat="1" ht="78" customHeight="1">
+      <c r="L45" s="29"/>
+      <c r="M45" s="46">
+        <f t="shared" si="2"/>
+        <v>1494.086956521739</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" s="24" customFormat="1" ht="78" customHeight="1">
       <c r="A46" s="18">
         <v>46</v>
       </c>
@@ -6024,7 +6204,7 @@
         <v>7.26</v>
       </c>
       <c r="H46" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0521739130434782</v>
       </c>
       <c r="I46" s="19"/>
@@ -6032,14 +6212,18 @@
         <v>3</v>
       </c>
       <c r="K46" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.1565217391304348</v>
       </c>
       <c r="L46" s="18" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="47" spans="1:12" s="24" customFormat="1" ht="62.1" customHeight="1">
+      <c r="M46" s="46">
+        <f t="shared" si="2"/>
+        <v>1494.086956521739</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" s="24" customFormat="1" ht="62.1" customHeight="1">
       <c r="A47" s="18">
         <v>47</v>
       </c>
@@ -6062,7 +6246,7 @@
         <v>0.22</v>
       </c>
       <c r="H47" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I47" s="19"/>
@@ -6070,14 +6254,18 @@
         <v>30</v>
       </c>
       <c r="K47" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.9565217391304347</v>
       </c>
       <c r="L47" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="48" spans="1:12" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
+      <c r="M47" s="46">
+        <f t="shared" si="2"/>
+        <v>45.275362318840578</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
       <c r="A48" s="18">
         <v>48</v>
       </c>
@@ -6100,7 +6288,7 @@
         <v>0.22</v>
       </c>
       <c r="H48" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I48" s="19"/>
@@ -6108,166 +6296,186 @@
         <v>30</v>
       </c>
       <c r="K48" s="23">
+        <f t="shared" si="4"/>
+        <v>0.9565217391304347</v>
+      </c>
+      <c r="L48" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="M48" s="46">
+        <f t="shared" si="2"/>
+        <v>45.275362318840578</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A49" s="18">
+        <v>49</v>
+      </c>
+      <c r="B49" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="D49" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="E49" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="F49" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" s="20">
+        <v>0.09</v>
+      </c>
+      <c r="H49" s="21">
+        <f t="shared" si="3"/>
+        <v>1.3043478260869565E-2</v>
+      </c>
+      <c r="I49" s="43"/>
+      <c r="J49" s="22">
+        <v>50</v>
+      </c>
+      <c r="K49" s="23">
+        <f t="shared" si="4"/>
+        <v>0.65217391304347827</v>
+      </c>
+      <c r="L49" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="M49" s="46">
+        <f t="shared" si="2"/>
+        <v>18.521739130434781</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A50" s="18">
+        <v>50</v>
+      </c>
+      <c r="B50" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="C50" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="D50" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="E50" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="F50" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" s="20">
+        <v>0.06</v>
+      </c>
+      <c r="H50" s="21">
+        <f t="shared" si="3"/>
+        <v>8.6956521739130418E-3</v>
+      </c>
+      <c r="I50" s="44"/>
+      <c r="J50" s="22">
+        <v>50</v>
+      </c>
+      <c r="K50" s="23">
+        <f t="shared" si="4"/>
+        <v>0.43478260869565211</v>
+      </c>
+      <c r="L50" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="M50" s="46">
+        <f t="shared" si="2"/>
+        <v>12.34782608695652</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A51" s="18">
+        <v>51</v>
+      </c>
+      <c r="B51" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="C51" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="E51" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="F51" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="20">
+        <v>0.2</v>
+      </c>
+      <c r="H51" s="21">
+        <f t="shared" si="3"/>
+        <v>2.8985507246376812E-2</v>
+      </c>
+      <c r="I51" s="45"/>
+      <c r="J51" s="22">
+        <v>50</v>
+      </c>
+      <c r="K51" s="23">
+        <f t="shared" si="4"/>
+        <v>1.4492753623188406</v>
+      </c>
+      <c r="L51" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="M51" s="46">
+        <f t="shared" si="2"/>
+        <v>41.159420289855071</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
+      <c r="A52" s="18">
+        <v>52</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>167</v>
+      </c>
+      <c r="C52" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="D52" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="E52" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="F52" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" s="20">
+        <v>6.6</v>
+      </c>
+      <c r="H52" s="21">
         <f t="shared" si="3"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="L48" s="18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A49" s="18">
-        <v>49</v>
-      </c>
-      <c r="B49" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="C49" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D49" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="E49" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="F49" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G49" s="20">
-        <v>0.09</v>
-      </c>
-      <c r="H49" s="21">
-        <f t="shared" si="2"/>
-        <v>1.3043478260869565E-2</v>
-      </c>
-      <c r="I49" s="28"/>
-      <c r="J49" s="22">
-        <v>50</v>
-      </c>
-      <c r="K49" s="23">
-        <f t="shared" si="3"/>
-        <v>0.65217391304347827</v>
-      </c>
-      <c r="L49" s="18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A50" s="18">
-        <v>50</v>
-      </c>
-      <c r="B50" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="C50" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D50" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="E50" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="F50" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="20">
-        <v>0.06</v>
-      </c>
-      <c r="H50" s="21">
-        <f t="shared" si="2"/>
-        <v>8.6956521739130418E-3</v>
-      </c>
-      <c r="I50" s="29"/>
-      <c r="J50" s="22">
-        <v>50</v>
-      </c>
-      <c r="K50" s="23">
-        <f t="shared" si="3"/>
-        <v>0.43478260869565211</v>
-      </c>
-      <c r="L50" s="18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A51" s="18">
-        <v>51</v>
-      </c>
-      <c r="B51" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D51" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="E51" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="F51" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G51" s="20">
-        <v>0.2</v>
-      </c>
-      <c r="H51" s="21">
-        <f t="shared" si="2"/>
-        <v>2.8985507246376812E-2</v>
-      </c>
-      <c r="I51" s="30"/>
-      <c r="J51" s="22">
-        <v>50</v>
-      </c>
-      <c r="K51" s="23">
-        <f t="shared" si="3"/>
-        <v>1.4492753623188406</v>
-      </c>
-      <c r="L51" s="18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
-      <c r="A52" s="18">
-        <v>52</v>
-      </c>
-      <c r="B52" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="D52" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="E52" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="F52" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="G52" s="20">
-        <v>6.6</v>
-      </c>
-      <c r="H52" s="21">
-        <f t="shared" si="2"/>
-        <v>0.9565217391304347</v>
-      </c>
-      <c r="I52" s="28"/>
+      <c r="I52" s="43"/>
       <c r="J52" s="22">
         <v>10</v>
       </c>
       <c r="K52" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9.5652173913043477</v>
       </c>
       <c r="L52" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="53" spans="1:12" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
+      <c r="M52" s="46">
+        <f t="shared" si="2"/>
+        <v>1358.2608695652173</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
       <c r="A53" s="18">
         <v>53</v>
       </c>
@@ -6290,22 +6498,26 @@
         <v>9.9</v>
       </c>
       <c r="H53" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.4347826086956521</v>
       </c>
-      <c r="I53" s="30"/>
+      <c r="I53" s="45"/>
       <c r="J53" s="22">
         <v>5</v>
       </c>
       <c r="K53" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7.1739130434782608</v>
       </c>
       <c r="L53" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="54" spans="1:12" s="24" customFormat="1" ht="45" customHeight="1">
+      <c r="M53" s="46">
+        <f t="shared" si="2"/>
+        <v>2037.391304347826</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" s="24" customFormat="1" ht="45" customHeight="1">
       <c r="A54" s="18">
         <v>54</v>
       </c>
@@ -6328,7 +6540,7 @@
         <v>14.85</v>
       </c>
       <c r="H54" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.152173913043478</v>
       </c>
       <c r="I54" s="19"/>
@@ -6336,14 +6548,18 @@
         <v>5</v>
       </c>
       <c r="K54" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10.760869565217391</v>
       </c>
       <c r="L54" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="55" spans="1:12" s="24" customFormat="1" ht="45" customHeight="1">
+      <c r="M54" s="46">
+        <f t="shared" si="2"/>
+        <v>3056.086956521739</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" s="24" customFormat="1" ht="45" customHeight="1">
       <c r="A55" s="18">
         <v>55</v>
       </c>
@@ -6366,7 +6582,7 @@
         <v>22</v>
       </c>
       <c r="H55" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1884057971014492</v>
       </c>
       <c r="I55" s="19"/>
@@ -6374,14 +6590,18 @@
         <v>5</v>
       </c>
       <c r="K55" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>15.942028985507246</v>
       </c>
       <c r="L55" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="56" spans="1:12" s="24" customFormat="1" ht="75.95" customHeight="1">
+      <c r="M55" s="46">
+        <f t="shared" si="2"/>
+        <v>4527.536231884058</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A56" s="18">
         <v>56</v>
       </c>
@@ -6404,7 +6624,7 @@
         <v>0.17</v>
       </c>
       <c r="H56" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.4637681159420291E-2</v>
       </c>
       <c r="I56" s="19"/>
@@ -6412,14 +6632,18 @@
         <v>50</v>
       </c>
       <c r="K56" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.2318840579710146</v>
       </c>
       <c r="L56" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="57" spans="1:12" s="24" customFormat="1" ht="75.95" customHeight="1">
+      <c r="M56" s="46">
+        <f t="shared" si="2"/>
+        <v>34.985507246376812</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A57" s="18">
         <v>57</v>
       </c>
@@ -6442,7 +6666,7 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="H57" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2753623188405798</v>
       </c>
       <c r="I57" s="19"/>
@@ -6450,22 +6674,26 @@
         <v>10</v>
       </c>
       <c r="K57" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>12.753623188405799</v>
       </c>
       <c r="L57" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="58" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
-      <c r="A58" s="33"/>
+      <c r="M57" s="46">
+        <f t="shared" si="2"/>
+        <v>1811.0144927536232</v>
+      </c>
+    </row>
+    <row r="58" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="A58" s="30"/>
       <c r="B58" s="19" t="s">
         <v>179</v>
       </c>
       <c r="C58" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="D58" s="33" t="s">
+      <c r="D58" s="30" t="s">
         <v>179</v>
       </c>
       <c r="E58" s="19" t="s">
@@ -6478,7 +6706,7 @@
         <v>0.44</v>
       </c>
       <c r="H58" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6.3768115942028983E-2</v>
       </c>
       <c r="I58" s="19"/>
@@ -6486,20 +6714,24 @@
         <v>50</v>
       </c>
       <c r="K58" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.1884057971014492</v>
       </c>
       <c r="L58" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="59" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A59" s="33"/>
+      <c r="M58" s="46">
+        <f t="shared" si="2"/>
+        <v>90.550724637681157</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A59" s="30"/>
       <c r="B59" s="19" t="s">
         <v>181</v>
       </c>
       <c r="C59" s="18"/>
-      <c r="D59" s="33" t="s">
+      <c r="D59" s="30" t="s">
         <v>182</v>
       </c>
       <c r="E59" s="19"/>
@@ -6518,20 +6750,24 @@
         <v>10</v>
       </c>
       <c r="K59" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.043478260869565</v>
       </c>
       <c r="L59" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A60" s="33"/>
+      <c r="M59" s="46">
+        <f t="shared" si="2"/>
+        <v>290.17391304347825</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A60" s="30"/>
       <c r="B60" s="19" t="s">
         <v>181</v>
       </c>
       <c r="C60" s="18"/>
-      <c r="D60" s="33" t="s">
+      <c r="D60" s="30" t="s">
         <v>183</v>
       </c>
       <c r="E60" s="19"/>
@@ -6542,7 +6778,7 @@
         <v>1.88</v>
       </c>
       <c r="H60" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.27246376811594197</v>
       </c>
       <c r="I60" s="19"/>
@@ -6550,19 +6786,23 @@
         <v>10</v>
       </c>
       <c r="K60" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.72463768115942</v>
       </c>
       <c r="L60" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="61" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A61" s="33"/>
+      <c r="M60" s="46">
+        <f t="shared" si="2"/>
+        <v>386.89855072463763</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A61" s="30"/>
       <c r="B61" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="C61" s="33"/>
+      <c r="C61" s="30"/>
       <c r="D61" s="18" t="s">
         <v>184</v>
       </c>
@@ -6572,11 +6812,11 @@
       <c r="F61" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G61" s="34">
+      <c r="G61" s="31">
         <v>2.0099999999999998</v>
       </c>
       <c r="H61" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.29130434782608688</v>
       </c>
       <c r="I61" s="19"/>
@@ -6584,19 +6824,23 @@
         <v>10</v>
       </c>
       <c r="K61" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.9130434782608687</v>
       </c>
       <c r="L61" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="62" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A62" s="33"/>
+      <c r="M61" s="46">
+        <f t="shared" si="2"/>
+        <v>413.65217391304338</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A62" s="30"/>
       <c r="B62" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="C62" s="33"/>
+      <c r="C62" s="30"/>
       <c r="D62" s="18" t="s">
         <v>199</v>
       </c>
@@ -6616,19 +6860,23 @@
         <v>10</v>
       </c>
       <c r="K62" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.043478260869565</v>
       </c>
       <c r="L62" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="63" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A63" s="33"/>
+      <c r="M62" s="46">
+        <f t="shared" si="2"/>
+        <v>290.17391304347825</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A63" s="30"/>
       <c r="B63" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="C63" s="33"/>
+      <c r="C63" s="30"/>
       <c r="D63" s="18" t="s">
         <v>200</v>
       </c>
@@ -6640,7 +6888,7 @@
         <v>1.88</v>
       </c>
       <c r="H63" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.27246376811594197</v>
       </c>
       <c r="I63" s="19"/>
@@ -6648,19 +6896,23 @@
         <v>10</v>
       </c>
       <c r="K63" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.72463768115942</v>
       </c>
       <c r="L63" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="64" spans="1:12" s="24" customFormat="1" ht="27" customHeight="1">
-      <c r="A64" s="33"/>
+      <c r="M63" s="46">
+        <f t="shared" si="2"/>
+        <v>386.89855072463763</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+      <c r="A64" s="30"/>
       <c r="B64" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="C64" s="33"/>
+      <c r="C64" s="30"/>
       <c r="D64" s="18" t="s">
         <v>201</v>
       </c>
@@ -6668,11 +6920,11 @@
       <c r="F64" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G64" s="34">
+      <c r="G64" s="31">
         <v>2.0099999999999998</v>
       </c>
       <c r="H64" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.29130434782608688</v>
       </c>
       <c r="I64" s="19"/>
@@ -6680,457 +6932,525 @@
         <v>10</v>
       </c>
       <c r="K64" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2.9130434782608687</v>
       </c>
       <c r="L64" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" s="24" customFormat="1" ht="78" customHeight="1">
-      <c r="A65" s="33"/>
-      <c r="B65" s="35"/>
-      <c r="C65" s="33"/>
-      <c r="D65" s="33" t="s">
+      <c r="M64" s="46">
+        <f t="shared" si="2"/>
+        <v>413.65217391304338</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" s="24" customFormat="1" ht="78" customHeight="1">
+      <c r="A65" s="30"/>
+      <c r="B65" s="32"/>
+      <c r="C65" s="30"/>
+      <c r="D65" s="30" t="s">
         <v>186</v>
       </c>
-      <c r="E65" s="33"/>
+      <c r="E65" s="30"/>
       <c r="F65" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G65" s="34">
+      <c r="G65" s="31">
         <v>0.88</v>
       </c>
       <c r="H65" s="21">
+        <f t="shared" si="3"/>
+        <v>0.12753623188405797</v>
+      </c>
+      <c r="I65" s="30"/>
+      <c r="J65" s="31">
+        <v>40</v>
+      </c>
+      <c r="K65" s="23">
+        <f t="shared" si="4"/>
+        <v>5.1014492753623184</v>
+      </c>
+      <c r="L65" s="30"/>
+      <c r="M65" s="46">
         <f t="shared" si="2"/>
-        <v>0.12753623188405797</v>
-      </c>
-      <c r="I65" s="33"/>
-      <c r="J65" s="34">
-        <v>40</v>
-      </c>
-      <c r="K65" s="23">
-        <f t="shared" si="3"/>
-        <v>5.1014492753623184</v>
-      </c>
-      <c r="L65" s="33"/>
-    </row>
-    <row r="66" spans="1:12" s="24" customFormat="1" ht="84" customHeight="1">
-      <c r="A66" s="33"/>
-      <c r="B66" s="35"/>
-      <c r="C66" s="33"/>
-      <c r="D66" s="33" t="s">
+        <v>181.10144927536231</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" s="24" customFormat="1" ht="84" customHeight="1">
+      <c r="A66" s="30"/>
+      <c r="B66" s="32"/>
+      <c r="C66" s="30"/>
+      <c r="D66" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="E66" s="33"/>
+      <c r="E66" s="30"/>
       <c r="F66" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G66" s="34">
+      <c r="G66" s="31">
         <v>2.5</v>
       </c>
       <c r="H66" s="21">
+        <f t="shared" si="3"/>
+        <v>0.36231884057971014</v>
+      </c>
+      <c r="I66" s="30"/>
+      <c r="J66" s="31">
+        <v>20</v>
+      </c>
+      <c r="K66" s="23">
+        <f t="shared" si="4"/>
+        <v>7.2463768115942031</v>
+      </c>
+      <c r="L66" s="30"/>
+      <c r="M66" s="46">
         <f t="shared" si="2"/>
-        <v>0.36231884057971014</v>
-      </c>
-      <c r="I66" s="33"/>
-      <c r="J66" s="34">
-        <v>20</v>
-      </c>
-      <c r="K66" s="23">
-        <f t="shared" si="3"/>
-        <v>7.2463768115942031</v>
-      </c>
-      <c r="L66" s="33"/>
-    </row>
-    <row r="67" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
-      <c r="A67" s="33"/>
-      <c r="B67" s="35"/>
-      <c r="C67" s="33"/>
-      <c r="D67" s="33" t="s">
+        <v>514.49275362318838</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="A67" s="30"/>
+      <c r="B67" s="32"/>
+      <c r="C67" s="30"/>
+      <c r="D67" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="E67" s="33"/>
+      <c r="E67" s="30"/>
       <c r="F67" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G67" s="34">
+      <c r="G67" s="31">
         <v>5</v>
       </c>
       <c r="H67" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.72463768115942029</v>
       </c>
-      <c r="I67" s="33"/>
-      <c r="J67" s="34">
+      <c r="I67" s="30"/>
+      <c r="J67" s="31">
         <v>5</v>
       </c>
       <c r="K67" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.6231884057971016</v>
       </c>
-      <c r="L67" s="33"/>
-    </row>
-    <row r="68" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
-      <c r="A68" s="33"/>
-      <c r="B68" s="35"/>
-      <c r="C68" s="33"/>
-      <c r="D68" s="33" t="s">
+      <c r="L67" s="30"/>
+      <c r="M67" s="46">
+        <f>1420*H67</f>
+        <v>1028.9855072463768</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="A68" s="30"/>
+      <c r="B68" s="32"/>
+      <c r="C68" s="30"/>
+      <c r="D68" s="30" t="s">
         <v>189</v>
       </c>
-      <c r="E68" s="33"/>
+      <c r="E68" s="30"/>
       <c r="F68" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G68" s="34">
+      <c r="G68" s="31">
         <v>50</v>
       </c>
       <c r="H68" s="21">
-        <f t="shared" si="2"/>
-        <v>7.2463768115942022</v>
-      </c>
-      <c r="I68" s="33"/>
-      <c r="J68" s="34">
-        <v>1</v>
-      </c>
-      <c r="K68" s="23">
         <f t="shared" si="3"/>
         <v>7.2463768115942022</v>
       </c>
-      <c r="L68" s="33"/>
-    </row>
-    <row r="69" spans="1:12" s="24" customFormat="1" ht="75.95" customHeight="1">
-      <c r="A69" s="33"/>
-      <c r="B69" s="35"/>
-      <c r="C69" s="33"/>
-      <c r="D69" s="33" t="s">
+      <c r="I68" s="30"/>
+      <c r="J68" s="31">
+        <v>1</v>
+      </c>
+      <c r="K68" s="23">
+        <f t="shared" si="4"/>
+        <v>7.2463768115942022</v>
+      </c>
+      <c r="L68" s="30"/>
+      <c r="M68" s="46">
+        <f t="shared" ref="M67:M80" si="5">1420*H68</f>
+        <v>10289.855072463768</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+      <c r="A69" s="30"/>
+      <c r="B69" s="32"/>
+      <c r="C69" s="30"/>
+      <c r="D69" s="30" t="s">
         <v>190</v>
       </c>
-      <c r="E69" s="33"/>
+      <c r="E69" s="30"/>
       <c r="F69" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G69" s="34">
+      <c r="G69" s="31">
         <v>2.09</v>
       </c>
       <c r="H69" s="21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.30289855072463767</v>
       </c>
-      <c r="I69" s="33"/>
-      <c r="J69" s="34">
+      <c r="I69" s="30"/>
+      <c r="J69" s="31">
         <v>20</v>
       </c>
       <c r="K69" s="23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>6.0579710144927539</v>
       </c>
-      <c r="L69" s="33"/>
-    </row>
-    <row r="70" spans="1:12" s="24" customFormat="1" ht="69" customHeight="1">
-      <c r="A70" s="33"/>
-      <c r="B70" s="35"/>
-      <c r="C70" s="33"/>
-      <c r="D70" s="33" t="s">
+      <c r="L69" s="30"/>
+      <c r="M69" s="46">
+        <f t="shared" si="5"/>
+        <v>430.1159420289855</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" s="24" customFormat="1" ht="69" customHeight="1">
+      <c r="A70" s="30"/>
+      <c r="B70" s="32"/>
+      <c r="C70" s="30"/>
+      <c r="D70" s="30" t="s">
         <v>191</v>
       </c>
-      <c r="E70" s="33"/>
+      <c r="E70" s="30"/>
       <c r="F70" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G70" s="34">
+      <c r="G70" s="31">
         <v>0.13</v>
       </c>
       <c r="H70" s="21">
-        <f t="shared" ref="H70:H75" si="4">G70/6.9</f>
+        <f t="shared" ref="H70:H75" si="6">G70/6.9</f>
         <v>1.8840579710144929E-2</v>
       </c>
-      <c r="I70" s="33"/>
-      <c r="J70" s="34">
+      <c r="I70" s="30"/>
+      <c r="J70" s="31">
         <v>50</v>
       </c>
       <c r="K70" s="23">
-        <f t="shared" ref="K70:K75" si="5">J70*H70</f>
+        <f t="shared" ref="K70:K75" si="7">J70*H70</f>
         <v>0.94202898550724645</v>
       </c>
-      <c r="L70" s="33"/>
-    </row>
-    <row r="71" spans="1:12" s="24" customFormat="1" ht="81" customHeight="1">
-      <c r="A71" s="33"/>
-      <c r="B71" s="35"/>
-      <c r="C71" s="33"/>
-      <c r="D71" s="35" t="s">
+      <c r="L70" s="30"/>
+      <c r="M70" s="46">
+        <f t="shared" si="5"/>
+        <v>26.753623188405797</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+      <c r="A71" s="30"/>
+      <c r="B71" s="32"/>
+      <c r="C71" s="30"/>
+      <c r="D71" s="32" t="s">
         <v>192</v>
       </c>
-      <c r="E71" s="33"/>
+      <c r="E71" s="30"/>
       <c r="F71" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G71" s="34">
+      <c r="G71" s="31">
         <v>13.2</v>
       </c>
       <c r="H71" s="21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.9130434782608694</v>
       </c>
-      <c r="I71" s="33"/>
-      <c r="J71" s="34">
+      <c r="I71" s="30"/>
+      <c r="J71" s="31">
         <v>10</v>
       </c>
       <c r="K71" s="23">
+        <f t="shared" si="7"/>
+        <v>19.130434782608695</v>
+      </c>
+      <c r="L71" s="30"/>
+      <c r="M71" s="46">
         <f t="shared" si="5"/>
-        <v>19.130434782608695</v>
-      </c>
-      <c r="L71" s="33"/>
-    </row>
-    <row r="72" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A72" s="33"/>
-      <c r="B72" s="35"/>
-      <c r="C72" s="33"/>
-      <c r="D72" s="33" t="s">
+        <v>2716.5217391304345</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A72" s="30"/>
+      <c r="B72" s="32"/>
+      <c r="C72" s="30"/>
+      <c r="D72" s="30" t="s">
         <v>193</v>
       </c>
-      <c r="E72" s="33"/>
+      <c r="E72" s="30"/>
       <c r="F72" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G72" s="34">
+      <c r="G72" s="31">
         <v>3.85</v>
       </c>
       <c r="H72" s="21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.55797101449275366</v>
       </c>
-      <c r="I72" s="33"/>
-      <c r="J72" s="34">
+      <c r="I72" s="30"/>
+      <c r="J72" s="31">
         <v>10</v>
       </c>
       <c r="K72" s="23">
+        <f t="shared" si="7"/>
+        <v>5.579710144927537</v>
+      </c>
+      <c r="L72" s="30"/>
+      <c r="M72" s="46">
         <f t="shared" si="5"/>
-        <v>5.579710144927537</v>
-      </c>
-      <c r="L72" s="33"/>
-    </row>
-    <row r="73" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A73" s="33"/>
-      <c r="B73" s="35"/>
-      <c r="C73" s="33"/>
-      <c r="D73" s="33" t="s">
+        <v>792.31884057971024</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A73" s="30"/>
+      <c r="B73" s="32"/>
+      <c r="C73" s="30"/>
+      <c r="D73" s="30" t="s">
         <v>194</v>
       </c>
-      <c r="E73" s="33"/>
+      <c r="E73" s="30"/>
       <c r="F73" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G73" s="34">
+      <c r="G73" s="31">
         <v>5.15</v>
       </c>
       <c r="H73" s="21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>0.74637681159420288</v>
       </c>
-      <c r="I73" s="33"/>
-      <c r="J73" s="34">
+      <c r="I73" s="30"/>
+      <c r="J73" s="31">
         <v>10</v>
       </c>
       <c r="K73" s="23">
+        <f t="shared" si="7"/>
+        <v>7.4637681159420293</v>
+      </c>
+      <c r="L73" s="30"/>
+      <c r="M73" s="46">
         <f t="shared" si="5"/>
-        <v>7.4637681159420293</v>
-      </c>
-      <c r="L73" s="33"/>
-    </row>
-    <row r="74" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A74" s="33"/>
-      <c r="B74" s="35"/>
-      <c r="C74" s="33"/>
-      <c r="D74" s="33" t="s">
+        <v>1059.855072463768</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A74" s="30"/>
+      <c r="B74" s="32"/>
+      <c r="C74" s="30"/>
+      <c r="D74" s="30" t="s">
         <v>195</v>
       </c>
-      <c r="E74" s="33"/>
+      <c r="E74" s="30"/>
       <c r="F74" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G74" s="34">
+      <c r="G74" s="31">
         <v>8.25</v>
       </c>
       <c r="H74" s="21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>1.1956521739130435</v>
       </c>
-      <c r="I74" s="33"/>
-      <c r="J74" s="34">
+      <c r="I74" s="30"/>
+      <c r="J74" s="31">
         <v>10</v>
       </c>
       <c r="K74" s="23">
+        <f t="shared" si="7"/>
+        <v>11.956521739130434</v>
+      </c>
+      <c r="L74" s="30"/>
+      <c r="M74" s="46">
         <f t="shared" si="5"/>
-        <v>11.956521739130434</v>
-      </c>
-      <c r="L74" s="33"/>
-    </row>
-    <row r="75" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A75" s="33"/>
-      <c r="B75" s="35"/>
-      <c r="C75" s="33"/>
-      <c r="D75" s="33" t="s">
+        <v>1697.8260869565217</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A75" s="30"/>
+      <c r="B75" s="32"/>
+      <c r="C75" s="30"/>
+      <c r="D75" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="E75" s="33"/>
+      <c r="E75" s="30"/>
       <c r="F75" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G75" s="34">
+      <c r="G75" s="31">
         <v>0.44</v>
       </c>
       <c r="H75" s="21">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>6.3768115942028983E-2</v>
       </c>
-      <c r="I75" s="33"/>
-      <c r="J75" s="34">
+      <c r="I75" s="30"/>
+      <c r="J75" s="31">
         <v>20</v>
       </c>
       <c r="K75" s="23">
+        <f t="shared" si="7"/>
+        <v>1.2753623188405796</v>
+      </c>
+      <c r="L75" s="30"/>
+      <c r="M75" s="46">
         <f t="shared" si="5"/>
-        <v>1.2753623188405796</v>
-      </c>
-      <c r="L75" s="33"/>
-    </row>
-    <row r="76" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A76" s="33"/>
-      <c r="B76" s="35"/>
-      <c r="C76" s="36" t="s">
+        <v>90.550724637681157</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A76" s="30"/>
+      <c r="B76" s="32"/>
+      <c r="C76" s="33" t="s">
         <v>197</v>
       </c>
-      <c r="D76" s="37" t="s">
+      <c r="D76" s="34" t="s">
         <v>198</v>
       </c>
-      <c r="E76" s="38" t="s">
+      <c r="E76" s="35" t="s">
         <v>115</v>
       </c>
       <c r="F76" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="G76" s="39"/>
-      <c r="H76" s="40">
+      <c r="G76" s="36"/>
+      <c r="H76" s="37">
         <v>29.8571428571429</v>
       </c>
-      <c r="I76" s="33"/>
-      <c r="J76" s="34">
+      <c r="I76" s="30"/>
+      <c r="J76" s="31">
         <v>1</v>
       </c>
       <c r="K76" s="23">
         <v>29.8571428571429</v>
       </c>
-      <c r="L76" s="33"/>
-    </row>
-    <row r="77" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A77" s="33"/>
-      <c r="B77" s="35"/>
-      <c r="C77" s="41" t="s">
+      <c r="L76" s="30"/>
+      <c r="M76" s="46">
+        <f t="shared" si="5"/>
+        <v>42397.142857142921</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A77" s="30"/>
+      <c r="B77" s="32"/>
+      <c r="C77" s="38" t="s">
         <v>202</v>
       </c>
-      <c r="D77" s="42" t="s">
+      <c r="D77" s="39" t="s">
         <v>203</v>
       </c>
-      <c r="E77" s="41" t="s">
+      <c r="E77" s="38" t="s">
         <v>204</v>
       </c>
       <c r="F77" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="G77" s="39"/>
-      <c r="H77" s="43">
+      <c r="G77" s="36"/>
+      <c r="H77" s="40">
         <v>8.4060000000000006</v>
       </c>
-      <c r="I77" s="33"/>
-      <c r="J77" s="34">
+      <c r="I77" s="30"/>
+      <c r="J77" s="31">
         <v>4</v>
       </c>
       <c r="K77" s="23">
         <f>H77*J77</f>
         <v>33.624000000000002</v>
       </c>
-      <c r="L77" s="33"/>
-    </row>
-    <row r="78" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A78" s="33"/>
-      <c r="B78" s="35"/>
-      <c r="C78" s="41" t="s">
+      <c r="L77" s="30"/>
+      <c r="M77" s="46">
+        <f t="shared" si="5"/>
+        <v>11936.52</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A78" s="30"/>
+      <c r="B78" s="32"/>
+      <c r="C78" s="38" t="s">
         <v>205</v>
       </c>
-      <c r="D78" s="42" t="s">
+      <c r="D78" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="E78" s="41"/>
+      <c r="E78" s="38"/>
       <c r="F78" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G78" s="39"/>
-      <c r="H78" s="43">
+      <c r="G78" s="36"/>
+      <c r="H78" s="40">
         <v>0.877</v>
       </c>
-      <c r="I78" s="33"/>
-      <c r="J78" s="34">
+      <c r="I78" s="30"/>
+      <c r="J78" s="31">
         <v>5</v>
       </c>
       <c r="K78" s="23">
         <f>J78*H78</f>
         <v>4.3849999999999998</v>
       </c>
-      <c r="L78" s="33"/>
-    </row>
-    <row r="79" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A79" s="33"/>
-      <c r="B79" s="35"/>
-      <c r="C79" s="44" t="s">
+      <c r="L78" s="30"/>
+      <c r="M78" s="46">
+        <f t="shared" si="5"/>
+        <v>1245.3399999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A79" s="30"/>
+      <c r="B79" s="32"/>
+      <c r="C79" s="41" t="s">
         <v>209</v>
       </c>
-      <c r="D79" s="42" t="s">
+      <c r="D79" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="E79" s="41"/>
+      <c r="E79" s="38"/>
       <c r="F79" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G79" s="39"/>
-      <c r="H79" s="43">
+      <c r="G79" s="36"/>
+      <c r="H79" s="40">
         <v>3.5070000000000001</v>
       </c>
-      <c r="I79" s="33"/>
-      <c r="J79" s="34">
+      <c r="I79" s="30"/>
+      <c r="J79" s="31">
         <v>5</v>
       </c>
       <c r="K79" s="23">
         <f>H79*J79</f>
         <v>17.535</v>
       </c>
-      <c r="L79" s="33"/>
-    </row>
-    <row r="80" spans="1:12" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A80" s="33"/>
-      <c r="B80" s="35"/>
+      <c r="L79" s="30"/>
+      <c r="M79" s="46">
+        <f t="shared" si="5"/>
+        <v>4979.9400000000005</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+      <c r="A80" s="30"/>
+      <c r="B80" s="32"/>
       <c r="C80" s="24" t="s">
         <v>207</v>
       </c>
-      <c r="D80" s="41" t="s">
+      <c r="D80" s="38" t="s">
         <v>208</v>
       </c>
-      <c r="E80" s="41"/>
+      <c r="E80" s="38"/>
       <c r="F80" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G80" s="39"/>
-      <c r="H80" s="45">
+      <c r="G80" s="36"/>
+      <c r="H80" s="42">
         <v>5.87</v>
       </c>
-      <c r="I80" s="33"/>
-      <c r="J80" s="34">
+      <c r="I80" s="30"/>
+      <c r="J80" s="31">
         <v>1</v>
       </c>
       <c r="K80" s="23">
         <v>5.87</v>
       </c>
-      <c r="L80" s="33"/>
+      <c r="L80" s="30"/>
+      <c r="M80" s="46">
+        <f t="shared" si="5"/>
+        <v>8335.4</v>
+      </c>
     </row>
     <row r="81" spans="1:12" ht="18.75">
       <c r="A81" s="15"/>

</xml_diff>

<commit_message>
feat: add 5 premium driftwood products and sync database migrations
</commit_message>
<xml_diff>
--- a/Binzhou_Houyi (1) (1).xlsx
+++ b/Binzhou_Houyi (1) (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Desktop\upload\FishWebClean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3774F72C-24EF-4548-A9DC-93D5F2D0065C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31F4617-BEDE-4963-9471-454D9AEDAD26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -687,10 +687,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="\$#,##0.00;\-\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.000;\-\$#,##0.000"/>
-    <numFmt numFmtId="170" formatCode="_([$IQD]\ * #,##0_);_([$IQD]\ * \(#,##0\);_([$IQD]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_([$IQD]\ * #,##0_);_([$IQD]\ * \(#,##0\);_([$IQD]\ * &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="_([$IQD]\ * #,##0.00_);_([$IQD]\ * \(#,##0.00\);_([$IQD]\ * &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -782,7 +783,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -842,6 +843,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -858,7 +872,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -984,6 +998,9 @@
     <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -993,7 +1010,22 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2942,15 +2974,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>145257</xdr:colOff>
+      <xdr:colOff>2382</xdr:colOff>
       <xdr:row>51</xdr:row>
-      <xdr:rowOff>421482</xdr:rowOff>
+      <xdr:rowOff>28576</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>100489</xdr:colOff>
-      <xdr:row>53</xdr:row>
-      <xdr:rowOff>314167</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>886302</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>349886</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2973,7 +3005,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="10015538" y="40950357"/>
+          <a:off x="9872663" y="40557451"/>
           <a:ext cx="883920" cy="749935"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4284,7 +4316,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M83"/>
+  <dimension ref="A1:Q83"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -4300,10 +4332,14 @@
     <col min="11" max="11" width="13.85546875" style="4" customWidth="1"/>
     <col min="12" max="12" width="33.140625" style="1" customWidth="1"/>
     <col min="13" max="13" width="25.28515625" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="9" style="1"/>
+    <col min="14" max="14" width="20.28515625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17" style="1" customWidth="1"/>
+    <col min="16" max="16" width="20.140625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="28.140625" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30">
+    <row r="1" spans="1:17" ht="30">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -4337,7 +4373,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:13" s="24" customFormat="1" ht="75" customHeight="1">
+    <row r="2" spans="1:17" s="24" customFormat="1" ht="75" customHeight="1">
       <c r="A2" s="18">
         <v>1</v>
       </c>
@@ -4374,12 +4410,28 @@
       <c r="L2" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="46">
+      <c r="M2" s="43">
         <f>1420*H2</f>
         <v>5433.0434782608691</v>
       </c>
+      <c r="N2" s="51">
+        <f t="shared" ref="N2:N65" si="0">M2*J2</f>
+        <v>16299.130434782608</v>
+      </c>
+      <c r="O2" s="50">
+        <f>(18000*J2)</f>
+        <v>54000</v>
+      </c>
+      <c r="P2" s="51">
+        <f t="shared" ref="P2:P65" si="1">O2-N2</f>
+        <v>37700.869565217392</v>
+      </c>
+      <c r="Q2" s="47">
+        <f t="shared" ref="Q2:Q65" si="2">P2/J2</f>
+        <v>12566.95652173913</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" s="24" customFormat="1" ht="84" customHeight="1">
+    <row r="3" spans="1:17" s="24" customFormat="1" ht="84" customHeight="1">
       <c r="A3" s="25">
         <v>2</v>
       </c>
@@ -4402,7 +4454,7 @@
         <v>2.42</v>
       </c>
       <c r="H3" s="21">
-        <f t="shared" ref="H3:H34" si="0">G3/6.9</f>
+        <f t="shared" ref="H3:H34" si="3">G3/6.9</f>
         <v>0.35072463768115941</v>
       </c>
       <c r="I3" s="19"/>
@@ -4410,18 +4462,34 @@
         <v>5</v>
       </c>
       <c r="K3" s="23">
-        <f t="shared" ref="K3:K34" si="1">J3*H3</f>
+        <f t="shared" ref="K3:K34" si="4">J3*H3</f>
         <v>1.7536231884057971</v>
       </c>
       <c r="L3" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="46">
-        <f t="shared" ref="M3:M66" si="2">1420*H3</f>
+      <c r="M3" s="43">
+        <f t="shared" ref="M3:M66" si="5">1420*H3</f>
         <v>498.02898550724638</v>
       </c>
+      <c r="N3" s="51">
+        <f t="shared" si="0"/>
+        <v>2490.144927536232</v>
+      </c>
+      <c r="O3" s="50">
+        <f>(3000*J3)</f>
+        <v>15000</v>
+      </c>
+      <c r="P3" s="51">
+        <f t="shared" si="1"/>
+        <v>12509.855072463768</v>
+      </c>
+      <c r="Q3" s="47">
+        <f t="shared" si="2"/>
+        <v>2501.9710144927535</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" s="24" customFormat="1" ht="78.95" customHeight="1">
+    <row r="4" spans="1:17" s="24" customFormat="1" ht="78.95" customHeight="1">
       <c r="A4" s="18">
         <v>3</v>
       </c>
@@ -4444,7 +4512,7 @@
         <v>4.7</v>
       </c>
       <c r="H4" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.6811594202898551</v>
       </c>
       <c r="I4" s="19"/>
@@ -4452,18 +4520,34 @@
         <v>5</v>
       </c>
       <c r="K4" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>3.4057971014492754</v>
       </c>
       <c r="L4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="46">
+      <c r="M4" s="43">
+        <f t="shared" si="5"/>
+        <v>967.24637681159425</v>
+      </c>
+      <c r="N4" s="51">
+        <f t="shared" si="0"/>
+        <v>4836.231884057971</v>
+      </c>
+      <c r="O4" s="50">
+        <f>(6000*J4)</f>
+        <v>30000</v>
+      </c>
+      <c r="P4" s="51">
+        <f t="shared" si="1"/>
+        <v>25163.768115942028</v>
+      </c>
+      <c r="Q4" s="47">
         <f t="shared" si="2"/>
-        <v>967.24637681159425</v>
+        <v>5032.753623188406</v>
       </c>
     </row>
-    <row r="5" spans="1:13" s="24" customFormat="1" ht="80.099999999999994" customHeight="1">
+    <row r="5" spans="1:17" s="24" customFormat="1" ht="80.099999999999994" customHeight="1">
       <c r="A5" s="18">
         <v>4</v>
       </c>
@@ -4486,7 +4570,7 @@
         <v>9.68</v>
       </c>
       <c r="H5" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.4028985507246376</v>
       </c>
       <c r="I5" s="19"/>
@@ -4494,18 +4578,34 @@
         <v>5</v>
       </c>
       <c r="K5" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>7.0144927536231885</v>
       </c>
       <c r="L5" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="46">
+      <c r="M5" s="43">
+        <f t="shared" si="5"/>
+        <v>1992.1159420289855</v>
+      </c>
+      <c r="N5" s="51">
+        <f t="shared" si="0"/>
+        <v>9960.579710144928</v>
+      </c>
+      <c r="O5" s="50">
+        <f>(10000*J5)</f>
+        <v>50000</v>
+      </c>
+      <c r="P5" s="51">
+        <f t="shared" si="1"/>
+        <v>40039.420289855072</v>
+      </c>
+      <c r="Q5" s="47">
         <f t="shared" si="2"/>
-        <v>1992.1159420289855</v>
+        <v>8007.884057971014</v>
       </c>
     </row>
-    <row r="6" spans="1:13" s="24" customFormat="1" ht="63" customHeight="1">
+    <row r="6" spans="1:17" s="24" customFormat="1" ht="63" customHeight="1">
       <c r="A6" s="18">
         <v>5</v>
       </c>
@@ -4528,7 +4628,7 @@
         <v>5.5</v>
       </c>
       <c r="H6" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.79710144927536231</v>
       </c>
       <c r="I6" s="19"/>
@@ -4536,18 +4636,34 @@
         <v>15</v>
       </c>
       <c r="K6" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>11.956521739130434</v>
       </c>
       <c r="L6" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M6" s="46">
+      <c r="M6" s="43">
+        <f t="shared" si="5"/>
+        <v>1131.8840579710145</v>
+      </c>
+      <c r="N6" s="51">
+        <f t="shared" si="0"/>
+        <v>16978.260869565216</v>
+      </c>
+      <c r="O6" s="50">
+        <f>(3500*J6)</f>
+        <v>52500</v>
+      </c>
+      <c r="P6" s="51">
+        <f t="shared" si="1"/>
+        <v>35521.739130434784</v>
+      </c>
+      <c r="Q6" s="47">
         <f t="shared" si="2"/>
-        <v>1131.8840579710145</v>
+        <v>2368.1159420289855</v>
       </c>
     </row>
-    <row r="7" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
+    <row r="7" spans="1:17" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A7" s="18">
         <v>6</v>
       </c>
@@ -4570,7 +4686,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="H7" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.15942028985507248</v>
       </c>
       <c r="I7" s="19"/>
@@ -4578,18 +4694,34 @@
         <v>15</v>
       </c>
       <c r="K7" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>2.3913043478260874</v>
       </c>
       <c r="L7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="46">
+      <c r="M7" s="43">
+        <f t="shared" si="5"/>
+        <v>226.37681159420291</v>
+      </c>
+      <c r="N7" s="51">
+        <f t="shared" si="0"/>
+        <v>3395.6521739130435</v>
+      </c>
+      <c r="O7" s="50">
+        <f>(1500*J7)</f>
+        <v>22500</v>
+      </c>
+      <c r="P7" s="51">
+        <f t="shared" si="1"/>
+        <v>19104.347826086956</v>
+      </c>
+      <c r="Q7" s="47">
         <f t="shared" si="2"/>
-        <v>226.37681159420291</v>
+        <v>1273.623188405797</v>
       </c>
     </row>
-    <row r="8" spans="1:13" s="24" customFormat="1" ht="66.95" customHeight="1">
+    <row r="8" spans="1:17" s="24" customFormat="1" ht="66.95" customHeight="1">
       <c r="A8" s="18">
         <v>7</v>
       </c>
@@ -4612,7 +4744,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="H8" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.15942028985507248</v>
       </c>
       <c r="I8" s="19"/>
@@ -4620,18 +4752,34 @@
         <v>20</v>
       </c>
       <c r="K8" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>3.1884057971014497</v>
       </c>
       <c r="L8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M8" s="46">
+      <c r="M8" s="43">
+        <f t="shared" si="5"/>
+        <v>226.37681159420291</v>
+      </c>
+      <c r="N8" s="51">
+        <f t="shared" si="0"/>
+        <v>4527.536231884058</v>
+      </c>
+      <c r="O8" s="50">
+        <f>(1500*J8)</f>
+        <v>30000</v>
+      </c>
+      <c r="P8" s="51">
+        <f t="shared" si="1"/>
+        <v>25472.463768115944</v>
+      </c>
+      <c r="Q8" s="47">
         <f t="shared" si="2"/>
-        <v>226.37681159420291</v>
+        <v>1273.6231884057972</v>
       </c>
     </row>
-    <row r="9" spans="1:13" s="24" customFormat="1" ht="69.95" customHeight="1">
+    <row r="9" spans="1:17" s="24" customFormat="1" ht="69.95" customHeight="1">
       <c r="A9" s="18">
         <v>8</v>
       </c>
@@ -4654,7 +4802,7 @@
         <v>17.600000000000001</v>
       </c>
       <c r="H9" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>2.5507246376811596</v>
       </c>
       <c r="I9" s="19"/>
@@ -4662,18 +4810,34 @@
         <v>5</v>
       </c>
       <c r="K9" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>12.753623188405799</v>
       </c>
       <c r="L9" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="46">
+      <c r="M9" s="43">
+        <f t="shared" si="5"/>
+        <v>3622.0289855072465</v>
+      </c>
+      <c r="N9" s="51">
+        <f t="shared" si="0"/>
+        <v>18110.144927536232</v>
+      </c>
+      <c r="O9" s="50">
+        <f>(12000*J9)</f>
+        <v>60000</v>
+      </c>
+      <c r="P9" s="51">
+        <f t="shared" si="1"/>
+        <v>41889.855072463768</v>
+      </c>
+      <c r="Q9" s="47">
         <f t="shared" si="2"/>
-        <v>3622.0289855072465</v>
+        <v>8377.971014492754</v>
       </c>
     </row>
-    <row r="10" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
+    <row r="10" spans="1:17" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A10" s="18">
         <v>9</v>
       </c>
@@ -4696,7 +4860,7 @@
         <v>10.89</v>
       </c>
       <c r="H10" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.5782608695652174</v>
       </c>
       <c r="I10" s="19"/>
@@ -4704,18 +4868,34 @@
         <v>8</v>
       </c>
       <c r="K10" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>12.626086956521739</v>
       </c>
       <c r="L10" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M10" s="46">
+      <c r="M10" s="43">
+        <f t="shared" si="5"/>
+        <v>2241.1304347826085</v>
+      </c>
+      <c r="N10" s="51">
+        <f t="shared" si="0"/>
+        <v>17929.043478260868</v>
+      </c>
+      <c r="O10" s="50">
+        <f>(6000*J10)</f>
+        <v>48000</v>
+      </c>
+      <c r="P10" s="51">
+        <f t="shared" si="1"/>
+        <v>30070.956521739132</v>
+      </c>
+      <c r="Q10" s="47">
         <f t="shared" si="2"/>
-        <v>2241.1304347826085</v>
+        <v>3758.8695652173915</v>
       </c>
     </row>
-    <row r="11" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
+    <row r="11" spans="1:17" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A11" s="18">
         <v>10</v>
       </c>
@@ -4738,26 +4918,42 @@
         <v>32</v>
       </c>
       <c r="H11" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>4.63768115942029</v>
       </c>
-      <c r="I11" s="43"/>
+      <c r="I11" s="44"/>
       <c r="J11" s="22">
         <v>2</v>
       </c>
       <c r="K11" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>9.27536231884058</v>
       </c>
       <c r="L11" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M11" s="46">
+      <c r="M11" s="43">
+        <f t="shared" si="5"/>
+        <v>6585.507246376812</v>
+      </c>
+      <c r="N11" s="51">
+        <f t="shared" si="0"/>
+        <v>13171.014492753624</v>
+      </c>
+      <c r="O11" s="50">
+        <f>(20000*J11)</f>
+        <v>40000</v>
+      </c>
+      <c r="P11" s="51">
+        <f t="shared" si="1"/>
+        <v>26828.985507246376</v>
+      </c>
+      <c r="Q11" s="47">
         <f t="shared" si="2"/>
-        <v>6585.507246376812</v>
+        <v>13414.492753623188</v>
       </c>
     </row>
-    <row r="12" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
+    <row r="12" spans="1:17" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A12" s="18">
         <v>11</v>
       </c>
@@ -4780,26 +4976,42 @@
         <v>50</v>
       </c>
       <c r="H12" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>7.2463768115942022</v>
       </c>
-      <c r="I12" s="44"/>
+      <c r="I12" s="45"/>
       <c r="J12" s="22">
         <v>2</v>
       </c>
       <c r="K12" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>14.492753623188404</v>
       </c>
       <c r="L12" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M12" s="46">
+      <c r="M12" s="43">
+        <f t="shared" si="5"/>
+        <v>10289.855072463768</v>
+      </c>
+      <c r="N12" s="51">
+        <f t="shared" si="0"/>
+        <v>20579.710144927536</v>
+      </c>
+      <c r="O12" s="50">
+        <f>(40000*J12)</f>
+        <v>80000</v>
+      </c>
+      <c r="P12" s="51">
+        <f t="shared" si="1"/>
+        <v>59420.289855072464</v>
+      </c>
+      <c r="Q12" s="47">
         <f t="shared" si="2"/>
-        <v>10289.855072463768</v>
+        <v>29710.144927536232</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
+    <row r="13" spans="1:17" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A13" s="18">
         <v>12</v>
       </c>
@@ -4822,26 +5034,42 @@
         <v>28</v>
       </c>
       <c r="H13" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>4.057971014492753</v>
       </c>
-      <c r="I13" s="44"/>
+      <c r="I13" s="45"/>
       <c r="J13" s="22">
         <v>2</v>
       </c>
       <c r="K13" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>8.115942028985506</v>
       </c>
       <c r="L13" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M13" s="46">
+      <c r="M13" s="43">
+        <f t="shared" si="5"/>
+        <v>5762.3188405797091</v>
+      </c>
+      <c r="N13" s="51">
+        <f t="shared" si="0"/>
+        <v>11524.637681159418</v>
+      </c>
+      <c r="O13" s="50">
+        <f t="shared" ref="O2:O65" si="6">(20000*J13)</f>
+        <v>40000</v>
+      </c>
+      <c r="P13" s="51">
+        <f t="shared" si="1"/>
+        <v>28475.362318840584</v>
+      </c>
+      <c r="Q13" s="47">
         <f t="shared" si="2"/>
-        <v>5762.3188405797091</v>
+        <v>14237.681159420292</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="24" customFormat="1" ht="21" customHeight="1">
+    <row r="14" spans="1:17" s="24" customFormat="1" ht="21" customHeight="1">
       <c r="A14" s="18">
         <v>13</v>
       </c>
@@ -4864,26 +5092,42 @@
         <v>32</v>
       </c>
       <c r="H14" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>4.63768115942029</v>
       </c>
-      <c r="I14" s="45"/>
+      <c r="I14" s="46"/>
       <c r="J14" s="22">
         <v>3</v>
       </c>
       <c r="K14" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>13.913043478260871</v>
       </c>
       <c r="L14" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M14" s="46">
+      <c r="M14" s="43">
+        <f t="shared" si="5"/>
+        <v>6585.507246376812</v>
+      </c>
+      <c r="N14" s="51">
+        <f t="shared" si="0"/>
+        <v>19756.521739130436</v>
+      </c>
+      <c r="O14" s="50">
+        <f t="shared" si="6"/>
+        <v>60000</v>
+      </c>
+      <c r="P14" s="51">
+        <f t="shared" si="1"/>
+        <v>40243.478260869568</v>
+      </c>
+      <c r="Q14" s="47">
         <f t="shared" si="2"/>
-        <v>6585.507246376812</v>
+        <v>13414.49275362319</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+    <row r="15" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A15" s="18">
         <v>14</v>
       </c>
@@ -4906,7 +5150,7 @@
         <v>36</v>
       </c>
       <c r="H15" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>5.2173913043478262</v>
       </c>
       <c r="I15" s="19"/>
@@ -4914,18 +5158,31 @@
         <v>2</v>
       </c>
       <c r="K15" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10.434782608695652</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M15" s="46">
+      <c r="M15" s="43">
+        <f t="shared" si="5"/>
+        <v>7408.695652173913</v>
+      </c>
+      <c r="N15" s="51">
+        <f t="shared" si="0"/>
+        <v>14817.391304347826</v>
+      </c>
+      <c r="O15" s="50">
+        <f>(28000*J15)</f>
+        <v>56000</v>
+      </c>
+      <c r="P15" s="51"/>
+      <c r="Q15" s="47">
         <f t="shared" si="2"/>
-        <v>7408.695652173913</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="24" customFormat="1" ht="74.099999999999994" customHeight="1">
+    <row r="16" spans="1:17" s="24" customFormat="1" ht="74.099999999999994" customHeight="1">
       <c r="A16" s="18">
         <v>15</v>
       </c>
@@ -4948,7 +5205,7 @@
         <v>13.2</v>
       </c>
       <c r="H16" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.9130434782608694</v>
       </c>
       <c r="I16" s="19"/>
@@ -4956,18 +5213,28 @@
         <v>5</v>
       </c>
       <c r="K16" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>9.5652173913043477</v>
       </c>
       <c r="L16" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M16" s="46">
+      <c r="M16" s="43">
+        <f t="shared" si="5"/>
+        <v>2716.5217391304345</v>
+      </c>
+      <c r="N16" s="51">
+        <f t="shared" si="0"/>
+        <v>13582.608695652172</v>
+      </c>
+      <c r="O16" s="50"/>
+      <c r="P16" s="51"/>
+      <c r="Q16" s="47">
         <f t="shared" si="2"/>
-        <v>2716.5217391304345</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
+    <row r="17" spans="1:17" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A17" s="18">
         <v>16</v>
       </c>
@@ -4990,26 +5257,36 @@
         <v>1</v>
       </c>
       <c r="H17" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.14492753623188406</v>
       </c>
-      <c r="I17" s="43"/>
+      <c r="I17" s="44"/>
       <c r="J17" s="22">
         <v>5</v>
       </c>
       <c r="K17" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0.72463768115942029</v>
       </c>
       <c r="L17" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="46">
+      <c r="M17" s="43">
+        <f t="shared" si="5"/>
+        <v>205.79710144927537</v>
+      </c>
+      <c r="N17" s="51">
+        <f t="shared" si="0"/>
+        <v>1028.985507246377</v>
+      </c>
+      <c r="O17" s="50"/>
+      <c r="P17" s="51"/>
+      <c r="Q17" s="47">
         <f t="shared" si="2"/>
-        <v>205.79710144927537</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
+    <row r="18" spans="1:17" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A18" s="18">
         <v>17</v>
       </c>
@@ -5032,26 +5309,36 @@
         <v>1.5</v>
       </c>
       <c r="H18" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.21739130434782608</v>
       </c>
-      <c r="I18" s="44"/>
+      <c r="I18" s="45"/>
       <c r="J18" s="22">
         <v>5</v>
       </c>
       <c r="K18" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1.0869565217391304</v>
       </c>
       <c r="L18" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="46">
+      <c r="M18" s="43">
+        <f t="shared" si="5"/>
+        <v>308.69565217391306</v>
+      </c>
+      <c r="N18" s="51">
+        <f t="shared" si="0"/>
+        <v>1543.4782608695652</v>
+      </c>
+      <c r="O18" s="50"/>
+      <c r="P18" s="51"/>
+      <c r="Q18" s="47">
         <f t="shared" si="2"/>
-        <v>308.69565217391306</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
+    <row r="19" spans="1:17" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A19" s="18">
         <v>18</v>
       </c>
@@ -5074,26 +5361,36 @@
         <v>3.6</v>
       </c>
       <c r="H19" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.52173913043478259</v>
       </c>
-      <c r="I19" s="44"/>
+      <c r="I19" s="45"/>
       <c r="J19" s="22">
         <v>5</v>
       </c>
       <c r="K19" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>2.6086956521739131</v>
       </c>
       <c r="L19" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="46">
+      <c r="M19" s="43">
+        <f t="shared" si="5"/>
+        <v>740.86956521739125</v>
+      </c>
+      <c r="N19" s="51">
+        <f t="shared" si="0"/>
+        <v>3704.347826086956</v>
+      </c>
+      <c r="O19" s="50"/>
+      <c r="P19" s="51"/>
+      <c r="Q19" s="47">
         <f t="shared" si="2"/>
-        <v>740.86956521739125</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="24" customFormat="1" ht="18.95" customHeight="1">
+    <row r="20" spans="1:17" s="24" customFormat="1" ht="18.95" customHeight="1">
       <c r="A20" s="18">
         <v>19</v>
       </c>
@@ -5116,26 +5413,36 @@
         <v>6.5</v>
       </c>
       <c r="H20" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.94202898550724634</v>
       </c>
-      <c r="I20" s="45"/>
+      <c r="I20" s="46"/>
       <c r="J20" s="22">
         <v>3</v>
       </c>
       <c r="K20" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>2.8260869565217392</v>
       </c>
       <c r="L20" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M20" s="46">
+      <c r="M20" s="43">
+        <f t="shared" si="5"/>
+        <v>1337.6811594202898</v>
+      </c>
+      <c r="N20" s="51">
+        <f t="shared" si="0"/>
+        <v>4013.0434782608691</v>
+      </c>
+      <c r="O20" s="50"/>
+      <c r="P20" s="51"/>
+      <c r="Q20" s="47">
         <f t="shared" si="2"/>
-        <v>1337.6811594202898</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="24" customFormat="1" ht="66.95" customHeight="1">
+    <row r="21" spans="1:17" s="24" customFormat="1" ht="66.95" customHeight="1">
       <c r="A21" s="18">
         <v>20</v>
       </c>
@@ -5158,7 +5465,7 @@
         <v>24</v>
       </c>
       <c r="H21" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>3.4782608695652173</v>
       </c>
       <c r="I21" s="19"/>
@@ -5166,18 +5473,28 @@
         <v>2</v>
       </c>
       <c r="K21" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6.9565217391304346</v>
       </c>
       <c r="L21" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M21" s="46">
+      <c r="M21" s="43">
+        <f t="shared" si="5"/>
+        <v>4939.130434782609</v>
+      </c>
+      <c r="N21" s="51">
+        <f t="shared" si="0"/>
+        <v>9878.2608695652179</v>
+      </c>
+      <c r="O21" s="50"/>
+      <c r="P21" s="51"/>
+      <c r="Q21" s="47">
         <f t="shared" si="2"/>
-        <v>4939.130434782609</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:13" s="24" customFormat="1" ht="56.1" customHeight="1">
+    <row r="22" spans="1:17" s="24" customFormat="1" ht="56.1" customHeight="1">
       <c r="A22" s="18">
         <v>21</v>
       </c>
@@ -5200,7 +5517,7 @@
         <v>20</v>
       </c>
       <c r="H22" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>2.8985507246376812</v>
       </c>
       <c r="I22" s="19"/>
@@ -5208,18 +5525,28 @@
         <v>3</v>
       </c>
       <c r="K22" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>8.695652173913043</v>
       </c>
       <c r="L22" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M22" s="46">
+      <c r="M22" s="43">
+        <f t="shared" si="5"/>
+        <v>4115.942028985507</v>
+      </c>
+      <c r="N22" s="51">
+        <f t="shared" si="0"/>
+        <v>12347.82608695652</v>
+      </c>
+      <c r="O22" s="50"/>
+      <c r="P22" s="51"/>
+      <c r="Q22" s="47">
         <f t="shared" si="2"/>
-        <v>4115.942028985507</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
+    <row r="23" spans="1:17" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A23" s="18">
         <v>22</v>
       </c>
@@ -5242,7 +5569,7 @@
         <v>80</v>
       </c>
       <c r="H23" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>11.594202898550725</v>
       </c>
       <c r="I23" s="19"/>
@@ -5250,18 +5577,28 @@
         <v>1</v>
       </c>
       <c r="K23" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>11.594202898550725</v>
       </c>
       <c r="L23" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M23" s="46">
+      <c r="M23" s="43">
+        <f>1420*H23</f>
+        <v>16463.768115942028</v>
+      </c>
+      <c r="N23" s="51">
+        <f>M23*J23</f>
+        <v>16463.768115942028</v>
+      </c>
+      <c r="O23" s="50"/>
+      <c r="P23" s="51"/>
+      <c r="Q23" s="47">
         <f t="shared" si="2"/>
-        <v>16463.768115942028</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+    <row r="24" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A24" s="18">
         <v>23</v>
       </c>
@@ -5284,7 +5621,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="H24" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.15942028985507248</v>
       </c>
       <c r="I24" s="19"/>
@@ -5292,18 +5629,28 @@
         <v>2</v>
       </c>
       <c r="K24" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>0.31884057971014496</v>
       </c>
       <c r="L24" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M24" s="46">
+      <c r="M24" s="43">
+        <f t="shared" si="5"/>
+        <v>226.37681159420291</v>
+      </c>
+      <c r="N24" s="51">
+        <f t="shared" si="0"/>
+        <v>452.75362318840581</v>
+      </c>
+      <c r="O24" s="50"/>
+      <c r="P24" s="51"/>
+      <c r="Q24" s="47">
         <f t="shared" si="2"/>
-        <v>226.37681159420291</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="25" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A25" s="18">
         <v>24</v>
       </c>
@@ -5326,7 +5673,7 @@
         <v>14.3</v>
       </c>
       <c r="H25" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>2.0724637681159419</v>
       </c>
       <c r="I25" s="19"/>
@@ -5334,18 +5681,34 @@
         <v>6</v>
       </c>
       <c r="K25" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>12.434782608695652</v>
       </c>
       <c r="L25" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M25" s="46">
+      <c r="M25" s="43">
+        <f t="shared" si="5"/>
+        <v>2942.8985507246375</v>
+      </c>
+      <c r="N25" s="51">
+        <f t="shared" si="0"/>
+        <v>17657.391304347824</v>
+      </c>
+      <c r="O25" s="50">
+        <f>(9000*J25)</f>
+        <v>54000</v>
+      </c>
+      <c r="P25" s="51">
+        <f t="shared" si="1"/>
+        <v>36342.608695652176</v>
+      </c>
+      <c r="Q25" s="47">
         <f t="shared" si="2"/>
-        <v>2942.8985507246375</v>
+        <v>6057.1014492753629</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
+    <row r="26" spans="1:17" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
       <c r="A26" s="18">
         <v>25</v>
       </c>
@@ -5368,7 +5731,7 @@
         <v>2</v>
       </c>
       <c r="H26" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.28985507246376813</v>
       </c>
       <c r="I26" s="19"/>
@@ -5376,18 +5739,34 @@
         <v>30</v>
       </c>
       <c r="K26" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>8.695652173913043</v>
       </c>
       <c r="L26" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="M26" s="46">
+      <c r="M26" s="43">
+        <f t="shared" si="5"/>
+        <v>411.59420289855075</v>
+      </c>
+      <c r="N26" s="51">
+        <f t="shared" si="0"/>
+        <v>12347.826086956522</v>
+      </c>
+      <c r="O26" s="50">
+        <f>(1500*J26)</f>
+        <v>45000</v>
+      </c>
+      <c r="P26" s="51">
+        <f t="shared" si="1"/>
+        <v>32652.17391304348</v>
+      </c>
+      <c r="Q26" s="47">
         <f t="shared" si="2"/>
-        <v>411.59420289855075</v>
+        <v>1088.4057971014493</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="24" customFormat="1" ht="66" customHeight="1">
+    <row r="27" spans="1:17" s="24" customFormat="1" ht="66" customHeight="1">
       <c r="A27" s="18">
         <v>26</v>
       </c>
@@ -5410,7 +5789,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="H27" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.31884057971014496</v>
       </c>
       <c r="I27" s="19"/>
@@ -5418,18 +5797,34 @@
         <v>20</v>
       </c>
       <c r="K27" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6.3768115942028993</v>
       </c>
       <c r="L27" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M27" s="46">
+      <c r="M27" s="43">
+        <f t="shared" si="5"/>
+        <v>452.75362318840581</v>
+      </c>
+      <c r="N27" s="51">
+        <f t="shared" si="0"/>
+        <v>9055.072463768116</v>
+      </c>
+      <c r="O27" s="50">
+        <f>(2000*J27)</f>
+        <v>40000</v>
+      </c>
+      <c r="P27" s="51">
+        <f t="shared" si="1"/>
+        <v>30944.927536231884</v>
+      </c>
+      <c r="Q27" s="47">
         <f t="shared" si="2"/>
-        <v>452.75362318840581</v>
+        <v>1547.2463768115942</v>
       </c>
     </row>
-    <row r="28" spans="1:13" s="24" customFormat="1" ht="68.099999999999994" customHeight="1">
+    <row r="28" spans="1:17" s="24" customFormat="1" ht="68.099999999999994" customHeight="1">
       <c r="A28" s="18"/>
       <c r="B28" s="19" t="s">
         <v>94</v>
@@ -5450,7 +5845,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="H28" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.31884057971014496</v>
       </c>
       <c r="I28" s="19"/>
@@ -5458,18 +5853,25 @@
         <v>15</v>
       </c>
       <c r="K28" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4.7826086956521747</v>
       </c>
       <c r="L28" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M28" s="46">
+      <c r="M28" s="43">
+        <f t="shared" si="5"/>
+        <v>452.75362318840581</v>
+      </c>
+      <c r="N28" s="51"/>
+      <c r="O28" s="50"/>
+      <c r="P28" s="51"/>
+      <c r="Q28" s="47">
         <f t="shared" si="2"/>
-        <v>452.75362318840581</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
+    <row r="29" spans="1:17" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A29" s="18">
         <v>28</v>
       </c>
@@ -5492,7 +5894,7 @@
         <v>1.32</v>
       </c>
       <c r="H29" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.19130434782608696</v>
       </c>
       <c r="I29" s="19"/>
@@ -5500,18 +5902,34 @@
         <v>10</v>
       </c>
       <c r="K29" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1.9130434782608696</v>
       </c>
       <c r="L29" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M29" s="46">
+      <c r="M29" s="43">
+        <f t="shared" si="5"/>
+        <v>271.6521739130435</v>
+      </c>
+      <c r="N29" s="51">
+        <f t="shared" si="0"/>
+        <v>2716.521739130435</v>
+      </c>
+      <c r="O29" s="50">
+        <f>(1500*J29)</f>
+        <v>15000</v>
+      </c>
+      <c r="P29" s="51">
+        <f t="shared" si="1"/>
+        <v>12283.478260869564</v>
+      </c>
+      <c r="Q29" s="47">
         <f t="shared" si="2"/>
-        <v>271.6521739130435</v>
+        <v>1228.3478260869565</v>
       </c>
     </row>
-    <row r="30" spans="1:13" s="24" customFormat="1" ht="72" customHeight="1">
+    <row r="30" spans="1:17" s="24" customFormat="1" ht="72" customHeight="1">
       <c r="A30" s="18">
         <v>29</v>
       </c>
@@ -5534,7 +5952,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="H30" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.31884057971014496</v>
       </c>
       <c r="I30" s="19"/>
@@ -5542,18 +5960,34 @@
         <v>6</v>
       </c>
       <c r="K30" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1.9130434782608696</v>
       </c>
       <c r="L30" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M30" s="46">
+      <c r="M30" s="43">
+        <f t="shared" si="5"/>
+        <v>452.75362318840581</v>
+      </c>
+      <c r="N30" s="51">
+        <f t="shared" si="0"/>
+        <v>2716.521739130435</v>
+      </c>
+      <c r="O30" s="50">
+        <f>(2500*J30)</f>
+        <v>15000</v>
+      </c>
+      <c r="P30" s="51">
+        <f t="shared" si="1"/>
+        <v>12283.478260869564</v>
+      </c>
+      <c r="Q30" s="47">
         <f t="shared" si="2"/>
-        <v>452.75362318840581</v>
+        <v>2047.246376811594</v>
       </c>
     </row>
-    <row r="31" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="31" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A31" s="18">
         <v>30</v>
       </c>
@@ -5576,7 +6010,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="H31" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.31884057971014496</v>
       </c>
       <c r="I31" s="19"/>
@@ -5584,18 +6018,34 @@
         <v>7</v>
       </c>
       <c r="K31" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>2.2318840579710146</v>
       </c>
       <c r="L31" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M31" s="46">
-        <f t="shared" si="2"/>
+      <c r="M31" s="43">
+        <f t="shared" si="5"/>
         <v>452.75362318840581</v>
       </c>
+      <c r="N31" s="51">
+        <f t="shared" si="0"/>
+        <v>3169.2753623188405</v>
+      </c>
+      <c r="O31" s="50">
+        <f>(3000*J31)</f>
+        <v>21000</v>
+      </c>
+      <c r="P31" s="51">
+        <f>O31-N31</f>
+        <v>17830.72463768116</v>
+      </c>
+      <c r="Q31" s="47">
+        <f>P31/J31</f>
+        <v>2547.2463768115945</v>
+      </c>
     </row>
-    <row r="32" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+    <row r="32" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A32" s="18">
         <v>32</v>
       </c>
@@ -5618,7 +6068,7 @@
         <v>1.32</v>
       </c>
       <c r="H32" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.19130434782608696</v>
       </c>
       <c r="I32" s="19"/>
@@ -5626,18 +6076,34 @@
         <v>25</v>
       </c>
       <c r="K32" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>4.7826086956521738</v>
       </c>
       <c r="L32" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M32" s="46">
+      <c r="M32" s="43">
+        <f t="shared" si="5"/>
+        <v>271.6521739130435</v>
+      </c>
+      <c r="N32" s="51">
+        <f t="shared" si="0"/>
+        <v>6791.3043478260879</v>
+      </c>
+      <c r="O32" s="50">
+        <f>(3000*J32)</f>
+        <v>75000</v>
+      </c>
+      <c r="P32" s="51">
+        <f t="shared" si="1"/>
+        <v>68208.695652173919</v>
+      </c>
+      <c r="Q32" s="47">
         <f t="shared" si="2"/>
-        <v>271.6521739130435</v>
+        <v>2728.347826086957</v>
       </c>
     </row>
-    <row r="33" spans="1:13" s="24" customFormat="1" ht="69.95" customHeight="1">
+    <row r="33" spans="1:17" s="24" customFormat="1" ht="69.95" customHeight="1">
       <c r="A33" s="18">
         <v>32</v>
       </c>
@@ -5660,7 +6126,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="H33" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.15942028985507248</v>
       </c>
       <c r="I33" s="19"/>
@@ -5668,18 +6134,34 @@
         <v>25</v>
       </c>
       <c r="K33" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>3.985507246376812</v>
       </c>
       <c r="L33" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M33" s="46">
+      <c r="M33" s="43">
+        <f t="shared" si="5"/>
+        <v>226.37681159420291</v>
+      </c>
+      <c r="N33" s="51">
+        <f t="shared" si="0"/>
+        <v>5659.420289855073</v>
+      </c>
+      <c r="O33" s="50">
+        <f>(3000*J33)</f>
+        <v>75000</v>
+      </c>
+      <c r="P33" s="51">
+        <f t="shared" si="1"/>
+        <v>69340.579710144928</v>
+      </c>
+      <c r="Q33" s="47">
         <f t="shared" si="2"/>
-        <v>226.37681159420291</v>
+        <v>2773.623188405797</v>
       </c>
     </row>
-    <row r="34" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="34" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A34" s="18">
         <v>34</v>
       </c>
@@ -5702,7 +6184,7 @@
         <v>0.22</v>
       </c>
       <c r="H34" s="21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I34" s="19"/>
@@ -5710,18 +6192,34 @@
         <v>50</v>
       </c>
       <c r="K34" s="23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>1.5942028985507246</v>
       </c>
       <c r="L34" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M34" s="46">
+      <c r="M34" s="43">
+        <f t="shared" si="5"/>
+        <v>45.275362318840578</v>
+      </c>
+      <c r="N34" s="51">
+        <f t="shared" si="0"/>
+        <v>2263.768115942029</v>
+      </c>
+      <c r="O34" s="50">
+        <f>(749*J34)</f>
+        <v>37450</v>
+      </c>
+      <c r="P34" s="51">
+        <f t="shared" si="1"/>
+        <v>35186.231884057968</v>
+      </c>
+      <c r="Q34" s="47">
         <f t="shared" si="2"/>
-        <v>45.275362318840578</v>
+        <v>703.72463768115938</v>
       </c>
     </row>
-    <row r="35" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="35" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A35" s="18">
         <v>35</v>
       </c>
@@ -5744,7 +6242,7 @@
         <v>1.97</v>
       </c>
       <c r="H35" s="21">
-        <f t="shared" ref="H35:H69" si="3">G35/6.9</f>
+        <f t="shared" ref="H35:H69" si="7">G35/6.9</f>
         <v>0.28550724637681157</v>
       </c>
       <c r="I35" s="19"/>
@@ -5752,18 +6250,34 @@
         <v>40</v>
       </c>
       <c r="K35" s="23">
-        <f t="shared" ref="K35:K69" si="4">J35*H35</f>
+        <f t="shared" ref="K35:K69" si="8">J35*H35</f>
         <v>11.420289855072463</v>
       </c>
       <c r="L35" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="M35" s="46">
+      <c r="M35" s="43">
+        <f t="shared" si="5"/>
+        <v>405.42028985507244</v>
+      </c>
+      <c r="N35" s="51">
+        <f t="shared" si="0"/>
+        <v>16216.811594202898</v>
+      </c>
+      <c r="O35" s="50">
+        <f>(2500*J35)</f>
+        <v>100000</v>
+      </c>
+      <c r="P35" s="51">
+        <f t="shared" si="1"/>
+        <v>83783.188405797104</v>
+      </c>
+      <c r="Q35" s="47">
         <f t="shared" si="2"/>
-        <v>405.42028985507244</v>
+        <v>2094.5797101449275</v>
       </c>
     </row>
-    <row r="36" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="36" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A36" s="18">
         <v>36</v>
       </c>
@@ -5786,7 +6300,7 @@
         <v>12</v>
       </c>
       <c r="H36" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>1.7391304347826086</v>
       </c>
       <c r="I36" s="19"/>
@@ -5794,18 +6308,34 @@
         <v>10</v>
       </c>
       <c r="K36" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>17.391304347826086</v>
       </c>
       <c r="L36" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="M36" s="46">
+      <c r="M36" s="43">
+        <f t="shared" si="5"/>
+        <v>2469.5652173913045</v>
+      </c>
+      <c r="N36" s="51">
+        <f t="shared" si="0"/>
+        <v>24695.652173913044</v>
+      </c>
+      <c r="O36" s="50">
+        <f>(10000*J36)</f>
+        <v>100000</v>
+      </c>
+      <c r="P36" s="51">
+        <f t="shared" si="1"/>
+        <v>75304.34782608696</v>
+      </c>
+      <c r="Q36" s="47">
         <f t="shared" si="2"/>
-        <v>2469.5652173913045</v>
+        <v>7530.434782608696</v>
       </c>
     </row>
-    <row r="37" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="37" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A37" s="18">
         <v>37</v>
       </c>
@@ -5828,7 +6358,7 @@
         <v>3</v>
       </c>
       <c r="H37" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.43478260869565216</v>
       </c>
       <c r="I37" s="19"/>
@@ -5836,18 +6366,34 @@
         <v>20</v>
       </c>
       <c r="K37" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>8.695652173913043</v>
       </c>
       <c r="L37" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="M37" s="46">
+      <c r="M37" s="43">
+        <f t="shared" si="5"/>
+        <v>617.39130434782612</v>
+      </c>
+      <c r="N37" s="51">
+        <f t="shared" si="0"/>
+        <v>12347.826086956522</v>
+      </c>
+      <c r="O37" s="50">
+        <f>(4500*J37)</f>
+        <v>90000</v>
+      </c>
+      <c r="P37" s="51">
+        <f t="shared" si="1"/>
+        <v>77652.173913043473</v>
+      </c>
+      <c r="Q37" s="47">
         <f t="shared" si="2"/>
-        <v>617.39130434782612</v>
+        <v>3882.6086956521735</v>
       </c>
     </row>
-    <row r="38" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="38" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A38" s="25">
         <v>38</v>
       </c>
@@ -5870,7 +6416,7 @@
         <v>28.6</v>
       </c>
       <c r="H38" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>4.1449275362318838</v>
       </c>
       <c r="I38" s="19"/>
@@ -5878,18 +6424,34 @@
         <v>2</v>
       </c>
       <c r="K38" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>8.2898550724637676</v>
       </c>
       <c r="L38" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="M38" s="46">
+      <c r="M38" s="43">
+        <f t="shared" si="5"/>
+        <v>5885.797101449275</v>
+      </c>
+      <c r="N38" s="51">
+        <f t="shared" si="0"/>
+        <v>11771.59420289855</v>
+      </c>
+      <c r="O38" s="50">
+        <f>(10000*J38)</f>
+        <v>20000</v>
+      </c>
+      <c r="P38" s="51">
+        <f t="shared" si="1"/>
+        <v>8228.4057971014499</v>
+      </c>
+      <c r="Q38" s="47">
         <f t="shared" si="2"/>
-        <v>5885.797101449275</v>
+        <v>4114.202898550725</v>
       </c>
     </row>
-    <row r="39" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
+    <row r="39" spans="1:17" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A39" s="18">
         <v>39</v>
       </c>
@@ -5912,7 +6474,7 @@
         <v>2.86</v>
       </c>
       <c r="H39" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.41449275362318838</v>
       </c>
       <c r="I39" s="19"/>
@@ -5920,18 +6482,34 @@
         <v>12</v>
       </c>
       <c r="K39" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>4.9739130434782606</v>
       </c>
       <c r="L39" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="M39" s="46">
+      <c r="M39" s="43">
+        <f t="shared" si="5"/>
+        <v>588.5797101449275</v>
+      </c>
+      <c r="N39" s="51">
+        <f t="shared" si="0"/>
+        <v>7062.95652173913</v>
+      </c>
+      <c r="O39" s="50">
+        <f>(4000*J39)</f>
+        <v>48000</v>
+      </c>
+      <c r="P39" s="51">
+        <f t="shared" si="1"/>
+        <v>40937.043478260872</v>
+      </c>
+      <c r="Q39" s="47">
         <f t="shared" si="2"/>
-        <v>588.5797101449275</v>
+        <v>3411.4202898550725</v>
       </c>
     </row>
-    <row r="40" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
+    <row r="40" spans="1:17" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A40" s="18">
         <v>40</v>
       </c>
@@ -5954,7 +6532,7 @@
         <v>4.84</v>
       </c>
       <c r="H40" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.70144927536231882</v>
       </c>
       <c r="I40" s="19"/>
@@ -5962,18 +6540,34 @@
         <v>10</v>
       </c>
       <c r="K40" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>7.0144927536231885</v>
       </c>
       <c r="L40" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="M40" s="46">
+      <c r="M40" s="43">
+        <f t="shared" si="5"/>
+        <v>996.05797101449275</v>
+      </c>
+      <c r="N40" s="51">
+        <f t="shared" si="0"/>
+        <v>9960.579710144928</v>
+      </c>
+      <c r="O40" s="50">
+        <f>(5000*J40)</f>
+        <v>50000</v>
+      </c>
+      <c r="P40" s="51">
+        <f t="shared" si="1"/>
+        <v>40039.420289855072</v>
+      </c>
+      <c r="Q40" s="47">
         <f t="shared" si="2"/>
-        <v>996.05797101449275</v>
+        <v>4003.942028985507</v>
       </c>
     </row>
-    <row r="41" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
+    <row r="41" spans="1:17" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A41" s="18">
         <v>41</v>
       </c>
@@ -5996,7 +6590,7 @@
         <v>3.3</v>
       </c>
       <c r="H41" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.47826086956521735</v>
       </c>
       <c r="I41" s="19"/>
@@ -6004,18 +6598,34 @@
         <v>10</v>
       </c>
       <c r="K41" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>4.7826086956521738</v>
       </c>
-      <c r="L41" s="18" t="s">
+      <c r="L41" s="48" t="s">
         <v>134</v>
       </c>
-      <c r="M41" s="46">
+      <c r="M41" s="50">
+        <f t="shared" si="5"/>
+        <v>679.13043478260863</v>
+      </c>
+      <c r="N41" s="51">
+        <f t="shared" si="0"/>
+        <v>6791.3043478260861</v>
+      </c>
+      <c r="O41" s="50">
+        <f>(4000*J41)</f>
+        <v>40000</v>
+      </c>
+      <c r="P41" s="51">
+        <f t="shared" si="1"/>
+        <v>33208.695652173912</v>
+      </c>
+      <c r="Q41" s="47">
         <f t="shared" si="2"/>
-        <v>679.13043478260863</v>
+        <v>3320.869565217391</v>
       </c>
     </row>
-    <row r="42" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
+    <row r="42" spans="1:17" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A42" s="18">
         <v>42</v>
       </c>
@@ -6038,7 +6648,7 @@
         <v>1.43</v>
       </c>
       <c r="H42" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.20724637681159419</v>
       </c>
       <c r="I42" s="19"/>
@@ -6046,18 +6656,34 @@
         <v>20</v>
       </c>
       <c r="K42" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>4.1449275362318838</v>
       </c>
-      <c r="L42" s="18" t="s">
+      <c r="L42" s="48" t="s">
         <v>138</v>
       </c>
-      <c r="M42" s="46">
+      <c r="M42" s="50">
+        <f t="shared" si="5"/>
+        <v>294.28985507246375</v>
+      </c>
+      <c r="N42" s="51">
+        <f t="shared" si="0"/>
+        <v>5885.797101449275</v>
+      </c>
+      <c r="O42" s="50">
+        <f>(3500*J42)</f>
+        <v>70000</v>
+      </c>
+      <c r="P42" s="51">
+        <f t="shared" si="1"/>
+        <v>64114.202898550728</v>
+      </c>
+      <c r="Q42" s="47">
         <f t="shared" si="2"/>
-        <v>294.28985507246375</v>
+        <v>3205.7101449275365</v>
       </c>
     </row>
-    <row r="43" spans="1:13" s="24" customFormat="1" ht="84.95" customHeight="1">
+    <row r="43" spans="1:17" s="24" customFormat="1" ht="84.95" customHeight="1">
       <c r="A43" s="18">
         <v>43</v>
       </c>
@@ -6080,7 +6706,7 @@
         <v>0.22</v>
       </c>
       <c r="H43" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I43" s="19"/>
@@ -6088,18 +6714,34 @@
         <v>40</v>
       </c>
       <c r="K43" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>1.2753623188405796</v>
       </c>
-      <c r="L43" s="18" t="s">
+      <c r="L43" s="48" t="s">
         <v>134</v>
       </c>
-      <c r="M43" s="46">
+      <c r="M43" s="50">
+        <f t="shared" si="5"/>
+        <v>45.275362318840578</v>
+      </c>
+      <c r="N43" s="51">
+        <f t="shared" si="0"/>
+        <v>1811.014492753623</v>
+      </c>
+      <c r="O43" s="50">
+        <f>(240*J43)</f>
+        <v>9600</v>
+      </c>
+      <c r="P43" s="51">
+        <f t="shared" si="1"/>
+        <v>7788.985507246377</v>
+      </c>
+      <c r="Q43" s="47">
         <f t="shared" si="2"/>
-        <v>45.275362318840578</v>
+        <v>194.72463768115944</v>
       </c>
     </row>
-    <row r="44" spans="1:13" s="24" customFormat="1" ht="83.1" customHeight="1">
+    <row r="44" spans="1:17" s="24" customFormat="1" ht="83.1" customHeight="1">
       <c r="A44" s="18">
         <v>44</v>
       </c>
@@ -6122,7 +6764,7 @@
         <v>210</v>
       </c>
       <c r="H44" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>30.434782608695652</v>
       </c>
       <c r="I44" s="19"/>
@@ -6130,18 +6772,34 @@
         <v>1</v>
       </c>
       <c r="K44" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>30.434782608695652</v>
       </c>
-      <c r="L44" s="18" t="s">
+      <c r="L44" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="M44" s="46">
+      <c r="M44" s="50">
+        <f t="shared" si="5"/>
+        <v>43217.391304347824</v>
+      </c>
+      <c r="N44" s="51">
+        <f t="shared" si="0"/>
+        <v>43217.391304347824</v>
+      </c>
+      <c r="O44" s="50">
+        <f t="shared" si="6"/>
+        <v>20000</v>
+      </c>
+      <c r="P44" s="51">
+        <f t="shared" si="1"/>
+        <v>-23217.391304347824</v>
+      </c>
+      <c r="Q44" s="47">
         <f t="shared" si="2"/>
-        <v>43217.391304347824</v>
+        <v>-23217.391304347824</v>
       </c>
     </row>
-    <row r="45" spans="1:13" s="24" customFormat="1" ht="78" customHeight="1">
+    <row r="45" spans="1:17" s="24" customFormat="1" ht="78" customHeight="1">
       <c r="A45" s="18">
         <v>45</v>
       </c>
@@ -6164,7 +6822,7 @@
         <v>7.26</v>
       </c>
       <c r="H45" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>1.0521739130434782</v>
       </c>
       <c r="I45" s="19"/>
@@ -6172,16 +6830,32 @@
         <v>3</v>
       </c>
       <c r="K45" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>3.1565217391304348</v>
       </c>
       <c r="L45" s="29"/>
-      <c r="M45" s="46">
+      <c r="M45" s="50">
+        <f t="shared" si="5"/>
+        <v>1494.086956521739</v>
+      </c>
+      <c r="N45" s="51">
+        <f t="shared" si="0"/>
+        <v>4482.260869565217</v>
+      </c>
+      <c r="O45" s="50">
+        <f>(4500*J45)</f>
+        <v>13500</v>
+      </c>
+      <c r="P45" s="51">
+        <f t="shared" si="1"/>
+        <v>9017.7391304347839</v>
+      </c>
+      <c r="Q45" s="47">
         <f t="shared" si="2"/>
-        <v>1494.086956521739</v>
+        <v>3005.9130434782614</v>
       </c>
     </row>
-    <row r="46" spans="1:13" s="24" customFormat="1" ht="78" customHeight="1">
+    <row r="46" spans="1:17" s="24" customFormat="1" ht="78" customHeight="1">
       <c r="A46" s="18">
         <v>46</v>
       </c>
@@ -6204,7 +6878,7 @@
         <v>7.26</v>
       </c>
       <c r="H46" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>1.0521739130434782</v>
       </c>
       <c r="I46" s="19"/>
@@ -6212,18 +6886,34 @@
         <v>3</v>
       </c>
       <c r="K46" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>3.1565217391304348</v>
       </c>
-      <c r="L46" s="18" t="s">
+      <c r="L46" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="M46" s="46">
+      <c r="M46" s="50">
+        <f t="shared" si="5"/>
+        <v>1494.086956521739</v>
+      </c>
+      <c r="N46" s="51">
+        <f t="shared" si="0"/>
+        <v>4482.260869565217</v>
+      </c>
+      <c r="O46" s="50">
+        <f>(4500*J46)</f>
+        <v>13500</v>
+      </c>
+      <c r="P46" s="51">
+        <f t="shared" si="1"/>
+        <v>9017.7391304347839</v>
+      </c>
+      <c r="Q46" s="47">
         <f t="shared" si="2"/>
-        <v>1494.086956521739</v>
+        <v>3005.9130434782614</v>
       </c>
     </row>
-    <row r="47" spans="1:13" s="24" customFormat="1" ht="62.1" customHeight="1">
+    <row r="47" spans="1:17" s="24" customFormat="1" ht="62.1" customHeight="1">
       <c r="A47" s="18">
         <v>47</v>
       </c>
@@ -6246,7 +6936,7 @@
         <v>0.22</v>
       </c>
       <c r="H47" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I47" s="19"/>
@@ -6254,18 +6944,34 @@
         <v>30</v>
       </c>
       <c r="K47" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="L47" s="18" t="s">
+      <c r="L47" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M47" s="46">
+      <c r="M47" s="50">
+        <f t="shared" si="5"/>
+        <v>45.275362318840578</v>
+      </c>
+      <c r="N47" s="51">
+        <f t="shared" si="0"/>
+        <v>1358.2608695652173</v>
+      </c>
+      <c r="O47" s="50">
+        <f>(150*J47)</f>
+        <v>4500</v>
+      </c>
+      <c r="P47" s="51">
+        <f t="shared" si="1"/>
+        <v>3141.739130434783</v>
+      </c>
+      <c r="Q47" s="47">
         <f t="shared" si="2"/>
-        <v>45.275362318840578</v>
+        <v>104.72463768115944</v>
       </c>
     </row>
-    <row r="48" spans="1:13" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
+    <row r="48" spans="1:17" s="24" customFormat="1" ht="71.099999999999994" customHeight="1">
       <c r="A48" s="18">
         <v>48</v>
       </c>
@@ -6288,7 +6994,7 @@
         <v>0.22</v>
       </c>
       <c r="H48" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>3.1884057971014491E-2</v>
       </c>
       <c r="I48" s="19"/>
@@ -6296,18 +7002,34 @@
         <v>30</v>
       </c>
       <c r="K48" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="L48" s="18" t="s">
+      <c r="L48" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M48" s="46">
+      <c r="M48" s="50">
+        <f t="shared" si="5"/>
+        <v>45.275362318840578</v>
+      </c>
+      <c r="N48" s="51">
+        <f t="shared" si="0"/>
+        <v>1358.2608695652173</v>
+      </c>
+      <c r="O48" s="50">
+        <f>(240*J48)</f>
+        <v>7200</v>
+      </c>
+      <c r="P48" s="51">
+        <f t="shared" si="1"/>
+        <v>5841.739130434783</v>
+      </c>
+      <c r="Q48" s="47">
         <f t="shared" si="2"/>
-        <v>45.275362318840578</v>
+        <v>194.72463768115944</v>
       </c>
     </row>
-    <row r="49" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="49" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A49" s="18">
         <v>49</v>
       </c>
@@ -6330,26 +7052,42 @@
         <v>0.09</v>
       </c>
       <c r="H49" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>1.3043478260869565E-2</v>
       </c>
-      <c r="I49" s="43"/>
+      <c r="I49" s="44"/>
       <c r="J49" s="22">
         <v>50</v>
       </c>
       <c r="K49" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0.65217391304347827</v>
       </c>
-      <c r="L49" s="18" t="s">
+      <c r="L49" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M49" s="46">
+      <c r="M49" s="50">
+        <f t="shared" si="5"/>
+        <v>18.521739130434781</v>
+      </c>
+      <c r="N49" s="51">
+        <f t="shared" si="0"/>
+        <v>926.08695652173901</v>
+      </c>
+      <c r="O49" s="50">
+        <f>(100*J49)</f>
+        <v>5000</v>
+      </c>
+      <c r="P49" s="51">
+        <f t="shared" si="1"/>
+        <v>4073.913043478261</v>
+      </c>
+      <c r="Q49" s="47">
         <f t="shared" si="2"/>
-        <v>18.521739130434781</v>
+        <v>81.478260869565219</v>
       </c>
     </row>
-    <row r="50" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="50" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A50" s="18">
         <v>50</v>
       </c>
@@ -6372,26 +7110,42 @@
         <v>0.06</v>
       </c>
       <c r="H50" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>8.6956521739130418E-3</v>
       </c>
-      <c r="I50" s="44"/>
+      <c r="I50" s="45"/>
       <c r="J50" s="22">
         <v>50</v>
       </c>
       <c r="K50" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>0.43478260869565211</v>
       </c>
-      <c r="L50" s="18" t="s">
+      <c r="L50" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M50" s="46">
+      <c r="M50" s="50">
+        <f t="shared" si="5"/>
+        <v>12.34782608695652</v>
+      </c>
+      <c r="N50" s="51">
+        <f t="shared" si="0"/>
+        <v>617.39130434782601</v>
+      </c>
+      <c r="O50" s="50">
+        <f>(150*J50)</f>
+        <v>7500</v>
+      </c>
+      <c r="P50" s="51">
+        <f t="shared" si="1"/>
+        <v>6882.608695652174</v>
+      </c>
+      <c r="Q50" s="47">
         <f t="shared" si="2"/>
-        <v>12.34782608695652</v>
+        <v>137.65217391304347</v>
       </c>
     </row>
-    <row r="51" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="51" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A51" s="18">
         <v>51</v>
       </c>
@@ -6414,26 +7168,42 @@
         <v>0.2</v>
       </c>
       <c r="H51" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>2.8985507246376812E-2</v>
       </c>
-      <c r="I51" s="45"/>
+      <c r="I51" s="46"/>
       <c r="J51" s="22">
         <v>50</v>
       </c>
       <c r="K51" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>1.4492753623188406</v>
       </c>
-      <c r="L51" s="18" t="s">
+      <c r="L51" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M51" s="46">
+      <c r="M51" s="50">
+        <f t="shared" si="5"/>
+        <v>41.159420289855071</v>
+      </c>
+      <c r="N51" s="51">
+        <f t="shared" si="0"/>
+        <v>2057.9710144927535</v>
+      </c>
+      <c r="O51" s="50">
+        <f>(150*J51)</f>
+        <v>7500</v>
+      </c>
+      <c r="P51" s="51">
+        <f t="shared" si="1"/>
+        <v>5442.028985507246</v>
+      </c>
+      <c r="Q51" s="47">
         <f t="shared" si="2"/>
-        <v>41.159420289855071</v>
+        <v>108.84057971014492</v>
       </c>
     </row>
-    <row r="52" spans="1:13" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
+    <row r="52" spans="1:17" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
       <c r="A52" s="18">
         <v>52</v>
       </c>
@@ -6456,26 +7226,42 @@
         <v>6.6</v>
       </c>
       <c r="H52" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="I52" s="43"/>
+      <c r="I52" s="44"/>
       <c r="J52" s="22">
         <v>10</v>
       </c>
       <c r="K52" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>9.5652173913043477</v>
       </c>
-      <c r="L52" s="18" t="s">
+      <c r="L52" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M52" s="46">
+      <c r="M52" s="50">
+        <f t="shared" si="5"/>
+        <v>1358.2608695652173</v>
+      </c>
+      <c r="N52" s="51">
+        <f>M52*J52</f>
+        <v>13582.608695652172</v>
+      </c>
+      <c r="O52" s="50">
+        <f>(5000*J52)</f>
+        <v>50000</v>
+      </c>
+      <c r="P52" s="51">
+        <f t="shared" si="1"/>
+        <v>36417.391304347824</v>
+      </c>
+      <c r="Q52" s="47">
         <f t="shared" si="2"/>
-        <v>1358.2608695652173</v>
+        <v>3641.7391304347825</v>
       </c>
     </row>
-    <row r="53" spans="1:13" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
+    <row r="53" spans="1:17" s="24" customFormat="1" ht="33.950000000000003" customHeight="1">
       <c r="A53" s="18">
         <v>53</v>
       </c>
@@ -6498,26 +7284,42 @@
         <v>9.9</v>
       </c>
       <c r="H53" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>1.4347826086956521</v>
       </c>
-      <c r="I53" s="45"/>
+      <c r="I53" s="46"/>
       <c r="J53" s="22">
         <v>5</v>
       </c>
       <c r="K53" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>7.1739130434782608</v>
       </c>
-      <c r="L53" s="18" t="s">
+      <c r="L53" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M53" s="46">
+      <c r="M53" s="50">
+        <f t="shared" si="5"/>
+        <v>2037.391304347826</v>
+      </c>
+      <c r="N53" s="51">
+        <f t="shared" si="0"/>
+        <v>10186.95652173913</v>
+      </c>
+      <c r="O53" s="50">
+        <f>(6000*J53)</f>
+        <v>30000</v>
+      </c>
+      <c r="P53" s="51">
+        <f t="shared" si="1"/>
+        <v>19813.043478260872</v>
+      </c>
+      <c r="Q53" s="47">
         <f t="shared" si="2"/>
-        <v>2037.391304347826</v>
+        <v>3962.6086956521744</v>
       </c>
     </row>
-    <row r="54" spans="1:13" s="24" customFormat="1" ht="45" customHeight="1">
+    <row r="54" spans="1:17" s="24" customFormat="1" ht="45" customHeight="1">
       <c r="A54" s="18">
         <v>54</v>
       </c>
@@ -6540,7 +7342,7 @@
         <v>14.85</v>
       </c>
       <c r="H54" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>2.152173913043478</v>
       </c>
       <c r="I54" s="19"/>
@@ -6548,18 +7350,34 @@
         <v>5</v>
       </c>
       <c r="K54" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>10.760869565217391</v>
       </c>
-      <c r="L54" s="18" t="s">
+      <c r="L54" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M54" s="46">
+      <c r="M54" s="50">
+        <f t="shared" si="5"/>
+        <v>3056.086956521739</v>
+      </c>
+      <c r="N54" s="51">
+        <f t="shared" si="0"/>
+        <v>15280.434782608696</v>
+      </c>
+      <c r="O54" s="50">
+        <f>(7000*J54)</f>
+        <v>35000</v>
+      </c>
+      <c r="P54" s="51">
+        <f t="shared" si="1"/>
+        <v>19719.565217391304</v>
+      </c>
+      <c r="Q54" s="47">
         <f t="shared" si="2"/>
-        <v>3056.086956521739</v>
+        <v>3943.913043478261</v>
       </c>
     </row>
-    <row r="55" spans="1:13" s="24" customFormat="1" ht="45" customHeight="1">
+    <row r="55" spans="1:17" s="24" customFormat="1" ht="45" customHeight="1">
       <c r="A55" s="18">
         <v>55</v>
       </c>
@@ -6582,7 +7400,7 @@
         <v>22</v>
       </c>
       <c r="H55" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>3.1884057971014492</v>
       </c>
       <c r="I55" s="19"/>
@@ -6590,18 +7408,34 @@
         <v>5</v>
       </c>
       <c r="K55" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>15.942028985507246</v>
       </c>
-      <c r="L55" s="18" t="s">
+      <c r="L55" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M55" s="46">
+      <c r="M55" s="50">
+        <f t="shared" si="5"/>
+        <v>4527.536231884058</v>
+      </c>
+      <c r="N55" s="51">
+        <f t="shared" si="0"/>
+        <v>22637.681159420288</v>
+      </c>
+      <c r="O55" s="50">
+        <f>(9000*J55)</f>
+        <v>45000</v>
+      </c>
+      <c r="P55" s="51">
+        <f t="shared" si="1"/>
+        <v>22362.318840579712</v>
+      </c>
+      <c r="Q55" s="47">
         <f t="shared" si="2"/>
-        <v>4527.536231884058</v>
+        <v>4472.463768115942</v>
       </c>
     </row>
-    <row r="56" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+    <row r="56" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A56" s="18">
         <v>56</v>
       </c>
@@ -6624,7 +7458,7 @@
         <v>0.17</v>
       </c>
       <c r="H56" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>2.4637681159420291E-2</v>
       </c>
       <c r="I56" s="19"/>
@@ -6632,18 +7466,34 @@
         <v>50</v>
       </c>
       <c r="K56" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>1.2318840579710146</v>
       </c>
-      <c r="L56" s="18" t="s">
+      <c r="L56" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M56" s="46">
+      <c r="M56" s="50">
+        <f t="shared" si="5"/>
+        <v>34.985507246376812</v>
+      </c>
+      <c r="N56" s="51">
+        <f t="shared" si="0"/>
+        <v>1749.2753623188405</v>
+      </c>
+      <c r="O56" s="50">
+        <f>(2000*J56)</f>
+        <v>100000</v>
+      </c>
+      <c r="P56" s="51">
+        <f t="shared" si="1"/>
+        <v>98250.724637681153</v>
+      </c>
+      <c r="Q56" s="47">
         <f t="shared" si="2"/>
-        <v>34.985507246376812</v>
+        <v>1965.014492753623</v>
       </c>
     </row>
-    <row r="57" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+    <row r="57" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A57" s="18">
         <v>57</v>
       </c>
@@ -6666,7 +7516,7 @@
         <v>8.8000000000000007</v>
       </c>
       <c r="H57" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>1.2753623188405798</v>
       </c>
       <c r="I57" s="19"/>
@@ -6674,18 +7524,34 @@
         <v>10</v>
       </c>
       <c r="K57" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>12.753623188405799</v>
       </c>
-      <c r="L57" s="18" t="s">
+      <c r="L57" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M57" s="46">
+      <c r="M57" s="50">
+        <f t="shared" si="5"/>
+        <v>1811.0144927536232</v>
+      </c>
+      <c r="N57" s="51">
+        <f t="shared" si="0"/>
+        <v>18110.144927536232</v>
+      </c>
+      <c r="O57" s="50">
+        <f>(6000*J57)</f>
+        <v>60000</v>
+      </c>
+      <c r="P57" s="51">
+        <f t="shared" si="1"/>
+        <v>41889.855072463768</v>
+      </c>
+      <c r="Q57" s="47">
         <f t="shared" si="2"/>
-        <v>1811.0144927536232</v>
+        <v>4188.985507246377</v>
       </c>
     </row>
-    <row r="58" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="58" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A58" s="30"/>
       <c r="B58" s="19" t="s">
         <v>179</v>
@@ -6706,7 +7572,7 @@
         <v>0.44</v>
       </c>
       <c r="H58" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>6.3768115942028983E-2</v>
       </c>
       <c r="I58" s="19"/>
@@ -6714,18 +7580,34 @@
         <v>50</v>
       </c>
       <c r="K58" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>3.1884057971014492</v>
       </c>
-      <c r="L58" s="18" t="s">
+      <c r="L58" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M58" s="46">
+      <c r="M58" s="50">
+        <f t="shared" si="5"/>
+        <v>90.550724637681157</v>
+      </c>
+      <c r="N58" s="51">
+        <f>M58*J58</f>
+        <v>4527.536231884058</v>
+      </c>
+      <c r="O58" s="50">
+        <f>(250*J58)</f>
+        <v>12500</v>
+      </c>
+      <c r="P58" s="51">
+        <f t="shared" si="1"/>
+        <v>7972.463768115942</v>
+      </c>
+      <c r="Q58" s="47">
         <f t="shared" si="2"/>
-        <v>90.550724637681157</v>
+        <v>159.44927536231884</v>
       </c>
     </row>
-    <row r="59" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="59" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A59" s="30"/>
       <c r="B59" s="19" t="s">
         <v>181</v>
@@ -6750,18 +7632,34 @@
         <v>10</v>
       </c>
       <c r="K59" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>2.043478260869565</v>
       </c>
-      <c r="L59" s="18" t="s">
+      <c r="L59" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M59" s="46">
+      <c r="M59" s="50">
+        <f t="shared" si="5"/>
+        <v>290.17391304347825</v>
+      </c>
+      <c r="N59" s="51">
+        <f t="shared" si="0"/>
+        <v>2901.7391304347825</v>
+      </c>
+      <c r="O59" s="50">
+        <f>(750*J59)</f>
+        <v>7500</v>
+      </c>
+      <c r="P59" s="51">
+        <f t="shared" si="1"/>
+        <v>4598.2608695652179</v>
+      </c>
+      <c r="Q59" s="47">
         <f t="shared" si="2"/>
-        <v>290.17391304347825</v>
+        <v>459.82608695652181</v>
       </c>
     </row>
-    <row r="60" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="60" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A60" s="30"/>
       <c r="B60" s="19" t="s">
         <v>181</v>
@@ -6778,7 +7676,7 @@
         <v>1.88</v>
       </c>
       <c r="H60" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.27246376811594197</v>
       </c>
       <c r="I60" s="19"/>
@@ -6786,18 +7684,34 @@
         <v>10</v>
       </c>
       <c r="K60" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>2.72463768115942</v>
       </c>
-      <c r="L60" s="18" t="s">
+      <c r="L60" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M60" s="46">
+      <c r="M60" s="50">
+        <f t="shared" si="5"/>
+        <v>386.89855072463763</v>
+      </c>
+      <c r="N60" s="51">
+        <f t="shared" si="0"/>
+        <v>3868.9855072463761</v>
+      </c>
+      <c r="O60" s="50">
+        <f>(920*J60)</f>
+        <v>9200</v>
+      </c>
+      <c r="P60" s="51">
+        <f t="shared" si="1"/>
+        <v>5331.0144927536239</v>
+      </c>
+      <c r="Q60" s="47">
         <f t="shared" si="2"/>
-        <v>386.89855072463763</v>
+        <v>533.10144927536237</v>
       </c>
     </row>
-    <row r="61" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="61" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A61" s="30"/>
       <c r="B61" s="19" t="s">
         <v>181</v>
@@ -6816,7 +7730,7 @@
         <v>2.0099999999999998</v>
       </c>
       <c r="H61" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.29130434782608688</v>
       </c>
       <c r="I61" s="19"/>
@@ -6824,18 +7738,34 @@
         <v>10</v>
       </c>
       <c r="K61" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>2.9130434782608687</v>
       </c>
-      <c r="L61" s="18" t="s">
+      <c r="L61" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M61" s="46">
+      <c r="M61" s="50">
+        <f t="shared" si="5"/>
+        <v>413.65217391304338</v>
+      </c>
+      <c r="N61" s="51">
+        <f t="shared" si="0"/>
+        <v>4136.5217391304341</v>
+      </c>
+      <c r="O61" s="50">
+        <f>(1471*J61)</f>
+        <v>14710</v>
+      </c>
+      <c r="P61" s="51">
+        <f t="shared" si="1"/>
+        <v>10573.478260869566</v>
+      </c>
+      <c r="Q61" s="47">
         <f t="shared" si="2"/>
-        <v>413.65217391304338</v>
+        <v>1057.3478260869565</v>
       </c>
     </row>
-    <row r="62" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="62" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A62" s="30"/>
       <c r="B62" s="19" t="s">
         <v>181</v>
@@ -6860,18 +7790,34 @@
         <v>10</v>
       </c>
       <c r="K62" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>2.043478260869565</v>
       </c>
-      <c r="L62" s="18" t="s">
+      <c r="L62" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M62" s="46">
+      <c r="M62" s="50">
+        <f t="shared" si="5"/>
+        <v>290.17391304347825</v>
+      </c>
+      <c r="N62" s="51">
+        <f t="shared" si="0"/>
+        <v>2901.7391304347825</v>
+      </c>
+      <c r="O62" s="50">
+        <f>(750*J62)</f>
+        <v>7500</v>
+      </c>
+      <c r="P62" s="51">
+        <f t="shared" si="1"/>
+        <v>4598.2608695652179</v>
+      </c>
+      <c r="Q62" s="47">
         <f t="shared" si="2"/>
-        <v>290.17391304347825</v>
+        <v>459.82608695652181</v>
       </c>
     </row>
-    <row r="63" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="63" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A63" s="30"/>
       <c r="B63" s="19" t="s">
         <v>181</v>
@@ -6888,7 +7834,7 @@
         <v>1.88</v>
       </c>
       <c r="H63" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.27246376811594197</v>
       </c>
       <c r="I63" s="19"/>
@@ -6896,18 +7842,34 @@
         <v>10</v>
       </c>
       <c r="K63" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>2.72463768115942</v>
       </c>
-      <c r="L63" s="18" t="s">
+      <c r="L63" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M63" s="46">
+      <c r="M63" s="50">
+        <f t="shared" si="5"/>
+        <v>386.89855072463763</v>
+      </c>
+      <c r="N63" s="51">
+        <f t="shared" si="0"/>
+        <v>3868.9855072463761</v>
+      </c>
+      <c r="O63" s="50">
+        <f>(996*J63)</f>
+        <v>9960</v>
+      </c>
+      <c r="P63" s="51">
+        <f t="shared" si="1"/>
+        <v>6091.0144927536239</v>
+      </c>
+      <c r="Q63" s="47">
         <f t="shared" si="2"/>
-        <v>386.89855072463763</v>
+        <v>609.10144927536237</v>
       </c>
     </row>
-    <row r="64" spans="1:13" s="24" customFormat="1" ht="27" customHeight="1">
+    <row r="64" spans="1:17" s="24" customFormat="1" ht="27" customHeight="1">
       <c r="A64" s="30"/>
       <c r="B64" s="19" t="s">
         <v>181</v>
@@ -6924,7 +7886,7 @@
         <v>2.0099999999999998</v>
       </c>
       <c r="H64" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.29130434782608688</v>
       </c>
       <c r="I64" s="19"/>
@@ -6932,18 +7894,34 @@
         <v>10</v>
       </c>
       <c r="K64" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>2.9130434782608687</v>
       </c>
-      <c r="L64" s="18" t="s">
+      <c r="L64" s="48" t="s">
         <v>14</v>
       </c>
-      <c r="M64" s="46">
+      <c r="M64" s="50">
+        <f t="shared" si="5"/>
+        <v>413.65217391304338</v>
+      </c>
+      <c r="N64" s="51">
+        <f t="shared" si="0"/>
+        <v>4136.5217391304341</v>
+      </c>
+      <c r="O64" s="50">
+        <f>(1471*J64)</f>
+        <v>14710</v>
+      </c>
+      <c r="P64" s="51">
+        <f t="shared" si="1"/>
+        <v>10573.478260869566</v>
+      </c>
+      <c r="Q64" s="47">
         <f t="shared" si="2"/>
-        <v>413.65217391304338</v>
+        <v>1057.3478260869565</v>
       </c>
     </row>
-    <row r="65" spans="1:13" s="24" customFormat="1" ht="78" customHeight="1">
+    <row r="65" spans="1:17" s="24" customFormat="1" ht="78" customHeight="1">
       <c r="A65" s="30"/>
       <c r="B65" s="32"/>
       <c r="C65" s="30"/>
@@ -6958,7 +7936,7 @@
         <v>0.88</v>
       </c>
       <c r="H65" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.12753623188405797</v>
       </c>
       <c r="I65" s="30"/>
@@ -6966,16 +7944,32 @@
         <v>40</v>
       </c>
       <c r="K65" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>5.1014492753623184</v>
       </c>
-      <c r="L65" s="30"/>
-      <c r="M65" s="46">
-        <f t="shared" si="2"/>
+      <c r="L65" s="49"/>
+      <c r="M65" s="50">
+        <f t="shared" si="5"/>
         <v>181.10144927536231</v>
       </c>
+      <c r="N65" s="51">
+        <f t="shared" si="0"/>
+        <v>7244.0579710144921</v>
+      </c>
+      <c r="O65" s="50">
+        <f>(1000*J65)</f>
+        <v>40000</v>
+      </c>
+      <c r="P65" s="51">
+        <f t="shared" si="1"/>
+        <v>32755.942028985508</v>
+      </c>
+      <c r="Q65" s="47">
+        <f>P65/J65</f>
+        <v>818.89855072463774</v>
+      </c>
     </row>
-    <row r="66" spans="1:13" s="24" customFormat="1" ht="84" customHeight="1">
+    <row r="66" spans="1:17" s="24" customFormat="1" ht="84" customHeight="1">
       <c r="A66" s="30"/>
       <c r="B66" s="32"/>
       <c r="C66" s="30"/>
@@ -6990,7 +7984,7 @@
         <v>2.5</v>
       </c>
       <c r="H66" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.36231884057971014</v>
       </c>
       <c r="I66" s="30"/>
@@ -6998,16 +7992,32 @@
         <v>20</v>
       </c>
       <c r="K66" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>7.2463768115942031</v>
       </c>
-      <c r="L66" s="30"/>
-      <c r="M66" s="46">
-        <f t="shared" si="2"/>
+      <c r="L66" s="49"/>
+      <c r="M66" s="50">
+        <f t="shared" si="5"/>
         <v>514.49275362318838</v>
       </c>
+      <c r="N66" s="51">
+        <f t="shared" ref="N66:N76" si="9">M66*J66</f>
+        <v>10289.855072463768</v>
+      </c>
+      <c r="O66" s="50">
+        <f>(1500*J66)</f>
+        <v>30000</v>
+      </c>
+      <c r="P66" s="51">
+        <f t="shared" ref="P66:P76" si="10">O66-N66</f>
+        <v>19710.144927536232</v>
+      </c>
+      <c r="Q66" s="47">
+        <f t="shared" ref="Q66:Q76" si="11">P66/J66</f>
+        <v>985.50724637681162</v>
+      </c>
     </row>
-    <row r="67" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="67" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A67" s="30"/>
       <c r="B67" s="32"/>
       <c r="C67" s="30"/>
@@ -7022,7 +8032,7 @@
         <v>5</v>
       </c>
       <c r="H67" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.72463768115942029</v>
       </c>
       <c r="I67" s="30"/>
@@ -7030,16 +8040,32 @@
         <v>5</v>
       </c>
       <c r="K67" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>3.6231884057971016</v>
       </c>
-      <c r="L67" s="30"/>
-      <c r="M67" s="46">
+      <c r="L67" s="49"/>
+      <c r="M67" s="50">
         <f>1420*H67</f>
         <v>1028.9855072463768</v>
       </c>
+      <c r="N67" s="51">
+        <f t="shared" si="9"/>
+        <v>5144.927536231884</v>
+      </c>
+      <c r="O67" s="50">
+        <f>(2500*J67)</f>
+        <v>12500</v>
+      </c>
+      <c r="P67" s="51">
+        <f t="shared" si="10"/>
+        <v>7355.072463768116</v>
+      </c>
+      <c r="Q67" s="47">
+        <f t="shared" si="11"/>
+        <v>1471.0144927536232</v>
+      </c>
     </row>
-    <row r="68" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="68" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A68" s="30"/>
       <c r="B68" s="32"/>
       <c r="C68" s="30"/>
@@ -7054,24 +8080,40 @@
         <v>50</v>
       </c>
       <c r="H68" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>7.2463768115942022</v>
       </c>
       <c r="I68" s="30"/>
       <c r="J68" s="31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K68" s="23">
-        <f t="shared" si="4"/>
-        <v>7.2463768115942022</v>
-      </c>
-      <c r="L68" s="30"/>
-      <c r="M68" s="46">
-        <f t="shared" ref="M67:M80" si="5">1420*H68</f>
+        <f t="shared" si="8"/>
+        <v>14.492753623188404</v>
+      </c>
+      <c r="L68" s="49"/>
+      <c r="M68" s="50">
+        <f t="shared" ref="M68:M80" si="12">1420*H68</f>
         <v>10289.855072463768</v>
       </c>
+      <c r="N68" s="51">
+        <f t="shared" si="9"/>
+        <v>20579.710144927536</v>
+      </c>
+      <c r="O68" s="50">
+        <f>(100000*J68)</f>
+        <v>200000</v>
+      </c>
+      <c r="P68" s="51">
+        <f t="shared" si="10"/>
+        <v>179420.28985507245</v>
+      </c>
+      <c r="Q68" s="47">
+        <f t="shared" si="11"/>
+        <v>89710.144927536225</v>
+      </c>
     </row>
-    <row r="69" spans="1:13" s="24" customFormat="1" ht="75.95" customHeight="1">
+    <row r="69" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
       <c r="A69" s="30"/>
       <c r="B69" s="32"/>
       <c r="C69" s="30"/>
@@ -7086,7 +8128,7 @@
         <v>2.09</v>
       </c>
       <c r="H69" s="21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>0.30289855072463767</v>
       </c>
       <c r="I69" s="30"/>
@@ -7094,16 +8136,32 @@
         <v>20</v>
       </c>
       <c r="K69" s="23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>6.0579710144927539</v>
       </c>
-      <c r="L69" s="30"/>
-      <c r="M69" s="46">
-        <f t="shared" si="5"/>
+      <c r="L69" s="49"/>
+      <c r="M69" s="50">
+        <f t="shared" si="12"/>
         <v>430.1159420289855</v>
       </c>
+      <c r="N69" s="51">
+        <f t="shared" si="9"/>
+        <v>8602.31884057971</v>
+      </c>
+      <c r="O69" s="50">
+        <f>(2000*J69)</f>
+        <v>40000</v>
+      </c>
+      <c r="P69" s="51">
+        <f t="shared" si="10"/>
+        <v>31397.681159420288</v>
+      </c>
+      <c r="Q69" s="47">
+        <f t="shared" si="11"/>
+        <v>1569.8840579710145</v>
+      </c>
     </row>
-    <row r="70" spans="1:13" s="24" customFormat="1" ht="69" customHeight="1">
+    <row r="70" spans="1:17" s="24" customFormat="1" ht="69" customHeight="1">
       <c r="A70" s="30"/>
       <c r="B70" s="32"/>
       <c r="C70" s="30"/>
@@ -7118,7 +8176,7 @@
         <v>0.13</v>
       </c>
       <c r="H70" s="21">
-        <f t="shared" ref="H70:H75" si="6">G70/6.9</f>
+        <f t="shared" ref="H70:H75" si="13">G70/6.9</f>
         <v>1.8840579710144929E-2</v>
       </c>
       <c r="I70" s="30"/>
@@ -7126,16 +8184,32 @@
         <v>50</v>
       </c>
       <c r="K70" s="23">
-        <f t="shared" ref="K70:K75" si="7">J70*H70</f>
+        <f t="shared" ref="K70:K75" si="14">J70*H70</f>
         <v>0.94202898550724645</v>
       </c>
-      <c r="L70" s="30"/>
-      <c r="M70" s="46">
-        <f t="shared" si="5"/>
+      <c r="L70" s="49"/>
+      <c r="M70" s="50">
+        <f t="shared" si="12"/>
         <v>26.753623188405797</v>
       </c>
+      <c r="N70" s="51">
+        <f t="shared" si="9"/>
+        <v>1337.6811594202898</v>
+      </c>
+      <c r="O70" s="50">
+        <f>(200*J70)</f>
+        <v>10000</v>
+      </c>
+      <c r="P70" s="51">
+        <f t="shared" si="10"/>
+        <v>8662.31884057971</v>
+      </c>
+      <c r="Q70" s="47">
+        <f t="shared" si="11"/>
+        <v>173.24637681159419</v>
+      </c>
     </row>
-    <row r="71" spans="1:13" s="24" customFormat="1" ht="81" customHeight="1">
+    <row r="71" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
       <c r="A71" s="30"/>
       <c r="B71" s="32"/>
       <c r="C71" s="30"/>
@@ -7150,7 +8224,7 @@
         <v>13.2</v>
       </c>
       <c r="H71" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>1.9130434782608694</v>
       </c>
       <c r="I71" s="30"/>
@@ -7158,16 +8232,32 @@
         <v>10</v>
       </c>
       <c r="K71" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>19.130434782608695</v>
       </c>
-      <c r="L71" s="30"/>
-      <c r="M71" s="46">
-        <f t="shared" si="5"/>
+      <c r="L71" s="49"/>
+      <c r="M71" s="50">
+        <f t="shared" si="12"/>
         <v>2716.5217391304345</v>
       </c>
+      <c r="N71" s="51">
+        <f t="shared" si="9"/>
+        <v>27165.217391304344</v>
+      </c>
+      <c r="O71" s="50">
+        <f>(7000*J71)</f>
+        <v>70000</v>
+      </c>
+      <c r="P71" s="51">
+        <f t="shared" si="10"/>
+        <v>42834.782608695656</v>
+      </c>
+      <c r="Q71" s="47">
+        <f t="shared" si="11"/>
+        <v>4283.4782608695659</v>
+      </c>
     </row>
-    <row r="72" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="72" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A72" s="30"/>
       <c r="B72" s="32"/>
       <c r="C72" s="30"/>
@@ -7182,7 +8272,7 @@
         <v>3.85</v>
       </c>
       <c r="H72" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>0.55797101449275366</v>
       </c>
       <c r="I72" s="30"/>
@@ -7190,16 +8280,32 @@
         <v>10</v>
       </c>
       <c r="K72" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>5.579710144927537</v>
       </c>
-      <c r="L72" s="30"/>
-      <c r="M72" s="46">
-        <f t="shared" si="5"/>
+      <c r="L72" s="49"/>
+      <c r="M72" s="50">
+        <f t="shared" si="12"/>
         <v>792.31884057971024</v>
       </c>
+      <c r="N72" s="51">
+        <f t="shared" si="9"/>
+        <v>7923.188405797102</v>
+      </c>
+      <c r="O72" s="50">
+        <f>(1999*J72)</f>
+        <v>19990</v>
+      </c>
+      <c r="P72" s="51">
+        <f>O72-N72</f>
+        <v>12066.811594202898</v>
+      </c>
+      <c r="Q72" s="47">
+        <f t="shared" si="11"/>
+        <v>1206.6811594202898</v>
+      </c>
     </row>
-    <row r="73" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="73" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A73" s="30"/>
       <c r="B73" s="32"/>
       <c r="C73" s="30"/>
@@ -7214,7 +8320,7 @@
         <v>5.15</v>
       </c>
       <c r="H73" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>0.74637681159420288</v>
       </c>
       <c r="I73" s="30"/>
@@ -7222,16 +8328,32 @@
         <v>10</v>
       </c>
       <c r="K73" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>7.4637681159420293</v>
       </c>
-      <c r="L73" s="30"/>
-      <c r="M73" s="46">
-        <f t="shared" si="5"/>
+      <c r="L73" s="49"/>
+      <c r="M73" s="50">
+        <f t="shared" si="12"/>
         <v>1059.855072463768</v>
       </c>
+      <c r="N73" s="51">
+        <f t="shared" si="9"/>
+        <v>10598.55072463768</v>
+      </c>
+      <c r="O73" s="50">
+        <f>(4000*J73)</f>
+        <v>40000</v>
+      </c>
+      <c r="P73" s="51">
+        <f t="shared" si="10"/>
+        <v>29401.44927536232</v>
+      </c>
+      <c r="Q73" s="47">
+        <f t="shared" si="11"/>
+        <v>2940.144927536232</v>
+      </c>
     </row>
-    <row r="74" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="74" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A74" s="30"/>
       <c r="B74" s="32"/>
       <c r="C74" s="30"/>
@@ -7246,7 +8368,7 @@
         <v>8.25</v>
       </c>
       <c r="H74" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>1.1956521739130435</v>
       </c>
       <c r="I74" s="30"/>
@@ -7254,16 +8376,32 @@
         <v>10</v>
       </c>
       <c r="K74" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>11.956521739130434</v>
       </c>
-      <c r="L74" s="30"/>
-      <c r="M74" s="46">
-        <f t="shared" si="5"/>
+      <c r="L74" s="49"/>
+      <c r="M74" s="50">
+        <f t="shared" si="12"/>
         <v>1697.8260869565217</v>
       </c>
+      <c r="N74" s="51">
+        <f t="shared" si="9"/>
+        <v>16978.260869565216</v>
+      </c>
+      <c r="O74" s="50">
+        <f>(5000*J74)</f>
+        <v>50000</v>
+      </c>
+      <c r="P74" s="51">
+        <f t="shared" si="10"/>
+        <v>33021.739130434784</v>
+      </c>
+      <c r="Q74" s="47">
+        <f t="shared" si="11"/>
+        <v>3302.1739130434785</v>
+      </c>
     </row>
-    <row r="75" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="75" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A75" s="30"/>
       <c r="B75" s="32"/>
       <c r="C75" s="30"/>
@@ -7278,7 +8416,7 @@
         <v>0.44</v>
       </c>
       <c r="H75" s="21">
-        <f t="shared" si="6"/>
+        <f t="shared" si="13"/>
         <v>6.3768115942028983E-2</v>
       </c>
       <c r="I75" s="30"/>
@@ -7286,16 +8424,32 @@
         <v>20</v>
       </c>
       <c r="K75" s="23">
-        <f t="shared" si="7"/>
+        <f t="shared" si="14"/>
         <v>1.2753623188405796</v>
       </c>
-      <c r="L75" s="30"/>
-      <c r="M75" s="46">
-        <f t="shared" si="5"/>
+      <c r="L75" s="49"/>
+      <c r="M75" s="50">
+        <f t="shared" si="12"/>
         <v>90.550724637681157</v>
       </c>
+      <c r="N75" s="51">
+        <f t="shared" si="9"/>
+        <v>1811.014492753623</v>
+      </c>
+      <c r="O75" s="50">
+        <f>(500*J75)</f>
+        <v>10000</v>
+      </c>
+      <c r="P75" s="51">
+        <f t="shared" si="10"/>
+        <v>8188.985507246377</v>
+      </c>
+      <c r="Q75" s="47">
+        <f t="shared" si="11"/>
+        <v>409.44927536231887</v>
+      </c>
     </row>
-    <row r="76" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="76" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A76" s="30"/>
       <c r="B76" s="32"/>
       <c r="C76" s="33" t="s">
@@ -7321,13 +8475,20 @@
       <c r="K76" s="23">
         <v>29.8571428571429</v>
       </c>
-      <c r="L76" s="30"/>
-      <c r="M76" s="46">
-        <f t="shared" si="5"/>
+      <c r="L76" s="49"/>
+      <c r="M76" s="50">
+        <f t="shared" si="12"/>
         <v>42397.142857142921</v>
       </c>
+      <c r="N76" s="51"/>
+      <c r="O76" s="50"/>
+      <c r="P76" s="51"/>
+      <c r="Q76" s="47">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="77" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="77" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A77" s="30"/>
       <c r="B77" s="32"/>
       <c r="C77" s="38" t="s">
@@ -7354,13 +8515,29 @@
         <f>H77*J77</f>
         <v>33.624000000000002</v>
       </c>
-      <c r="L77" s="30"/>
-      <c r="M77" s="46">
-        <f t="shared" si="5"/>
+      <c r="L77" s="49"/>
+      <c r="M77" s="50">
+        <f>1420*H77</f>
         <v>11936.52</v>
       </c>
+      <c r="N77" s="51">
+        <f>M77*J77</f>
+        <v>47746.080000000002</v>
+      </c>
+      <c r="O77" s="50">
+        <f>(20000*J77)</f>
+        <v>80000</v>
+      </c>
+      <c r="P77" s="51">
+        <f>O77-N77</f>
+        <v>32253.919999999998</v>
+      </c>
+      <c r="Q77" s="47">
+        <f>P77/J77</f>
+        <v>8063.48</v>
+      </c>
     </row>
-    <row r="78" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="78" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A78" s="30"/>
       <c r="B78" s="32"/>
       <c r="C78" s="38" t="s">
@@ -7385,13 +8562,29 @@
         <f>J78*H78</f>
         <v>4.3849999999999998</v>
       </c>
-      <c r="L78" s="30"/>
-      <c r="M78" s="46">
-        <f t="shared" si="5"/>
+      <c r="L78" s="49"/>
+      <c r="M78" s="50">
+        <f t="shared" si="12"/>
         <v>1245.3399999999999</v>
       </c>
+      <c r="N78" s="51">
+        <f t="shared" ref="N78:N80" si="15">M78*J78</f>
+        <v>6226.7</v>
+      </c>
+      <c r="O78" s="50">
+        <f>(3000*J78)</f>
+        <v>15000</v>
+      </c>
+      <c r="P78" s="51">
+        <f t="shared" ref="P78:P80" si="16">O78-N78</f>
+        <v>8773.2999999999993</v>
+      </c>
+      <c r="Q78" s="47">
+        <f t="shared" ref="Q78:Q80" si="17">P78/J78</f>
+        <v>1754.6599999999999</v>
+      </c>
     </row>
-    <row r="79" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="79" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A79" s="30"/>
       <c r="B79" s="32"/>
       <c r="C79" s="41" t="s">
@@ -7416,13 +8609,29 @@
         <f>H79*J79</f>
         <v>17.535</v>
       </c>
-      <c r="L79" s="30"/>
-      <c r="M79" s="46">
-        <f t="shared" si="5"/>
+      <c r="L79" s="49"/>
+      <c r="M79" s="50">
+        <f t="shared" si="12"/>
         <v>4979.9400000000005</v>
       </c>
+      <c r="N79" s="51">
+        <f t="shared" si="15"/>
+        <v>24899.700000000004</v>
+      </c>
+      <c r="O79" s="50">
+        <f>(8000*J79)</f>
+        <v>40000</v>
+      </c>
+      <c r="P79" s="51">
+        <f t="shared" si="16"/>
+        <v>15100.299999999996</v>
+      </c>
+      <c r="Q79" s="47">
+        <f t="shared" si="17"/>
+        <v>3020.059999999999</v>
+      </c>
     </row>
-    <row r="80" spans="1:13" s="24" customFormat="1" ht="72.95" customHeight="1">
+    <row r="80" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
       <c r="A80" s="30"/>
       <c r="B80" s="32"/>
       <c r="C80" s="24" t="s">
@@ -7446,13 +8655,20 @@
       <c r="K80" s="23">
         <v>5.87</v>
       </c>
-      <c r="L80" s="30"/>
-      <c r="M80" s="46">
-        <f t="shared" si="5"/>
+      <c r="L80" s="49"/>
+      <c r="M80" s="50">
+        <f t="shared" si="12"/>
         <v>8335.4</v>
       </c>
+      <c r="N80" s="51"/>
+      <c r="O80" s="50"/>
+      <c r="P80" s="51">
+        <f>SUM(P2:P79)</f>
+        <v>1937904.4765217388</v>
+      </c>
+      <c r="Q80" s="47"/>
     </row>
-    <row r="81" spans="1:12" ht="18.75">
+    <row r="81" spans="1:16" ht="33.75" customHeight="1">
       <c r="A81" s="15"/>
       <c r="B81" s="14"/>
       <c r="C81" s="17"/>
@@ -7465,8 +8681,12 @@
       <c r="J81" s="10"/>
       <c r="K81" s="12"/>
       <c r="L81" s="9"/>
+      <c r="P81" s="52">
+        <f>P80-1180000</f>
+        <v>757904.4765217388</v>
+      </c>
     </row>
-    <row r="82" spans="1:12">
+    <row r="82" spans="1:16">
       <c r="A82" s="9"/>
       <c r="B82" s="11"/>
       <c r="C82" s="9"/>
@@ -7479,11 +8699,11 @@
       <c r="J82" s="10"/>
       <c r="K82" s="13">
         <f>SUM(K2:K81)</f>
-        <v>567.94505590062101</v>
+        <v>575.19143271221526</v>
       </c>
       <c r="L82" s="9"/>
     </row>
-    <row r="83" spans="1:12">
+    <row r="83" spans="1:16">
       <c r="A83" s="9"/>
       <c r="B83" s="11"/>
       <c r="C83" s="9"/>

</xml_diff>

<commit_message>
feat(seo): implement SSR JSON-LD generation for GEO/AEO optimization 2026
</commit_message>
<xml_diff>
--- a/Binzhou_Houyi (1) (1).xlsx
+++ b/Binzhou_Houyi (1) (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaafa\Desktop\upload\FishWebClean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31F4617-BEDE-4963-9471-454D9AEDAD26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FB3F105-52F1-49D2-9F92-1B331CCF89AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -745,7 +745,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -780,6 +780,18 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FFFFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor rgb="FFC8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -872,7 +884,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -995,20 +1007,8 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1026,6 +1026,69 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="8" borderId="1" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1658,102 +1721,6 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>50800</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1271</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>802640</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="16" name="图片 15">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9048750" y="12585700"/>
-          <a:ext cx="991870" cy="751840"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>635</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="17" name="图片 16">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9039225" y="13417550"/>
-          <a:ext cx="1019175" cy="673735"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
@@ -1778,7 +1745,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1787,54 +1754,6 @@
         <a:xfrm>
           <a:off x="9067800" y="14122400"/>
           <a:ext cx="989330" cy="880745"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>2541</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>933450</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="19" name="图片 18">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000013000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="9058275" y="15078075"/>
-          <a:ext cx="926465" cy="866775"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1874,7 +1793,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1918,7 +1837,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1966,7 +1885,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2014,7 +1933,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2062,7 +1981,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2110,7 +2029,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2158,7 +2077,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2206,7 +2125,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2254,7 +2173,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2302,7 +2221,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2350,7 +2269,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2398,7 +2317,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2446,7 +2365,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2490,7 +2409,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2534,7 +2453,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2578,7 +2497,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2622,7 +2541,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId31"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2666,7 +2585,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId32"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2714,7 +2633,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId33"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2762,7 +2681,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId34"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2810,7 +2729,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId35"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2858,7 +2777,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId39"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2906,7 +2825,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId37"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2954,7 +2873,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -2998,7 +2917,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId39"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3042,7 +2961,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId43"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3086,7 +3005,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId41"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3130,7 +3049,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId45"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3174,7 +3093,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId43"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3218,7 +3137,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId47"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3262,7 +3181,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId45"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3306,7 +3225,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId49"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3354,7 +3273,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId50"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId47"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3402,7 +3321,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId51"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3450,7 +3369,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId52"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId49"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3494,7 +3413,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId53"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId50"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3538,7 +3457,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId54"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId51"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3586,7 +3505,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId55"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId52"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3630,7 +3549,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId56"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId53"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3674,7 +3593,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId57"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId54"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3718,7 +3637,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId58"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId55"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3762,7 +3681,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId59">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId56">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -3823,7 +3742,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId60" r:link="rId61"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId57" r:link="rId58"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3871,7 +3790,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId62"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId59"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3919,7 +3838,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId63"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId60"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3932,54 +3851,6 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>18775</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>868208</xdr:colOff>
-      <xdr:row>79</xdr:row>
-      <xdr:rowOff>904875</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="66" name="图片 110">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD07763F-5D82-4A38-AEA8-6B17675CA3EA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId64"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="9889056" y="62150625"/>
-          <a:ext cx="849433" cy="714375"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525">
-          <a:noFill/>
-        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -4011,7 +3882,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId65"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId61"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4410,24 +4281,24 @@
       <c r="L2" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="43">
+      <c r="M2" s="42">
         <f>1420*H2</f>
         <v>5433.0434782608691</v>
       </c>
-      <c r="N2" s="51">
+      <c r="N2" s="47">
         <f t="shared" ref="N2:N65" si="0">M2*J2</f>
         <v>16299.130434782608</v>
       </c>
-      <c r="O2" s="50">
+      <c r="O2" s="46">
         <f>(18000*J2)</f>
         <v>54000</v>
       </c>
-      <c r="P2" s="51">
+      <c r="P2" s="47">
         <f t="shared" ref="P2:P65" si="1">O2-N2</f>
         <v>37700.869565217392</v>
       </c>
-      <c r="Q2" s="47">
-        <f t="shared" ref="Q2:Q65" si="2">P2/J2</f>
+      <c r="Q2" s="43">
+        <f t="shared" ref="Q2:Q22" si="2">P2/J2</f>
         <v>12566.95652173913</v>
       </c>
     </row>
@@ -4468,23 +4339,23 @@
       <c r="L3" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M3" s="43">
+      <c r="M3" s="42">
         <f t="shared" ref="M3:M66" si="5">1420*H3</f>
         <v>498.02898550724638</v>
       </c>
-      <c r="N3" s="51">
+      <c r="N3" s="47">
         <f t="shared" si="0"/>
         <v>2490.144927536232</v>
       </c>
-      <c r="O3" s="50">
+      <c r="O3" s="46">
         <f>(3000*J3)</f>
         <v>15000</v>
       </c>
-      <c r="P3" s="51">
+      <c r="P3" s="47">
         <f t="shared" si="1"/>
         <v>12509.855072463768</v>
       </c>
-      <c r="Q3" s="47">
+      <c r="Q3" s="43">
         <f t="shared" si="2"/>
         <v>2501.9710144927535</v>
       </c>
@@ -4526,23 +4397,23 @@
       <c r="L4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="43">
+      <c r="M4" s="42">
         <f t="shared" si="5"/>
         <v>967.24637681159425</v>
       </c>
-      <c r="N4" s="51">
+      <c r="N4" s="47">
         <f t="shared" si="0"/>
         <v>4836.231884057971</v>
       </c>
-      <c r="O4" s="50">
+      <c r="O4" s="46">
         <f>(6000*J4)</f>
         <v>30000</v>
       </c>
-      <c r="P4" s="51">
+      <c r="P4" s="47">
         <f t="shared" si="1"/>
         <v>25163.768115942028</v>
       </c>
-      <c r="Q4" s="47">
+      <c r="Q4" s="43">
         <f t="shared" si="2"/>
         <v>5032.753623188406</v>
       </c>
@@ -4584,23 +4455,23 @@
       <c r="L5" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="43">
+      <c r="M5" s="42">
         <f t="shared" si="5"/>
         <v>1992.1159420289855</v>
       </c>
-      <c r="N5" s="51">
+      <c r="N5" s="47">
         <f t="shared" si="0"/>
         <v>9960.579710144928</v>
       </c>
-      <c r="O5" s="50">
+      <c r="O5" s="46">
         <f>(10000*J5)</f>
         <v>50000</v>
       </c>
-      <c r="P5" s="51">
+      <c r="P5" s="47">
         <f t="shared" si="1"/>
         <v>40039.420289855072</v>
       </c>
-      <c r="Q5" s="47">
+      <c r="Q5" s="43">
         <f t="shared" si="2"/>
         <v>8007.884057971014</v>
       </c>
@@ -4642,23 +4513,23 @@
       <c r="L6" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M6" s="43">
+      <c r="M6" s="42">
         <f t="shared" si="5"/>
         <v>1131.8840579710145</v>
       </c>
-      <c r="N6" s="51">
+      <c r="N6" s="47">
         <f t="shared" si="0"/>
         <v>16978.260869565216</v>
       </c>
-      <c r="O6" s="50">
+      <c r="O6" s="46">
         <f>(3500*J6)</f>
         <v>52500</v>
       </c>
-      <c r="P6" s="51">
+      <c r="P6" s="47">
         <f t="shared" si="1"/>
         <v>35521.739130434784</v>
       </c>
-      <c r="Q6" s="47">
+      <c r="Q6" s="43">
         <f t="shared" si="2"/>
         <v>2368.1159420289855</v>
       </c>
@@ -4700,23 +4571,23 @@
       <c r="L7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="43">
+      <c r="M7" s="42">
         <f t="shared" si="5"/>
         <v>226.37681159420291</v>
       </c>
-      <c r="N7" s="51">
+      <c r="N7" s="47">
         <f t="shared" si="0"/>
         <v>3395.6521739130435</v>
       </c>
-      <c r="O7" s="50">
+      <c r="O7" s="46">
         <f>(1500*J7)</f>
         <v>22500</v>
       </c>
-      <c r="P7" s="51">
+      <c r="P7" s="47">
         <f t="shared" si="1"/>
         <v>19104.347826086956</v>
       </c>
-      <c r="Q7" s="47">
+      <c r="Q7" s="43">
         <f t="shared" si="2"/>
         <v>1273.623188405797</v>
       </c>
@@ -4758,23 +4629,23 @@
       <c r="L8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M8" s="43">
+      <c r="M8" s="42">
         <f t="shared" si="5"/>
         <v>226.37681159420291</v>
       </c>
-      <c r="N8" s="51">
+      <c r="N8" s="47">
         <f t="shared" si="0"/>
         <v>4527.536231884058</v>
       </c>
-      <c r="O8" s="50">
+      <c r="O8" s="46">
         <f>(1500*J8)</f>
         <v>30000</v>
       </c>
-      <c r="P8" s="51">
+      <c r="P8" s="47">
         <f t="shared" si="1"/>
         <v>25472.463768115944</v>
       </c>
-      <c r="Q8" s="47">
+      <c r="Q8" s="43">
         <f t="shared" si="2"/>
         <v>1273.6231884057972</v>
       </c>
@@ -4816,23 +4687,23 @@
       <c r="L9" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="43">
+      <c r="M9" s="42">
         <f t="shared" si="5"/>
         <v>3622.0289855072465</v>
       </c>
-      <c r="N9" s="51">
+      <c r="N9" s="47">
         <f t="shared" si="0"/>
         <v>18110.144927536232</v>
       </c>
-      <c r="O9" s="50">
+      <c r="O9" s="46">
         <f>(12000*J9)</f>
         <v>60000</v>
       </c>
-      <c r="P9" s="51">
+      <c r="P9" s="47">
         <f t="shared" si="1"/>
         <v>41889.855072463768</v>
       </c>
-      <c r="Q9" s="47">
+      <c r="Q9" s="43">
         <f t="shared" si="2"/>
         <v>8377.971014492754</v>
       </c>
@@ -4874,23 +4745,23 @@
       <c r="L10" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="M10" s="43">
+      <c r="M10" s="42">
         <f t="shared" si="5"/>
         <v>2241.1304347826085</v>
       </c>
-      <c r="N10" s="51">
+      <c r="N10" s="47">
         <f t="shared" si="0"/>
         <v>17929.043478260868</v>
       </c>
-      <c r="O10" s="50">
+      <c r="O10" s="46">
         <f>(6000*J10)</f>
         <v>48000</v>
       </c>
-      <c r="P10" s="51">
+      <c r="P10" s="47">
         <f t="shared" si="1"/>
         <v>30070.956521739132</v>
       </c>
-      <c r="Q10" s="47">
+      <c r="Q10" s="43">
         <f t="shared" si="2"/>
         <v>3758.8695652173915</v>
       </c>
@@ -4921,7 +4792,7 @@
         <f t="shared" si="3"/>
         <v>4.63768115942029</v>
       </c>
-      <c r="I11" s="44"/>
+      <c r="I11" s="49"/>
       <c r="J11" s="22">
         <v>2</v>
       </c>
@@ -4932,23 +4803,23 @@
       <c r="L11" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M11" s="43">
+      <c r="M11" s="42">
         <f t="shared" si="5"/>
         <v>6585.507246376812</v>
       </c>
-      <c r="N11" s="51">
+      <c r="N11" s="47">
         <f t="shared" si="0"/>
         <v>13171.014492753624</v>
       </c>
-      <c r="O11" s="50">
+      <c r="O11" s="46">
         <f>(20000*J11)</f>
         <v>40000</v>
       </c>
-      <c r="P11" s="51">
+      <c r="P11" s="47">
         <f t="shared" si="1"/>
         <v>26828.985507246376</v>
       </c>
-      <c r="Q11" s="47">
+      <c r="Q11" s="43">
         <f t="shared" si="2"/>
         <v>13414.492753623188</v>
       </c>
@@ -4979,7 +4850,7 @@
         <f t="shared" si="3"/>
         <v>7.2463768115942022</v>
       </c>
-      <c r="I12" s="45"/>
+      <c r="I12" s="50"/>
       <c r="J12" s="22">
         <v>2</v>
       </c>
@@ -4990,23 +4861,23 @@
       <c r="L12" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M12" s="43">
+      <c r="M12" s="42">
         <f t="shared" si="5"/>
         <v>10289.855072463768</v>
       </c>
-      <c r="N12" s="51">
+      <c r="N12" s="47">
         <f t="shared" si="0"/>
         <v>20579.710144927536</v>
       </c>
-      <c r="O12" s="50">
+      <c r="O12" s="46">
         <f>(40000*J12)</f>
         <v>80000</v>
       </c>
-      <c r="P12" s="51">
+      <c r="P12" s="47">
         <f t="shared" si="1"/>
         <v>59420.289855072464</v>
       </c>
-      <c r="Q12" s="47">
+      <c r="Q12" s="43">
         <f t="shared" si="2"/>
         <v>29710.144927536232</v>
       </c>
@@ -5037,7 +4908,7 @@
         <f t="shared" si="3"/>
         <v>4.057971014492753</v>
       </c>
-      <c r="I13" s="45"/>
+      <c r="I13" s="50"/>
       <c r="J13" s="22">
         <v>2</v>
       </c>
@@ -5048,23 +4919,23 @@
       <c r="L13" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M13" s="43">
+      <c r="M13" s="42">
         <f t="shared" si="5"/>
         <v>5762.3188405797091</v>
       </c>
-      <c r="N13" s="51">
+      <c r="N13" s="47">
         <f t="shared" si="0"/>
         <v>11524.637681159418</v>
       </c>
-      <c r="O13" s="50">
-        <f t="shared" ref="O2:O65" si="6">(20000*J13)</f>
+      <c r="O13" s="46">
+        <f t="shared" ref="O13:O44" si="6">(20000*J13)</f>
         <v>40000</v>
       </c>
-      <c r="P13" s="51">
+      <c r="P13" s="47">
         <f t="shared" si="1"/>
         <v>28475.362318840584</v>
       </c>
-      <c r="Q13" s="47">
+      <c r="Q13" s="43">
         <f t="shared" si="2"/>
         <v>14237.681159420292</v>
       </c>
@@ -5095,7 +4966,7 @@
         <f t="shared" si="3"/>
         <v>4.63768115942029</v>
       </c>
-      <c r="I14" s="46"/>
+      <c r="I14" s="51"/>
       <c r="J14" s="22">
         <v>3</v>
       </c>
@@ -5106,23 +4977,23 @@
       <c r="L14" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M14" s="43">
+      <c r="M14" s="42">
         <f t="shared" si="5"/>
         <v>6585.507246376812</v>
       </c>
-      <c r="N14" s="51">
+      <c r="N14" s="47">
         <f t="shared" si="0"/>
         <v>19756.521739130436</v>
       </c>
-      <c r="O14" s="50">
+      <c r="O14" s="46">
         <f t="shared" si="6"/>
         <v>60000</v>
       </c>
-      <c r="P14" s="51">
+      <c r="P14" s="47">
         <f t="shared" si="1"/>
         <v>40243.478260869568</v>
       </c>
-      <c r="Q14" s="47">
+      <c r="Q14" s="43">
         <f t="shared" si="2"/>
         <v>13414.49275362319</v>
       </c>
@@ -5164,22 +5035,25 @@
       <c r="L15" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M15" s="43">
+      <c r="M15" s="42">
         <f t="shared" si="5"/>
         <v>7408.695652173913</v>
       </c>
-      <c r="N15" s="51">
+      <c r="N15" s="47">
         <f t="shared" si="0"/>
         <v>14817.391304347826</v>
       </c>
-      <c r="O15" s="50">
+      <c r="O15" s="46">
         <f>(28000*J15)</f>
         <v>56000</v>
       </c>
-      <c r="P15" s="51"/>
-      <c r="Q15" s="47">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="P15" s="47">
+        <f>O15-N15</f>
+        <v>41182.608695652176</v>
+      </c>
+      <c r="Q15" s="43">
+        <f>P15/J15</f>
+        <v>20591.304347826088</v>
       </c>
     </row>
     <row r="16" spans="1:17" s="24" customFormat="1" ht="74.099999999999994" customHeight="1">
@@ -5219,17 +5093,17 @@
       <c r="L16" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M16" s="43">
+      <c r="M16" s="42">
         <f t="shared" si="5"/>
         <v>2716.5217391304345</v>
       </c>
-      <c r="N16" s="51">
+      <c r="N16" s="47">
         <f t="shared" si="0"/>
         <v>13582.608695652172</v>
       </c>
-      <c r="O16" s="50"/>
-      <c r="P16" s="51"/>
-      <c r="Q16" s="47">
+      <c r="O16" s="46"/>
+      <c r="P16" s="47"/>
+      <c r="Q16" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -5260,7 +5134,7 @@
         <f t="shared" si="3"/>
         <v>0.14492753623188406</v>
       </c>
-      <c r="I17" s="44"/>
+      <c r="I17" s="49"/>
       <c r="J17" s="22">
         <v>5</v>
       </c>
@@ -5271,17 +5145,17 @@
       <c r="L17" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M17" s="43">
+      <c r="M17" s="42">
         <f t="shared" si="5"/>
         <v>205.79710144927537</v>
       </c>
-      <c r="N17" s="51">
+      <c r="N17" s="47">
         <f t="shared" si="0"/>
         <v>1028.985507246377</v>
       </c>
-      <c r="O17" s="50"/>
-      <c r="P17" s="51"/>
-      <c r="Q17" s="47">
+      <c r="O17" s="46"/>
+      <c r="P17" s="47"/>
+      <c r="Q17" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -5312,7 +5186,7 @@
         <f t="shared" si="3"/>
         <v>0.21739130434782608</v>
       </c>
-      <c r="I18" s="45"/>
+      <c r="I18" s="50"/>
       <c r="J18" s="22">
         <v>5</v>
       </c>
@@ -5323,17 +5197,17 @@
       <c r="L18" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="43">
+      <c r="M18" s="42">
         <f t="shared" si="5"/>
         <v>308.69565217391306</v>
       </c>
-      <c r="N18" s="51">
+      <c r="N18" s="47">
         <f t="shared" si="0"/>
         <v>1543.4782608695652</v>
       </c>
-      <c r="O18" s="50"/>
-      <c r="P18" s="51"/>
-      <c r="Q18" s="47">
+      <c r="O18" s="46"/>
+      <c r="P18" s="47"/>
+      <c r="Q18" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -5364,7 +5238,7 @@
         <f t="shared" si="3"/>
         <v>0.52173913043478259</v>
       </c>
-      <c r="I19" s="45"/>
+      <c r="I19" s="50"/>
       <c r="J19" s="22">
         <v>5</v>
       </c>
@@ -5375,17 +5249,17 @@
       <c r="L19" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M19" s="43">
+      <c r="M19" s="42">
         <f t="shared" si="5"/>
         <v>740.86956521739125</v>
       </c>
-      <c r="N19" s="51">
+      <c r="N19" s="47">
         <f t="shared" si="0"/>
         <v>3704.347826086956</v>
       </c>
-      <c r="O19" s="50"/>
-      <c r="P19" s="51"/>
-      <c r="Q19" s="47">
+      <c r="O19" s="46"/>
+      <c r="P19" s="47"/>
+      <c r="Q19" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -5416,7 +5290,7 @@
         <f t="shared" si="3"/>
         <v>0.94202898550724634</v>
       </c>
-      <c r="I20" s="46"/>
+      <c r="I20" s="51"/>
       <c r="J20" s="22">
         <v>3</v>
       </c>
@@ -5427,121 +5301,121 @@
       <c r="L20" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M20" s="43">
+      <c r="M20" s="42">
         <f t="shared" si="5"/>
         <v>1337.6811594202898</v>
       </c>
-      <c r="N20" s="51">
+      <c r="N20" s="47">
         <f t="shared" si="0"/>
         <v>4013.0434782608691</v>
       </c>
-      <c r="O20" s="50"/>
-      <c r="P20" s="51"/>
-      <c r="Q20" s="47">
+      <c r="O20" s="46"/>
+      <c r="P20" s="47"/>
+      <c r="Q20" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:17" s="24" customFormat="1" ht="66.95" customHeight="1">
-      <c r="A21" s="18">
+      <c r="A21" s="52">
         <v>20</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="D21" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="E21" s="19" t="s">
+      <c r="E21" s="53" t="s">
         <v>71</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="54">
         <v>24</v>
       </c>
-      <c r="H21" s="21">
+      <c r="H21" s="55">
         <f t="shared" si="3"/>
         <v>3.4782608695652173</v>
       </c>
-      <c r="I21" s="19"/>
-      <c r="J21" s="22">
+      <c r="I21" s="53"/>
+      <c r="J21" s="56">
         <v>2</v>
       </c>
-      <c r="K21" s="23">
+      <c r="K21" s="57">
         <f t="shared" si="4"/>
         <v>6.9565217391304346</v>
       </c>
-      <c r="L21" s="18" t="s">
+      <c r="L21" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="M21" s="43">
+      <c r="M21" s="58">
         <f t="shared" si="5"/>
         <v>4939.130434782609</v>
       </c>
-      <c r="N21" s="51">
+      <c r="N21" s="59">
         <f t="shared" si="0"/>
         <v>9878.2608695652179</v>
       </c>
-      <c r="O21" s="50"/>
-      <c r="P21" s="51"/>
-      <c r="Q21" s="47">
+      <c r="O21" s="60"/>
+      <c r="P21" s="59"/>
+      <c r="Q21" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:17" s="24" customFormat="1" ht="56.1" customHeight="1">
-      <c r="A22" s="18">
+      <c r="A22" s="52">
         <v>21</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="53" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="D22" s="52" t="s">
         <v>74</v>
       </c>
-      <c r="E22" s="19" t="s">
+      <c r="E22" s="53" t="s">
         <v>75</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="G22" s="20">
+      <c r="G22" s="54">
         <v>20</v>
       </c>
-      <c r="H22" s="21">
+      <c r="H22" s="55">
         <f t="shared" si="3"/>
         <v>2.8985507246376812</v>
       </c>
-      <c r="I22" s="19"/>
-      <c r="J22" s="22">
+      <c r="I22" s="53"/>
+      <c r="J22" s="56">
         <v>3</v>
       </c>
-      <c r="K22" s="23">
+      <c r="K22" s="57">
         <f t="shared" si="4"/>
         <v>8.695652173913043</v>
       </c>
-      <c r="L22" s="18" t="s">
+      <c r="L22" s="52" t="s">
         <v>43</v>
       </c>
-      <c r="M22" s="43">
+      <c r="M22" s="58">
         <f t="shared" si="5"/>
         <v>4115.942028985507</v>
       </c>
-      <c r="N22" s="51">
+      <c r="N22" s="59">
         <f t="shared" si="0"/>
         <v>12347.82608695652</v>
       </c>
-      <c r="O22" s="50"/>
-      <c r="P22" s="51"/>
-      <c r="Q22" s="47">
+      <c r="O22" s="60"/>
+      <c r="P22" s="59"/>
+      <c r="Q22" s="43">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
@@ -5583,70 +5457,76 @@
       <c r="L23" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="M23" s="43">
+      <c r="M23" s="42">
         <f>1420*H23</f>
         <v>16463.768115942028</v>
       </c>
-      <c r="N23" s="51">
+      <c r="N23" s="47">
         <f>M23*J23</f>
         <v>16463.768115942028</v>
       </c>
-      <c r="O23" s="50"/>
-      <c r="P23" s="51"/>
-      <c r="Q23" s="47">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="O23" s="46">
+        <f>6*8000</f>
+        <v>48000</v>
+      </c>
+      <c r="P23" s="47">
+        <f>O23-N23</f>
+        <v>31536.231884057972</v>
+      </c>
+      <c r="Q23" s="43">
+        <f>P23/J23</f>
+        <v>31536.231884057972</v>
       </c>
     </row>
     <row r="24" spans="1:17" s="24" customFormat="1" ht="75.95" customHeight="1">
-      <c r="A24" s="18">
+      <c r="A24" s="52">
         <v>23</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="52" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="D24" s="52" t="s">
         <v>81</v>
       </c>
-      <c r="E24" s="19" t="s">
+      <c r="E24" s="53" t="s">
         <v>82</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="G24" s="20">
+      <c r="G24" s="54">
         <v>1.1000000000000001</v>
       </c>
-      <c r="H24" s="21">
+      <c r="H24" s="55">
         <f t="shared" si="3"/>
         <v>0.15942028985507248</v>
       </c>
-      <c r="I24" s="19"/>
-      <c r="J24" s="22">
+      <c r="I24" s="53"/>
+      <c r="J24" s="56">
         <v>2</v>
       </c>
-      <c r="K24" s="23">
+      <c r="K24" s="57">
         <f t="shared" si="4"/>
         <v>0.31884057971014496</v>
       </c>
-      <c r="L24" s="18" t="s">
+      <c r="L24" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="M24" s="43">
+      <c r="M24" s="58">
         <f t="shared" si="5"/>
         <v>226.37681159420291</v>
       </c>
-      <c r="N24" s="51">
+      <c r="N24" s="59">
         <f t="shared" si="0"/>
         <v>452.75362318840581</v>
       </c>
-      <c r="O24" s="50"/>
-      <c r="P24" s="51"/>
-      <c r="Q24" s="47">
-        <f t="shared" si="2"/>
+      <c r="O24" s="60"/>
+      <c r="P24" s="59"/>
+      <c r="Q24" s="43">
+        <f>P24/J24</f>
         <v>0</v>
       </c>
     </row>
@@ -5687,24 +5567,24 @@
       <c r="L25" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M25" s="43">
+      <c r="M25" s="42">
         <f t="shared" si="5"/>
         <v>2942.8985507246375</v>
       </c>
-      <c r="N25" s="51">
+      <c r="N25" s="47">
         <f t="shared" si="0"/>
         <v>17657.391304347824</v>
       </c>
-      <c r="O25" s="50">
+      <c r="O25" s="46">
         <f>(9000*J25)</f>
         <v>54000</v>
       </c>
-      <c r="P25" s="51">
+      <c r="P25" s="47">
         <f t="shared" si="1"/>
         <v>36342.608695652176</v>
       </c>
-      <c r="Q25" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q25" s="43">
+        <f>P25/J25</f>
         <v>6057.1014492753629</v>
       </c>
     </row>
@@ -5745,25 +5625,25 @@
       <c r="L26" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="M26" s="43">
+      <c r="M26" s="42">
         <f t="shared" si="5"/>
         <v>411.59420289855075</v>
       </c>
-      <c r="N26" s="51">
-        <f t="shared" si="0"/>
+      <c r="N26" s="47">
+        <f>M26*J26</f>
         <v>12347.826086956522</v>
       </c>
-      <c r="O26" s="50">
-        <f>(1500*J26)</f>
-        <v>45000</v>
-      </c>
-      <c r="P26" s="51">
+      <c r="O26" s="46">
+        <f>(2000*J26)</f>
+        <v>60000</v>
+      </c>
+      <c r="P26" s="47">
         <f t="shared" si="1"/>
-        <v>32652.17391304348</v>
-      </c>
-      <c r="Q26" s="47">
-        <f t="shared" si="2"/>
-        <v>1088.4057971014493</v>
+        <v>47652.17391304348</v>
+      </c>
+      <c r="Q26" s="43">
+        <f>P26/J26</f>
+        <v>1588.4057971014493</v>
       </c>
     </row>
     <row r="27" spans="1:17" s="24" customFormat="1" ht="66" customHeight="1">
@@ -5803,24 +5683,24 @@
       <c r="L27" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M27" s="43">
+      <c r="M27" s="42">
         <f t="shared" si="5"/>
         <v>452.75362318840581</v>
       </c>
-      <c r="N27" s="51">
+      <c r="N27" s="47">
         <f t="shared" si="0"/>
         <v>9055.072463768116</v>
       </c>
-      <c r="O27" s="50">
+      <c r="O27" s="46">
         <f>(2000*J27)</f>
         <v>40000</v>
       </c>
-      <c r="P27" s="51">
+      <c r="P27" s="47">
         <f t="shared" si="1"/>
         <v>30944.927536231884</v>
       </c>
-      <c r="Q27" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q27" s="43">
+        <f>P27/J27</f>
         <v>1547.2463768115942</v>
       </c>
     </row>
@@ -5859,15 +5739,15 @@
       <c r="L28" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M28" s="43">
+      <c r="M28" s="42">
         <f t="shared" si="5"/>
         <v>452.75362318840581</v>
       </c>
-      <c r="N28" s="51"/>
-      <c r="O28" s="50"/>
-      <c r="P28" s="51"/>
-      <c r="Q28" s="47">
-        <f t="shared" si="2"/>
+      <c r="N28" s="47"/>
+      <c r="O28" s="46"/>
+      <c r="P28" s="47"/>
+      <c r="Q28" s="43">
+        <f>P28/J28</f>
         <v>0</v>
       </c>
     </row>
@@ -5908,24 +5788,24 @@
       <c r="L29" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M29" s="43">
+      <c r="M29" s="42">
         <f t="shared" si="5"/>
         <v>271.6521739130435</v>
       </c>
-      <c r="N29" s="51">
+      <c r="N29" s="47">
         <f t="shared" si="0"/>
         <v>2716.521739130435</v>
       </c>
-      <c r="O29" s="50">
+      <c r="O29" s="46">
         <f>(1500*J29)</f>
         <v>15000</v>
       </c>
-      <c r="P29" s="51">
+      <c r="P29" s="47">
         <f t="shared" si="1"/>
         <v>12283.478260869564</v>
       </c>
-      <c r="Q29" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q29" s="43">
+        <f>P29/J29</f>
         <v>1228.3478260869565</v>
       </c>
     </row>
@@ -5966,24 +5846,24 @@
       <c r="L30" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="M30" s="43">
+      <c r="M30" s="42">
         <f t="shared" si="5"/>
         <v>452.75362318840581</v>
       </c>
-      <c r="N30" s="51">
+      <c r="N30" s="47">
         <f t="shared" si="0"/>
         <v>2716.521739130435</v>
       </c>
-      <c r="O30" s="50">
+      <c r="O30" s="46">
         <f>(2500*J30)</f>
         <v>15000</v>
       </c>
-      <c r="P30" s="51">
+      <c r="P30" s="47">
         <f t="shared" si="1"/>
         <v>12283.478260869564</v>
       </c>
-      <c r="Q30" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q30" s="43">
+        <f>P30/J30</f>
         <v>2047.246376811594</v>
       </c>
     </row>
@@ -6024,23 +5904,23 @@
       <c r="L31" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M31" s="43">
+      <c r="M31" s="42">
         <f t="shared" si="5"/>
         <v>452.75362318840581</v>
       </c>
-      <c r="N31" s="51">
+      <c r="N31" s="47">
         <f t="shared" si="0"/>
         <v>3169.2753623188405</v>
       </c>
-      <c r="O31" s="50">
+      <c r="O31" s="46">
         <f>(3000*J31)</f>
         <v>21000</v>
       </c>
-      <c r="P31" s="51">
+      <c r="P31" s="47">
         <f>O31-N31</f>
         <v>17830.72463768116</v>
       </c>
-      <c r="Q31" s="47">
+      <c r="Q31" s="43">
         <f>P31/J31</f>
         <v>2547.2463768115945</v>
       </c>
@@ -6082,25 +5962,25 @@
       <c r="L32" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M32" s="43">
+      <c r="M32" s="42">
         <f t="shared" si="5"/>
         <v>271.6521739130435</v>
       </c>
-      <c r="N32" s="51">
+      <c r="N32" s="47">
         <f t="shared" si="0"/>
         <v>6791.3043478260879</v>
       </c>
-      <c r="O32" s="50">
-        <f>(3000*J32)</f>
-        <v>75000</v>
-      </c>
-      <c r="P32" s="51">
+      <c r="O32" s="46">
+        <f>(3500*J32)</f>
+        <v>87500</v>
+      </c>
+      <c r="P32" s="47">
         <f t="shared" si="1"/>
-        <v>68208.695652173919</v>
-      </c>
-      <c r="Q32" s="47">
-        <f t="shared" si="2"/>
-        <v>2728.347826086957</v>
+        <v>80708.695652173919</v>
+      </c>
+      <c r="Q32" s="43">
+        <f>P32/J32</f>
+        <v>3228.347826086957</v>
       </c>
     </row>
     <row r="33" spans="1:17" s="24" customFormat="1" ht="69.95" customHeight="1">
@@ -6140,25 +6020,25 @@
       <c r="L33" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M33" s="43">
+      <c r="M33" s="42">
         <f t="shared" si="5"/>
         <v>226.37681159420291</v>
       </c>
-      <c r="N33" s="51">
+      <c r="N33" s="47">
         <f t="shared" si="0"/>
         <v>5659.420289855073</v>
       </c>
-      <c r="O33" s="50">
-        <f>(3000*J33)</f>
-        <v>75000</v>
-      </c>
-      <c r="P33" s="51">
+      <c r="O33" s="46">
+        <f>(3500*J33)</f>
+        <v>87500</v>
+      </c>
+      <c r="P33" s="47">
         <f t="shared" si="1"/>
-        <v>69340.579710144928</v>
-      </c>
-      <c r="Q33" s="47">
-        <f t="shared" si="2"/>
-        <v>2773.623188405797</v>
+        <v>81840.579710144928</v>
+      </c>
+      <c r="Q33" s="43">
+        <f>P33/J33</f>
+        <v>3273.623188405797</v>
       </c>
     </row>
     <row r="34" spans="1:17" s="24" customFormat="1" ht="81" customHeight="1">
@@ -6198,24 +6078,24 @@
       <c r="L34" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="M34" s="43">
+      <c r="M34" s="42">
         <f t="shared" si="5"/>
         <v>45.275362318840578</v>
       </c>
-      <c r="N34" s="51">
+      <c r="N34" s="47">
         <f t="shared" si="0"/>
         <v>2263.768115942029</v>
       </c>
-      <c r="O34" s="50">
+      <c r="O34" s="46">
         <f>(749*J34)</f>
         <v>37450</v>
       </c>
-      <c r="P34" s="51">
+      <c r="P34" s="47">
         <f t="shared" si="1"/>
         <v>35186.231884057968</v>
       </c>
-      <c r="Q34" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q34" s="43">
+        <f>P34/J34</f>
         <v>703.72463768115938</v>
       </c>
     </row>
@@ -6256,24 +6136,24 @@
       <c r="L35" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="M35" s="43">
+      <c r="M35" s="42">
         <f t="shared" si="5"/>
         <v>405.42028985507244</v>
       </c>
-      <c r="N35" s="51">
+      <c r="N35" s="47">
         <f t="shared" si="0"/>
         <v>16216.811594202898</v>
       </c>
-      <c r="O35" s="50">
+      <c r="O35" s="46">
         <f>(2500*J35)</f>
         <v>100000</v>
       </c>
-      <c r="P35" s="51">
+      <c r="P35" s="47">
         <f t="shared" si="1"/>
         <v>83783.188405797104</v>
       </c>
-      <c r="Q35" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q35" s="43">
+        <f>P35/J35</f>
         <v>2094.5797101449275</v>
       </c>
     </row>
@@ -6314,24 +6194,24 @@
       <c r="L36" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="M36" s="43">
+      <c r="M36" s="42">
         <f t="shared" si="5"/>
         <v>2469.5652173913045</v>
       </c>
-      <c r="N36" s="51">
+      <c r="N36" s="47">
         <f t="shared" si="0"/>
         <v>24695.652173913044</v>
       </c>
-      <c r="O36" s="50">
+      <c r="O36" s="46">
         <f>(10000*J36)</f>
         <v>100000</v>
       </c>
-      <c r="P36" s="51">
+      <c r="P36" s="47">
         <f t="shared" si="1"/>
         <v>75304.34782608696</v>
       </c>
-      <c r="Q36" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q36" s="43">
+        <f>P36/J36</f>
         <v>7530.434782608696</v>
       </c>
     </row>
@@ -6372,24 +6252,24 @@
       <c r="L37" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="M37" s="43">
+      <c r="M37" s="42">
         <f t="shared" si="5"/>
         <v>617.39130434782612</v>
       </c>
-      <c r="N37" s="51">
+      <c r="N37" s="47">
         <f t="shared" si="0"/>
         <v>12347.826086956522</v>
       </c>
-      <c r="O37" s="50">
+      <c r="O37" s="46">
         <f>(4500*J37)</f>
         <v>90000</v>
       </c>
-      <c r="P37" s="51">
+      <c r="P37" s="47">
         <f t="shared" si="1"/>
         <v>77652.173913043473</v>
       </c>
-      <c r="Q37" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q37" s="43">
+        <f>P37/J37</f>
         <v>3882.6086956521735</v>
       </c>
     </row>
@@ -6430,24 +6310,24 @@
       <c r="L38" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="M38" s="43">
+      <c r="M38" s="42">
         <f t="shared" si="5"/>
         <v>5885.797101449275</v>
       </c>
-      <c r="N38" s="51">
+      <c r="N38" s="47">
         <f t="shared" si="0"/>
         <v>11771.59420289855</v>
       </c>
-      <c r="O38" s="50">
+      <c r="O38" s="46">
         <f>(10000*J38)</f>
         <v>20000</v>
       </c>
-      <c r="P38" s="51">
+      <c r="P38" s="47">
         <f t="shared" si="1"/>
         <v>8228.4057971014499</v>
       </c>
-      <c r="Q38" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q38" s="43">
+        <f>P38/J38</f>
         <v>4114.202898550725</v>
       </c>
     </row>
@@ -6488,24 +6368,24 @@
       <c r="L39" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="M39" s="43">
+      <c r="M39" s="42">
         <f t="shared" si="5"/>
         <v>588.5797101449275</v>
       </c>
-      <c r="N39" s="51">
+      <c r="N39" s="47">
         <f t="shared" si="0"/>
         <v>7062.95652173913</v>
       </c>
-      <c r="O39" s="50">
+      <c r="O39" s="46">
         <f>(4000*J39)</f>
         <v>48000</v>
       </c>
-      <c r="P39" s="51">
+      <c r="P39" s="47">
         <f t="shared" si="1"/>
         <v>40937.043478260872</v>
       </c>
-      <c r="Q39" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q39" s="43">
+        <f>P39/J39</f>
         <v>3411.4202898550725</v>
       </c>
     </row>
@@ -6546,24 +6426,24 @@
       <c r="L40" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="M40" s="43">
+      <c r="M40" s="42">
         <f t="shared" si="5"/>
         <v>996.05797101449275</v>
       </c>
-      <c r="N40" s="51">
+      <c r="N40" s="47">
         <f t="shared" si="0"/>
         <v>9960.579710144928</v>
       </c>
-      <c r="O40" s="50">
+      <c r="O40" s="46">
         <f>(5000*J40)</f>
         <v>50000</v>
       </c>
-      <c r="P40" s="51">
+      <c r="P40" s="47">
         <f t="shared" si="1"/>
         <v>40039.420289855072</v>
       </c>
-      <c r="Q40" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q40" s="43">
+        <f>P40/J40</f>
         <v>4003.942028985507</v>
       </c>
     </row>
@@ -6601,27 +6481,27 @@
         <f t="shared" si="8"/>
         <v>4.7826086956521738</v>
       </c>
-      <c r="L41" s="48" t="s">
+      <c r="L41" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="M41" s="50">
+      <c r="M41" s="46">
         <f t="shared" si="5"/>
         <v>679.13043478260863</v>
       </c>
-      <c r="N41" s="51">
+      <c r="N41" s="47">
         <f t="shared" si="0"/>
         <v>6791.3043478260861</v>
       </c>
-      <c r="O41" s="50">
+      <c r="O41" s="46">
         <f>(4000*J41)</f>
         <v>40000</v>
       </c>
-      <c r="P41" s="51">
+      <c r="P41" s="47">
         <f t="shared" si="1"/>
         <v>33208.695652173912</v>
       </c>
-      <c r="Q41" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q41" s="43">
+        <f>P41/J41</f>
         <v>3320.869565217391</v>
       </c>
     </row>
@@ -6659,27 +6539,27 @@
         <f t="shared" si="8"/>
         <v>4.1449275362318838</v>
       </c>
-      <c r="L42" s="48" t="s">
+      <c r="L42" s="44" t="s">
         <v>138</v>
       </c>
-      <c r="M42" s="50">
+      <c r="M42" s="46">
         <f t="shared" si="5"/>
         <v>294.28985507246375</v>
       </c>
-      <c r="N42" s="51">
+      <c r="N42" s="47">
         <f t="shared" si="0"/>
         <v>5885.797101449275</v>
       </c>
-      <c r="O42" s="50">
+      <c r="O42" s="46">
         <f>(3500*J42)</f>
         <v>70000</v>
       </c>
-      <c r="P42" s="51">
+      <c r="P42" s="47">
         <f t="shared" si="1"/>
         <v>64114.202898550728</v>
       </c>
-      <c r="Q42" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q42" s="43">
+        <f>P42/J42</f>
         <v>3205.7101449275365</v>
       </c>
     </row>
@@ -6717,27 +6597,27 @@
         <f t="shared" si="8"/>
         <v>1.2753623188405796</v>
       </c>
-      <c r="L43" s="48" t="s">
+      <c r="L43" s="44" t="s">
         <v>134</v>
       </c>
-      <c r="M43" s="50">
+      <c r="M43" s="46">
         <f t="shared" si="5"/>
         <v>45.275362318840578</v>
       </c>
-      <c r="N43" s="51">
+      <c r="N43" s="47">
         <f t="shared" si="0"/>
         <v>1811.014492753623</v>
       </c>
-      <c r="O43" s="50">
+      <c r="O43" s="46">
         <f>(240*J43)</f>
         <v>9600</v>
       </c>
-      <c r="P43" s="51">
+      <c r="P43" s="47">
         <f t="shared" si="1"/>
         <v>7788.985507246377</v>
       </c>
-      <c r="Q43" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q43" s="43">
+        <f>P43/J43</f>
         <v>194.72463768115944</v>
       </c>
     </row>
@@ -6775,27 +6655,27 @@
         <f t="shared" si="8"/>
         <v>30.434782608695652</v>
       </c>
-      <c r="L44" s="48" t="s">
+      <c r="L44" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="M44" s="50">
+      <c r="M44" s="46">
         <f t="shared" si="5"/>
         <v>43217.391304347824</v>
       </c>
-      <c r="N44" s="51">
+      <c r="N44" s="47">
         <f t="shared" si="0"/>
         <v>43217.391304347824</v>
       </c>
-      <c r="O44" s="50">
+      <c r="O44" s="46">
         <f t="shared" si="6"/>
         <v>20000</v>
       </c>
-      <c r="P44" s="51">
+      <c r="P44" s="47">
         <f t="shared" si="1"/>
         <v>-23217.391304347824</v>
       </c>
-      <c r="Q44" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q44" s="43">
+        <f>P44/J44</f>
         <v>-23217.391304347824</v>
       </c>
     </row>
@@ -6834,24 +6714,24 @@
         <v>3.1565217391304348</v>
       </c>
       <c r="L45" s="29"/>
-      <c r="M45" s="50">
+      <c r="M45" s="46">
         <f t="shared" si="5"/>
         <v>1494.086956521739</v>
       </c>
-      <c r="N45" s="51">
+      <c r="N45" s="47">
         <f t="shared" si="0"/>
         <v>4482.260869565217</v>
       </c>
-      <c r="O45" s="50">
+      <c r="O45" s="46">
         <f>(4500*J45)</f>
         <v>13500</v>
       </c>
-      <c r="P45" s="51">
+      <c r="P45" s="47">
         <f t="shared" si="1"/>
         <v>9017.7391304347839</v>
       </c>
-      <c r="Q45" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q45" s="43">
+        <f>P45/J45</f>
         <v>3005.9130434782614</v>
       </c>
     </row>
@@ -6889,27 +6769,27 @@
         <f t="shared" si="8"/>
         <v>3.1565217391304348</v>
       </c>
-      <c r="L46" s="48" t="s">
+      <c r="L46" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="M46" s="50">
+      <c r="M46" s="46">
         <f t="shared" si="5"/>
         <v>1494.086956521739</v>
       </c>
-      <c r="N46" s="51">
+      <c r="N46" s="47">
         <f t="shared" si="0"/>
         <v>4482.260869565217</v>
       </c>
-      <c r="O46" s="50">
+      <c r="O46" s="46">
         <f>(4500*J46)</f>
         <v>13500</v>
       </c>
-      <c r="P46" s="51">
+      <c r="P46" s="47">
         <f t="shared" si="1"/>
         <v>9017.7391304347839</v>
       </c>
-      <c r="Q46" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q46" s="43">
+        <f>P46/J46</f>
         <v>3005.9130434782614</v>
       </c>
     </row>
@@ -6947,27 +6827,27 @@
         <f t="shared" si="8"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="L47" s="48" t="s">
+      <c r="L47" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M47" s="50">
+      <c r="M47" s="46">
         <f t="shared" si="5"/>
         <v>45.275362318840578</v>
       </c>
-      <c r="N47" s="51">
+      <c r="N47" s="47">
         <f t="shared" si="0"/>
         <v>1358.2608695652173</v>
       </c>
-      <c r="O47" s="50">
+      <c r="O47" s="46">
         <f>(150*J47)</f>
         <v>4500</v>
       </c>
-      <c r="P47" s="51">
+      <c r="P47" s="47">
         <f t="shared" si="1"/>
         <v>3141.739130434783</v>
       </c>
-      <c r="Q47" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q47" s="43">
+        <f>P47/J47</f>
         <v>104.72463768115944</v>
       </c>
     </row>
@@ -7005,27 +6885,27 @@
         <f t="shared" si="8"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="L48" s="48" t="s">
+      <c r="L48" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M48" s="50">
+      <c r="M48" s="46">
         <f t="shared" si="5"/>
         <v>45.275362318840578</v>
       </c>
-      <c r="N48" s="51">
+      <c r="N48" s="47">
         <f t="shared" si="0"/>
         <v>1358.2608695652173</v>
       </c>
-      <c r="O48" s="50">
+      <c r="O48" s="46">
         <f>(240*J48)</f>
         <v>7200</v>
       </c>
-      <c r="P48" s="51">
+      <c r="P48" s="47">
         <f t="shared" si="1"/>
         <v>5841.739130434783</v>
       </c>
-      <c r="Q48" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q48" s="43">
+        <f>P48/J48</f>
         <v>194.72463768115944</v>
       </c>
     </row>
@@ -7055,7 +6935,7 @@
         <f t="shared" si="7"/>
         <v>1.3043478260869565E-2</v>
       </c>
-      <c r="I49" s="44"/>
+      <c r="I49" s="49"/>
       <c r="J49" s="22">
         <v>50</v>
       </c>
@@ -7063,27 +6943,27 @@
         <f t="shared" si="8"/>
         <v>0.65217391304347827</v>
       </c>
-      <c r="L49" s="48" t="s">
+      <c r="L49" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M49" s="50">
+      <c r="M49" s="46">
         <f t="shared" si="5"/>
         <v>18.521739130434781</v>
       </c>
-      <c r="N49" s="51">
+      <c r="N49" s="47">
         <f t="shared" si="0"/>
         <v>926.08695652173901</v>
       </c>
-      <c r="O49" s="50">
+      <c r="O49" s="46">
         <f>(100*J49)</f>
         <v>5000</v>
       </c>
-      <c r="P49" s="51">
+      <c r="P49" s="47">
         <f t="shared" si="1"/>
         <v>4073.913043478261</v>
       </c>
-      <c r="Q49" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q49" s="43">
+        <f>P49/J49</f>
         <v>81.478260869565219</v>
       </c>
     </row>
@@ -7113,7 +6993,7 @@
         <f t="shared" si="7"/>
         <v>8.6956521739130418E-3</v>
       </c>
-      <c r="I50" s="45"/>
+      <c r="I50" s="50"/>
       <c r="J50" s="22">
         <v>50</v>
       </c>
@@ -7121,27 +7001,27 @@
         <f t="shared" si="8"/>
         <v>0.43478260869565211</v>
       </c>
-      <c r="L50" s="48" t="s">
+      <c r="L50" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M50" s="50">
+      <c r="M50" s="46">
         <f t="shared" si="5"/>
         <v>12.34782608695652</v>
       </c>
-      <c r="N50" s="51">
+      <c r="N50" s="47">
         <f t="shared" si="0"/>
         <v>617.39130434782601</v>
       </c>
-      <c r="O50" s="50">
+      <c r="O50" s="46">
         <f>(150*J50)</f>
         <v>7500</v>
       </c>
-      <c r="P50" s="51">
+      <c r="P50" s="47">
         <f t="shared" si="1"/>
         <v>6882.608695652174</v>
       </c>
-      <c r="Q50" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q50" s="43">
+        <f>P50/J50</f>
         <v>137.65217391304347</v>
       </c>
     </row>
@@ -7171,7 +7051,7 @@
         <f t="shared" si="7"/>
         <v>2.8985507246376812E-2</v>
       </c>
-      <c r="I51" s="46"/>
+      <c r="I51" s="51"/>
       <c r="J51" s="22">
         <v>50</v>
       </c>
@@ -7179,27 +7059,27 @@
         <f t="shared" si="8"/>
         <v>1.4492753623188406</v>
       </c>
-      <c r="L51" s="48" t="s">
+      <c r="L51" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M51" s="50">
+      <c r="M51" s="46">
         <f t="shared" si="5"/>
         <v>41.159420289855071</v>
       </c>
-      <c r="N51" s="51">
+      <c r="N51" s="47">
         <f t="shared" si="0"/>
         <v>2057.9710144927535</v>
       </c>
-      <c r="O51" s="50">
+      <c r="O51" s="46">
         <f>(150*J51)</f>
         <v>7500</v>
       </c>
-      <c r="P51" s="51">
+      <c r="P51" s="47">
         <f t="shared" si="1"/>
         <v>5442.028985507246</v>
       </c>
-      <c r="Q51" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q51" s="43">
+        <f>P51/J51</f>
         <v>108.84057971014492</v>
       </c>
     </row>
@@ -7229,7 +7109,7 @@
         <f t="shared" si="7"/>
         <v>0.9565217391304347</v>
       </c>
-      <c r="I52" s="44"/>
+      <c r="I52" s="49"/>
       <c r="J52" s="22">
         <v>10</v>
       </c>
@@ -7237,27 +7117,27 @@
         <f t="shared" si="8"/>
         <v>9.5652173913043477</v>
       </c>
-      <c r="L52" s="48" t="s">
+      <c r="L52" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M52" s="50">
+      <c r="M52" s="46">
         <f t="shared" si="5"/>
         <v>1358.2608695652173</v>
       </c>
-      <c r="N52" s="51">
+      <c r="N52" s="47">
         <f>M52*J52</f>
         <v>13582.608695652172</v>
       </c>
-      <c r="O52" s="50">
+      <c r="O52" s="46">
         <f>(5000*J52)</f>
         <v>50000</v>
       </c>
-      <c r="P52" s="51">
+      <c r="P52" s="47">
         <f t="shared" si="1"/>
         <v>36417.391304347824</v>
       </c>
-      <c r="Q52" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q52" s="43">
+        <f>P52/J52</f>
         <v>3641.7391304347825</v>
       </c>
     </row>
@@ -7287,7 +7167,7 @@
         <f t="shared" si="7"/>
         <v>1.4347826086956521</v>
       </c>
-      <c r="I53" s="46"/>
+      <c r="I53" s="51"/>
       <c r="J53" s="22">
         <v>5</v>
       </c>
@@ -7295,27 +7175,27 @@
         <f t="shared" si="8"/>
         <v>7.1739130434782608</v>
       </c>
-      <c r="L53" s="48" t="s">
+      <c r="L53" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M53" s="50">
+      <c r="M53" s="46">
         <f t="shared" si="5"/>
         <v>2037.391304347826</v>
       </c>
-      <c r="N53" s="51">
+      <c r="N53" s="47">
         <f t="shared" si="0"/>
         <v>10186.95652173913</v>
       </c>
-      <c r="O53" s="50">
+      <c r="O53" s="46">
         <f>(6000*J53)</f>
         <v>30000</v>
       </c>
-      <c r="P53" s="51">
+      <c r="P53" s="47">
         <f t="shared" si="1"/>
         <v>19813.043478260872</v>
       </c>
-      <c r="Q53" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q53" s="43">
+        <f>P53/J53</f>
         <v>3962.6086956521744</v>
       </c>
     </row>
@@ -7353,27 +7233,27 @@
         <f t="shared" si="8"/>
         <v>10.760869565217391</v>
       </c>
-      <c r="L54" s="48" t="s">
+      <c r="L54" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M54" s="50">
+      <c r="M54" s="46">
         <f t="shared" si="5"/>
         <v>3056.086956521739</v>
       </c>
-      <c r="N54" s="51">
-        <f t="shared" si="0"/>
+      <c r="N54" s="47">
+        <f>M54*J54</f>
         <v>15280.434782608696</v>
       </c>
-      <c r="O54" s="50">
+      <c r="O54" s="46">
         <f>(7000*J54)</f>
         <v>35000</v>
       </c>
-      <c r="P54" s="51">
+      <c r="P54" s="47">
         <f t="shared" si="1"/>
         <v>19719.565217391304</v>
       </c>
-      <c r="Q54" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q54" s="43">
+        <f>P54/J54</f>
         <v>3943.913043478261</v>
       </c>
     </row>
@@ -7411,27 +7291,27 @@
         <f t="shared" si="8"/>
         <v>15.942028985507246</v>
       </c>
-      <c r="L55" s="48" t="s">
+      <c r="L55" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M55" s="50">
+      <c r="M55" s="46">
         <f t="shared" si="5"/>
         <v>4527.536231884058</v>
       </c>
-      <c r="N55" s="51">
+      <c r="N55" s="47">
         <f t="shared" si="0"/>
         <v>22637.681159420288</v>
       </c>
-      <c r="O55" s="50">
+      <c r="O55" s="46">
         <f>(9000*J55)</f>
         <v>45000</v>
       </c>
-      <c r="P55" s="51">
+      <c r="P55" s="47">
         <f t="shared" si="1"/>
         <v>22362.318840579712</v>
       </c>
-      <c r="Q55" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q55" s="43">
+        <f>P55/J55</f>
         <v>4472.463768115942</v>
       </c>
     </row>
@@ -7469,27 +7349,27 @@
         <f t="shared" si="8"/>
         <v>1.2318840579710146</v>
       </c>
-      <c r="L56" s="48" t="s">
+      <c r="L56" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M56" s="50">
+      <c r="M56" s="46">
         <f t="shared" si="5"/>
         <v>34.985507246376812</v>
       </c>
-      <c r="N56" s="51">
+      <c r="N56" s="47">
         <f t="shared" si="0"/>
         <v>1749.2753623188405</v>
       </c>
-      <c r="O56" s="50">
+      <c r="O56" s="46">
         <f>(2000*J56)</f>
         <v>100000</v>
       </c>
-      <c r="P56" s="51">
+      <c r="P56" s="47">
         <f t="shared" si="1"/>
         <v>98250.724637681153</v>
       </c>
-      <c r="Q56" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q56" s="43">
+        <f>P56/J56</f>
         <v>1965.014492753623</v>
       </c>
     </row>
@@ -7527,27 +7407,27 @@
         <f t="shared" si="8"/>
         <v>12.753623188405799</v>
       </c>
-      <c r="L57" s="48" t="s">
+      <c r="L57" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M57" s="50">
+      <c r="M57" s="46">
         <f t="shared" si="5"/>
         <v>1811.0144927536232</v>
       </c>
-      <c r="N57" s="51">
+      <c r="N57" s="47">
         <f t="shared" si="0"/>
         <v>18110.144927536232</v>
       </c>
-      <c r="O57" s="50">
+      <c r="O57" s="46">
         <f>(6000*J57)</f>
         <v>60000</v>
       </c>
-      <c r="P57" s="51">
+      <c r="P57" s="47">
         <f t="shared" si="1"/>
         <v>41889.855072463768</v>
       </c>
-      <c r="Q57" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q57" s="43">
+        <f>P57/J57</f>
         <v>4188.985507246377</v>
       </c>
     </row>
@@ -7583,27 +7463,27 @@
         <f t="shared" si="8"/>
         <v>3.1884057971014492</v>
       </c>
-      <c r="L58" s="48" t="s">
+      <c r="L58" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M58" s="50">
+      <c r="M58" s="46">
         <f t="shared" si="5"/>
         <v>90.550724637681157</v>
       </c>
-      <c r="N58" s="51">
+      <c r="N58" s="47">
         <f>M58*J58</f>
         <v>4527.536231884058</v>
       </c>
-      <c r="O58" s="50">
+      <c r="O58" s="46">
         <f>(250*J58)</f>
         <v>12500</v>
       </c>
-      <c r="P58" s="51">
+      <c r="P58" s="47">
         <f t="shared" si="1"/>
         <v>7972.463768115942</v>
       </c>
-      <c r="Q58" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q58" s="43">
+        <f>P58/J58</f>
         <v>159.44927536231884</v>
       </c>
     </row>
@@ -7635,27 +7515,27 @@
         <f t="shared" si="8"/>
         <v>2.043478260869565</v>
       </c>
-      <c r="L59" s="48" t="s">
+      <c r="L59" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M59" s="50">
+      <c r="M59" s="46">
         <f t="shared" si="5"/>
         <v>290.17391304347825</v>
       </c>
-      <c r="N59" s="51">
+      <c r="N59" s="47">
         <f t="shared" si="0"/>
         <v>2901.7391304347825</v>
       </c>
-      <c r="O59" s="50">
+      <c r="O59" s="46">
         <f>(750*J59)</f>
         <v>7500</v>
       </c>
-      <c r="P59" s="51">
+      <c r="P59" s="47">
         <f t="shared" si="1"/>
         <v>4598.2608695652179</v>
       </c>
-      <c r="Q59" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q59" s="43">
+        <f>P59/J59</f>
         <v>459.82608695652181</v>
       </c>
     </row>
@@ -7687,27 +7567,27 @@
         <f t="shared" si="8"/>
         <v>2.72463768115942</v>
       </c>
-      <c r="L60" s="48" t="s">
+      <c r="L60" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M60" s="50">
+      <c r="M60" s="46">
         <f t="shared" si="5"/>
         <v>386.89855072463763</v>
       </c>
-      <c r="N60" s="51">
+      <c r="N60" s="47">
         <f t="shared" si="0"/>
         <v>3868.9855072463761</v>
       </c>
-      <c r="O60" s="50">
+      <c r="O60" s="46">
         <f>(920*J60)</f>
         <v>9200</v>
       </c>
-      <c r="P60" s="51">
+      <c r="P60" s="47">
         <f t="shared" si="1"/>
         <v>5331.0144927536239</v>
       </c>
-      <c r="Q60" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q60" s="43">
+        <f>P60/J60</f>
         <v>533.10144927536237</v>
       </c>
     </row>
@@ -7741,27 +7621,27 @@
         <f t="shared" si="8"/>
         <v>2.9130434782608687</v>
       </c>
-      <c r="L61" s="48" t="s">
+      <c r="L61" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M61" s="50">
+      <c r="M61" s="46">
         <f t="shared" si="5"/>
         <v>413.65217391304338</v>
       </c>
-      <c r="N61" s="51">
+      <c r="N61" s="47">
         <f t="shared" si="0"/>
         <v>4136.5217391304341</v>
       </c>
-      <c r="O61" s="50">
+      <c r="O61" s="46">
         <f>(1471*J61)</f>
         <v>14710</v>
       </c>
-      <c r="P61" s="51">
+      <c r="P61" s="47">
         <f t="shared" si="1"/>
         <v>10573.478260869566</v>
       </c>
-      <c r="Q61" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q61" s="43">
+        <f>P61/J61</f>
         <v>1057.3478260869565</v>
       </c>
     </row>
@@ -7793,27 +7673,27 @@
         <f t="shared" si="8"/>
         <v>2.043478260869565</v>
       </c>
-      <c r="L62" s="48" t="s">
+      <c r="L62" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M62" s="50">
+      <c r="M62" s="46">
         <f t="shared" si="5"/>
         <v>290.17391304347825</v>
       </c>
-      <c r="N62" s="51">
+      <c r="N62" s="47">
         <f t="shared" si="0"/>
         <v>2901.7391304347825</v>
       </c>
-      <c r="O62" s="50">
+      <c r="O62" s="46">
         <f>(750*J62)</f>
         <v>7500</v>
       </c>
-      <c r="P62" s="51">
+      <c r="P62" s="47">
         <f t="shared" si="1"/>
         <v>4598.2608695652179</v>
       </c>
-      <c r="Q62" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q62" s="43">
+        <f>P62/J62</f>
         <v>459.82608695652181</v>
       </c>
     </row>
@@ -7845,27 +7725,27 @@
         <f t="shared" si="8"/>
         <v>2.72463768115942</v>
       </c>
-      <c r="L63" s="48" t="s">
+      <c r="L63" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M63" s="50">
+      <c r="M63" s="46">
         <f t="shared" si="5"/>
         <v>386.89855072463763</v>
       </c>
-      <c r="N63" s="51">
+      <c r="N63" s="47">
         <f t="shared" si="0"/>
         <v>3868.9855072463761</v>
       </c>
-      <c r="O63" s="50">
+      <c r="O63" s="46">
         <f>(996*J63)</f>
         <v>9960</v>
       </c>
-      <c r="P63" s="51">
+      <c r="P63" s="47">
         <f t="shared" si="1"/>
         <v>6091.0144927536239</v>
       </c>
-      <c r="Q63" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q63" s="43">
+        <f>P63/J63</f>
         <v>609.10144927536237</v>
       </c>
     </row>
@@ -7897,27 +7777,27 @@
         <f t="shared" si="8"/>
         <v>2.9130434782608687</v>
       </c>
-      <c r="L64" s="48" t="s">
+      <c r="L64" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="M64" s="50">
+      <c r="M64" s="46">
         <f t="shared" si="5"/>
         <v>413.65217391304338</v>
       </c>
-      <c r="N64" s="51">
+      <c r="N64" s="47">
         <f t="shared" si="0"/>
         <v>4136.5217391304341</v>
       </c>
-      <c r="O64" s="50">
+      <c r="O64" s="46">
         <f>(1471*J64)</f>
         <v>14710</v>
       </c>
-      <c r="P64" s="51">
+      <c r="P64" s="47">
         <f t="shared" si="1"/>
         <v>10573.478260869566</v>
       </c>
-      <c r="Q64" s="47">
-        <f t="shared" si="2"/>
+      <c r="Q64" s="43">
+        <f>P64/J64</f>
         <v>1057.3478260869565</v>
       </c>
     </row>
@@ -7947,24 +7827,24 @@
         <f t="shared" si="8"/>
         <v>5.1014492753623184</v>
       </c>
-      <c r="L65" s="49"/>
-      <c r="M65" s="50">
+      <c r="L65" s="45"/>
+      <c r="M65" s="46">
         <f t="shared" si="5"/>
         <v>181.10144927536231</v>
       </c>
-      <c r="N65" s="51">
+      <c r="N65" s="47">
         <f t="shared" si="0"/>
         <v>7244.0579710144921</v>
       </c>
-      <c r="O65" s="50">
+      <c r="O65" s="46">
         <f>(1000*J65)</f>
         <v>40000</v>
       </c>
-      <c r="P65" s="51">
+      <c r="P65" s="47">
         <f t="shared" si="1"/>
         <v>32755.942028985508</v>
       </c>
-      <c r="Q65" s="47">
+      <c r="Q65" s="43">
         <f>P65/J65</f>
         <v>818.89855072463774</v>
       </c>
@@ -7995,24 +7875,24 @@
         <f t="shared" si="8"/>
         <v>7.2463768115942031</v>
       </c>
-      <c r="L66" s="49"/>
-      <c r="M66" s="50">
+      <c r="L66" s="45"/>
+      <c r="M66" s="46">
         <f t="shared" si="5"/>
         <v>514.49275362318838</v>
       </c>
-      <c r="N66" s="51">
-        <f t="shared" ref="N66:N76" si="9">M66*J66</f>
+      <c r="N66" s="47">
+        <f t="shared" ref="N66:N75" si="9">M66*J66</f>
         <v>10289.855072463768</v>
       </c>
-      <c r="O66" s="50">
+      <c r="O66" s="46">
         <f>(1500*J66)</f>
         <v>30000</v>
       </c>
-      <c r="P66" s="51">
-        <f t="shared" ref="P66:P76" si="10">O66-N66</f>
+      <c r="P66" s="47">
+        <f t="shared" ref="P66:P75" si="10">O66-N66</f>
         <v>19710.144927536232</v>
       </c>
-      <c r="Q66" s="47">
+      <c r="Q66" s="43">
         <f t="shared" ref="Q66:Q76" si="11">P66/J66</f>
         <v>985.50724637681162</v>
       </c>
@@ -8043,24 +7923,24 @@
         <f t="shared" si="8"/>
         <v>3.6231884057971016</v>
       </c>
-      <c r="L67" s="49"/>
-      <c r="M67" s="50">
+      <c r="L67" s="45"/>
+      <c r="M67" s="46">
         <f>1420*H67</f>
         <v>1028.9855072463768</v>
       </c>
-      <c r="N67" s="51">
+      <c r="N67" s="47">
         <f t="shared" si="9"/>
         <v>5144.927536231884</v>
       </c>
-      <c r="O67" s="50">
+      <c r="O67" s="46">
         <f>(2500*J67)</f>
         <v>12500</v>
       </c>
-      <c r="P67" s="51">
+      <c r="P67" s="47">
         <f t="shared" si="10"/>
         <v>7355.072463768116</v>
       </c>
-      <c r="Q67" s="47">
+      <c r="Q67" s="43">
         <f t="shared" si="11"/>
         <v>1471.0144927536232</v>
       </c>
@@ -8091,24 +7971,24 @@
         <f t="shared" si="8"/>
         <v>14.492753623188404</v>
       </c>
-      <c r="L68" s="49"/>
-      <c r="M68" s="50">
+      <c r="L68" s="45"/>
+      <c r="M68" s="46">
         <f t="shared" ref="M68:M80" si="12">1420*H68</f>
         <v>10289.855072463768</v>
       </c>
-      <c r="N68" s="51">
+      <c r="N68" s="47">
         <f t="shared" si="9"/>
         <v>20579.710144927536</v>
       </c>
-      <c r="O68" s="50">
+      <c r="O68" s="46">
         <f>(100000*J68)</f>
         <v>200000</v>
       </c>
-      <c r="P68" s="51">
+      <c r="P68" s="47">
         <f t="shared" si="10"/>
         <v>179420.28985507245</v>
       </c>
-      <c r="Q68" s="47">
+      <c r="Q68" s="43">
         <f t="shared" si="11"/>
         <v>89710.144927536225</v>
       </c>
@@ -8139,24 +8019,24 @@
         <f t="shared" si="8"/>
         <v>6.0579710144927539</v>
       </c>
-      <c r="L69" s="49"/>
-      <c r="M69" s="50">
+      <c r="L69" s="45"/>
+      <c r="M69" s="46">
         <f t="shared" si="12"/>
         <v>430.1159420289855</v>
       </c>
-      <c r="N69" s="51">
+      <c r="N69" s="47">
         <f t="shared" si="9"/>
         <v>8602.31884057971</v>
       </c>
-      <c r="O69" s="50">
+      <c r="O69" s="46">
         <f>(2000*J69)</f>
         <v>40000</v>
       </c>
-      <c r="P69" s="51">
+      <c r="P69" s="47">
         <f t="shared" si="10"/>
         <v>31397.681159420288</v>
       </c>
-      <c r="Q69" s="47">
+      <c r="Q69" s="43">
         <f t="shared" si="11"/>
         <v>1569.8840579710145</v>
       </c>
@@ -8187,24 +8067,24 @@
         <f t="shared" ref="K70:K75" si="14">J70*H70</f>
         <v>0.94202898550724645</v>
       </c>
-      <c r="L70" s="49"/>
-      <c r="M70" s="50">
+      <c r="L70" s="45"/>
+      <c r="M70" s="46">
         <f t="shared" si="12"/>
         <v>26.753623188405797</v>
       </c>
-      <c r="N70" s="51">
+      <c r="N70" s="47">
         <f t="shared" si="9"/>
         <v>1337.6811594202898</v>
       </c>
-      <c r="O70" s="50">
+      <c r="O70" s="46">
         <f>(200*J70)</f>
         <v>10000</v>
       </c>
-      <c r="P70" s="51">
+      <c r="P70" s="47">
         <f t="shared" si="10"/>
         <v>8662.31884057971</v>
       </c>
-      <c r="Q70" s="47">
+      <c r="Q70" s="43">
         <f t="shared" si="11"/>
         <v>173.24637681159419</v>
       </c>
@@ -8235,24 +8115,24 @@
         <f t="shared" si="14"/>
         <v>19.130434782608695</v>
       </c>
-      <c r="L71" s="49"/>
-      <c r="M71" s="50">
+      <c r="L71" s="45"/>
+      <c r="M71" s="46">
         <f t="shared" si="12"/>
         <v>2716.5217391304345</v>
       </c>
-      <c r="N71" s="51">
+      <c r="N71" s="47">
         <f t="shared" si="9"/>
         <v>27165.217391304344</v>
       </c>
-      <c r="O71" s="50">
+      <c r="O71" s="46">
         <f>(7000*J71)</f>
         <v>70000</v>
       </c>
-      <c r="P71" s="51">
+      <c r="P71" s="47">
         <f t="shared" si="10"/>
         <v>42834.782608695656</v>
       </c>
-      <c r="Q71" s="47">
+      <c r="Q71" s="43">
         <f t="shared" si="11"/>
         <v>4283.4782608695659</v>
       </c>
@@ -8283,24 +8163,24 @@
         <f t="shared" si="14"/>
         <v>5.579710144927537</v>
       </c>
-      <c r="L72" s="49"/>
-      <c r="M72" s="50">
+      <c r="L72" s="45"/>
+      <c r="M72" s="46">
         <f t="shared" si="12"/>
         <v>792.31884057971024</v>
       </c>
-      <c r="N72" s="51">
+      <c r="N72" s="47">
         <f t="shared" si="9"/>
         <v>7923.188405797102</v>
       </c>
-      <c r="O72" s="50">
+      <c r="O72" s="46">
         <f>(1999*J72)</f>
         <v>19990</v>
       </c>
-      <c r="P72" s="51">
+      <c r="P72" s="47">
         <f>O72-N72</f>
         <v>12066.811594202898</v>
       </c>
-      <c r="Q72" s="47">
+      <c r="Q72" s="43">
         <f t="shared" si="11"/>
         <v>1206.6811594202898</v>
       </c>
@@ -8331,24 +8211,24 @@
         <f t="shared" si="14"/>
         <v>7.4637681159420293</v>
       </c>
-      <c r="L73" s="49"/>
-      <c r="M73" s="50">
+      <c r="L73" s="45"/>
+      <c r="M73" s="46">
         <f t="shared" si="12"/>
         <v>1059.855072463768</v>
       </c>
-      <c r="N73" s="51">
+      <c r="N73" s="47">
         <f t="shared" si="9"/>
         <v>10598.55072463768</v>
       </c>
-      <c r="O73" s="50">
+      <c r="O73" s="46">
         <f>(4000*J73)</f>
         <v>40000</v>
       </c>
-      <c r="P73" s="51">
+      <c r="P73" s="47">
         <f t="shared" si="10"/>
         <v>29401.44927536232</v>
       </c>
-      <c r="Q73" s="47">
+      <c r="Q73" s="43">
         <f t="shared" si="11"/>
         <v>2940.144927536232</v>
       </c>
@@ -8379,24 +8259,24 @@
         <f t="shared" si="14"/>
         <v>11.956521739130434</v>
       </c>
-      <c r="L74" s="49"/>
-      <c r="M74" s="50">
+      <c r="L74" s="45"/>
+      <c r="M74" s="46">
         <f t="shared" si="12"/>
         <v>1697.8260869565217</v>
       </c>
-      <c r="N74" s="51">
+      <c r="N74" s="47">
         <f t="shared" si="9"/>
         <v>16978.260869565216</v>
       </c>
-      <c r="O74" s="50">
+      <c r="O74" s="46">
         <f>(5000*J74)</f>
         <v>50000</v>
       </c>
-      <c r="P74" s="51">
+      <c r="P74" s="47">
         <f t="shared" si="10"/>
         <v>33021.739130434784</v>
       </c>
-      <c r="Q74" s="47">
+      <c r="Q74" s="43">
         <f t="shared" si="11"/>
         <v>3302.1739130434785</v>
       </c>
@@ -8427,24 +8307,24 @@
         <f t="shared" si="14"/>
         <v>1.2753623188405796</v>
       </c>
-      <c r="L75" s="49"/>
-      <c r="M75" s="50">
+      <c r="L75" s="45"/>
+      <c r="M75" s="46">
         <f t="shared" si="12"/>
         <v>90.550724637681157</v>
       </c>
-      <c r="N75" s="51">
+      <c r="N75" s="47">
         <f t="shared" si="9"/>
         <v>1811.014492753623</v>
       </c>
-      <c r="O75" s="50">
+      <c r="O75" s="46">
         <f>(500*J75)</f>
         <v>10000</v>
       </c>
-      <c r="P75" s="51">
+      <c r="P75" s="47">
         <f t="shared" si="10"/>
         <v>8188.985507246377</v>
       </c>
-      <c r="Q75" s="47">
+      <c r="Q75" s="43">
         <f t="shared" si="11"/>
         <v>409.44927536231887</v>
       </c>
@@ -8475,15 +8355,15 @@
       <c r="K76" s="23">
         <v>29.8571428571429</v>
       </c>
-      <c r="L76" s="49"/>
-      <c r="M76" s="50">
+      <c r="L76" s="45"/>
+      <c r="M76" s="46">
         <f t="shared" si="12"/>
         <v>42397.142857142921</v>
       </c>
-      <c r="N76" s="51"/>
-      <c r="O76" s="50"/>
-      <c r="P76" s="51"/>
-      <c r="Q76" s="47">
+      <c r="N76" s="47"/>
+      <c r="O76" s="46"/>
+      <c r="P76" s="47"/>
+      <c r="Q76" s="43">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -8515,24 +8395,24 @@
         <f>H77*J77</f>
         <v>33.624000000000002</v>
       </c>
-      <c r="L77" s="49"/>
-      <c r="M77" s="50">
+      <c r="L77" s="45"/>
+      <c r="M77" s="46">
         <f>1420*H77</f>
         <v>11936.52</v>
       </c>
-      <c r="N77" s="51">
+      <c r="N77" s="47">
         <f>M77*J77</f>
         <v>47746.080000000002</v>
       </c>
-      <c r="O77" s="50">
+      <c r="O77" s="46">
         <f>(20000*J77)</f>
         <v>80000</v>
       </c>
-      <c r="P77" s="51">
+      <c r="P77" s="47">
         <f>O77-N77</f>
         <v>32253.919999999998</v>
       </c>
-      <c r="Q77" s="47">
+      <c r="Q77" s="43">
         <f>P77/J77</f>
         <v>8063.48</v>
       </c>
@@ -8562,25 +8442,25 @@
         <f>J78*H78</f>
         <v>4.3849999999999998</v>
       </c>
-      <c r="L78" s="49"/>
-      <c r="M78" s="50">
+      <c r="L78" s="45"/>
+      <c r="M78" s="46">
         <f t="shared" si="12"/>
         <v>1245.3399999999999</v>
       </c>
-      <c r="N78" s="51">
-        <f t="shared" ref="N78:N80" si="15">M78*J78</f>
+      <c r="N78" s="47">
+        <f t="shared" ref="N78:N79" si="15">M78*J78</f>
         <v>6226.7</v>
       </c>
-      <c r="O78" s="50">
+      <c r="O78" s="46">
         <f>(3000*J78)</f>
         <v>15000</v>
       </c>
-      <c r="P78" s="51">
-        <f t="shared" ref="P78:P80" si="16">O78-N78</f>
+      <c r="P78" s="47">
+        <f t="shared" ref="P78:P79" si="16">O78-N78</f>
         <v>8773.2999999999993</v>
       </c>
-      <c r="Q78" s="47">
-        <f t="shared" ref="Q78:Q80" si="17">P78/J78</f>
+      <c r="Q78" s="43">
+        <f t="shared" ref="Q78:Q79" si="17">P78/J78</f>
         <v>1754.6599999999999</v>
       </c>
     </row>
@@ -8609,64 +8489,64 @@
         <f>H79*J79</f>
         <v>17.535</v>
       </c>
-      <c r="L79" s="49"/>
-      <c r="M79" s="50">
+      <c r="L79" s="45"/>
+      <c r="M79" s="46">
         <f t="shared" si="12"/>
         <v>4979.9400000000005</v>
       </c>
-      <c r="N79" s="51">
+      <c r="N79" s="47">
         <f t="shared" si="15"/>
         <v>24899.700000000004</v>
       </c>
-      <c r="O79" s="50">
+      <c r="O79" s="46">
         <f>(8000*J79)</f>
         <v>40000</v>
       </c>
-      <c r="P79" s="51">
+      <c r="P79" s="47">
         <f t="shared" si="16"/>
         <v>15100.299999999996</v>
       </c>
-      <c r="Q79" s="47">
+      <c r="Q79" s="43">
         <f t="shared" si="17"/>
         <v>3020.059999999999</v>
       </c>
     </row>
     <row r="80" spans="1:17" s="24" customFormat="1" ht="72.95" customHeight="1">
-      <c r="A80" s="30"/>
-      <c r="B80" s="32"/>
-      <c r="C80" s="24" t="s">
+      <c r="A80" s="61"/>
+      <c r="B80" s="62"/>
+      <c r="C80" s="63" t="s">
         <v>207</v>
       </c>
-      <c r="D80" s="38" t="s">
+      <c r="D80" s="64" t="s">
         <v>208</v>
       </c>
-      <c r="E80" s="38"/>
-      <c r="F80" s="16" t="s">
+      <c r="E80" s="64"/>
+      <c r="F80" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="G80" s="36"/>
-      <c r="H80" s="42">
+      <c r="G80" s="66"/>
+      <c r="H80" s="67">
         <v>5.87</v>
       </c>
-      <c r="I80" s="30"/>
-      <c r="J80" s="31">
+      <c r="I80" s="61"/>
+      <c r="J80" s="68">
         <v>1</v>
       </c>
-      <c r="K80" s="23">
+      <c r="K80" s="57">
         <v>5.87</v>
       </c>
-      <c r="L80" s="49"/>
-      <c r="M80" s="50">
+      <c r="L80" s="69"/>
+      <c r="M80" s="60">
         <f t="shared" si="12"/>
         <v>8335.4</v>
       </c>
-      <c r="N80" s="51"/>
-      <c r="O80" s="50"/>
-      <c r="P80" s="51">
+      <c r="N80" s="59"/>
+      <c r="O80" s="60"/>
+      <c r="P80" s="59">
         <f>SUM(P2:P79)</f>
-        <v>1937904.4765217388</v>
-      </c>
-      <c r="Q80" s="47"/>
+        <v>2050623.3171014492</v>
+      </c>
+      <c r="Q80" s="43"/>
     </row>
     <row r="81" spans="1:16" ht="33.75" customHeight="1">
       <c r="A81" s="15"/>
@@ -8681,9 +8561,9 @@
       <c r="J81" s="10"/>
       <c r="K81" s="12"/>
       <c r="L81" s="9"/>
-      <c r="P81" s="52">
+      <c r="P81" s="48">
         <f>P80-1180000</f>
-        <v>757904.4765217388</v>
+        <v>870623.31710144924</v>
       </c>
     </row>
     <row r="82" spans="1:16">

</xml_diff>